<commit_message>
Rafraîchissement des données (run de vérification des scrapers)
https://claude.ai/code/session_018Du4woKWpz1MpbftXwWJ97
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$406</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$413</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K406"/>
+  <dimension ref="A1:K413"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19557,8 +19557,337 @@
         <v>36298572</v>
       </c>
     </row>
+    <row r="407">
+      <c r="A407" s="2" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>07:45</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F407" t="n">
+        <v>11</v>
+      </c>
+      <c r="G407" t="n">
+        <v>28</v>
+      </c>
+      <c r="H407" t="inlineStr">
+        <is>
+          <t>11/28</t>
+        </is>
+      </c>
+      <c r="I407" s="4" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="J407" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K407" t="n">
+        <v>37089999</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" s="2" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F408" t="n">
+        <v>4</v>
+      </c>
+      <c r="G408" t="n">
+        <v>32</v>
+      </c>
+      <c r="H408" t="inlineStr">
+        <is>
+          <t>4/32</t>
+        </is>
+      </c>
+      <c r="I408" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="J408" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K408" t="n">
+        <v>37230107</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" s="2" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F409" t="n">
+        <v>14</v>
+      </c>
+      <c r="G409" t="n">
+        <v>28</v>
+      </c>
+      <c r="H409" t="inlineStr">
+        <is>
+          <t>14/28</t>
+        </is>
+      </c>
+      <c r="I409" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J409" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K409" t="n">
+        <v>36321554</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="2" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F410" t="n">
+        <v>4</v>
+      </c>
+      <c r="G410" t="n">
+        <v>18</v>
+      </c>
+      <c r="H410" t="inlineStr">
+        <is>
+          <t>4/18</t>
+        </is>
+      </c>
+      <c r="I410" s="4" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="J410" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K410" t="n">
+        <v>36929376</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" s="2" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F411" t="n">
+        <v>5</v>
+      </c>
+      <c r="G411" t="n">
+        <v>18</v>
+      </c>
+      <c r="H411" t="inlineStr">
+        <is>
+          <t>5/18</t>
+        </is>
+      </c>
+      <c r="I411" s="4" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="J411" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K411" t="n">
+        <v>36298749</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" s="2" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F412" t="n">
+        <v>25</v>
+      </c>
+      <c r="G412" t="n">
+        <v>28</v>
+      </c>
+      <c r="H412" t="inlineStr">
+        <is>
+          <t>25/28</t>
+        </is>
+      </c>
+      <c r="I412" s="3" t="n">
+        <v>89.3</v>
+      </c>
+      <c r="J412" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K412" t="n">
+        <v>36298803</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" s="2" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F413" t="n">
+        <v>33</v>
+      </c>
+      <c r="G413" t="n">
+        <v>33</v>
+      </c>
+      <c r="H413" t="inlineStr">
+        <is>
+          <t>33/33</t>
+        </is>
+      </c>
+      <c r="I413" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J413" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K413" t="n">
+        <v>36298856</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K406"/>
+  <autoFilter ref="A1:K413"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-05-30)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$413</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$420</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K413"/>
+  <dimension ref="A1:K420"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19886,8 +19886,337 @@
         <v>36298856</v>
       </c>
     </row>
+    <row r="414">
+      <c r="A414" s="2" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F414" t="n">
+        <v>13</v>
+      </c>
+      <c r="G414" t="n">
+        <v>28</v>
+      </c>
+      <c r="H414" t="inlineStr">
+        <is>
+          <t>13/28</t>
+        </is>
+      </c>
+      <c r="I414" s="4" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="J414" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K414" t="n">
+        <v>36319492</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" s="2" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F415" t="n">
+        <v>9</v>
+      </c>
+      <c r="G415" t="n">
+        <v>16</v>
+      </c>
+      <c r="H415" t="inlineStr">
+        <is>
+          <t>9/16</t>
+        </is>
+      </c>
+      <c r="I415" s="5" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="J415" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K415" t="n">
+        <v>36320650</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" s="2" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F416" t="n">
+        <v>2</v>
+      </c>
+      <c r="G416" t="n">
+        <v>16</v>
+      </c>
+      <c r="H416" t="inlineStr">
+        <is>
+          <t>2/16</t>
+        </is>
+      </c>
+      <c r="I416" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="J416" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K416" t="n">
+        <v>36320049</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" s="2" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F417" t="n">
+        <v>8</v>
+      </c>
+      <c r="G417" t="n">
+        <v>28</v>
+      </c>
+      <c r="H417" t="inlineStr">
+        <is>
+          <t>8/28</t>
+        </is>
+      </c>
+      <c r="I417" s="4" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="J417" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K417" t="n">
+        <v>36320773</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" s="2" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F418" t="n">
+        <v>21</v>
+      </c>
+      <c r="G418" t="n">
+        <v>28</v>
+      </c>
+      <c r="H418" t="inlineStr">
+        <is>
+          <t>21/28</t>
+        </is>
+      </c>
+      <c r="I418" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="J418" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K418" t="n">
+        <v>36320883</v>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" s="2" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F419" t="n">
+        <v>20</v>
+      </c>
+      <c r="G419" t="n">
+        <v>20</v>
+      </c>
+      <c r="H419" t="inlineStr">
+        <is>
+          <t>20/20</t>
+        </is>
+      </c>
+      <c r="I419" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J419" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K419" t="n">
+        <v>36893820</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" s="2" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F420" t="n">
+        <v>5</v>
+      </c>
+      <c r="G420" t="n">
+        <v>20</v>
+      </c>
+      <c r="H420" t="inlineStr">
+        <is>
+          <t>5/20</t>
+        </is>
+      </c>
+      <c r="I420" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="J420" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K420" t="n">
+        <v>36893866</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K413"/>
+  <autoFilter ref="A1:K420"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-05-31)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$420</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$425</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K420"/>
+  <dimension ref="A1:K425"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20215,8 +20215,243 @@
         <v>36893866</v>
       </c>
     </row>
+    <row r="421">
+      <c r="A421" s="2" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F421" t="n">
+        <v>4</v>
+      </c>
+      <c r="G421" t="n">
+        <v>32</v>
+      </c>
+      <c r="H421" t="inlineStr">
+        <is>
+          <t>4/32</t>
+        </is>
+      </c>
+      <c r="I421" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="J421" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K421" t="n">
+        <v>36323267</v>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" s="2" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>RE-BOOST  (English version)</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>alice dunoyer</t>
+        </is>
+      </c>
+      <c r="F422" t="n">
+        <v>16</v>
+      </c>
+      <c r="G422" t="n">
+        <v>28</v>
+      </c>
+      <c r="H422" t="inlineStr">
+        <is>
+          <t>16/28</t>
+        </is>
+      </c>
+      <c r="I422" s="5" t="n">
+        <v>57.1</v>
+      </c>
+      <c r="J422" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K422" t="n">
+        <v>36323113</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" s="2" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F423" t="n">
+        <v>9</v>
+      </c>
+      <c r="G423" t="n">
+        <v>28</v>
+      </c>
+      <c r="H423" t="inlineStr">
+        <is>
+          <t>9/28</t>
+        </is>
+      </c>
+      <c r="I423" s="4" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="J423" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K423" t="n">
+        <v>36329195</v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" s="2" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F424" t="n">
+        <v>8</v>
+      </c>
+      <c r="G424" t="n">
+        <v>28</v>
+      </c>
+      <c r="H424" t="inlineStr">
+        <is>
+          <t>8/28</t>
+        </is>
+      </c>
+      <c r="I424" s="4" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="J424" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K424" t="n">
+        <v>36329736</v>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" s="2" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F425" t="n">
+        <v>10</v>
+      </c>
+      <c r="G425" t="n">
+        <v>28</v>
+      </c>
+      <c r="H425" t="inlineStr">
+        <is>
+          <t>10/28</t>
+        </is>
+      </c>
+      <c r="I425" s="4" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="J425" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K425" t="n">
+        <v>36329960</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K420"/>
+  <autoFilter ref="A1:K425"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-06-01)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$425</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$432</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K425"/>
+  <dimension ref="A1:K432"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20450,8 +20450,337 @@
         <v>36329960</v>
       </c>
     </row>
+    <row r="426">
+      <c r="A426" s="2" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F426" t="n">
+        <v>8</v>
+      </c>
+      <c r="G426" t="n">
+        <v>36</v>
+      </c>
+      <c r="H426" t="inlineStr">
+        <is>
+          <t>8/36</t>
+        </is>
+      </c>
+      <c r="I426" s="4" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="J426" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K426" t="n">
+        <v>37240277</v>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" s="2" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F427" t="n">
+        <v>7</v>
+      </c>
+      <c r="G427" t="n">
+        <v>33</v>
+      </c>
+      <c r="H427" t="inlineStr">
+        <is>
+          <t>7/33</t>
+        </is>
+      </c>
+      <c r="I427" s="4" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="J427" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K427" t="n">
+        <v>36336023</v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" s="2" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F428" t="n">
+        <v>10</v>
+      </c>
+      <c r="G428" t="n">
+        <v>32</v>
+      </c>
+      <c r="H428" t="inlineStr">
+        <is>
+          <t>10/32</t>
+        </is>
+      </c>
+      <c r="I428" s="4" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="J428" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K428" t="n">
+        <v>37240420</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" s="2" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F429" t="n">
+        <v>8</v>
+      </c>
+      <c r="G429" t="n">
+        <v>32</v>
+      </c>
+      <c r="H429" t="inlineStr">
+        <is>
+          <t>8/32</t>
+        </is>
+      </c>
+      <c r="I429" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="J429" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K429" t="n">
+        <v>36892137</v>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" s="2" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F430" t="n">
+        <v>22</v>
+      </c>
+      <c r="G430" t="n">
+        <v>28</v>
+      </c>
+      <c r="H430" t="inlineStr">
+        <is>
+          <t>22/28</t>
+        </is>
+      </c>
+      <c r="I430" s="5" t="n">
+        <v>78.59999999999999</v>
+      </c>
+      <c r="J430" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K430" t="n">
+        <v>36336238</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" s="2" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F431" t="n">
+        <v>31</v>
+      </c>
+      <c r="G431" t="n">
+        <v>28</v>
+      </c>
+      <c r="H431" t="inlineStr">
+        <is>
+          <t>31/28</t>
+        </is>
+      </c>
+      <c r="I431" s="3" t="n">
+        <v>110.7</v>
+      </c>
+      <c r="J431" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K431" t="n">
+        <v>36692750</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" s="2" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F432" t="n">
+        <v>16</v>
+      </c>
+      <c r="G432" t="n">
+        <v>32</v>
+      </c>
+      <c r="H432" t="inlineStr">
+        <is>
+          <t>16/32</t>
+        </is>
+      </c>
+      <c r="I432" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J432" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K432" t="n">
+        <v>36892092</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K425"/>
+  <autoFilter ref="A1:K432"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-06-02)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$432</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$438</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K432"/>
+  <dimension ref="A1:K438"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20779,8 +20779,290 @@
         <v>36892092</v>
       </c>
     </row>
+    <row r="433">
+      <c r="A433" s="2" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F433" t="n">
+        <v>13</v>
+      </c>
+      <c r="G433" t="n">
+        <v>28</v>
+      </c>
+      <c r="H433" t="inlineStr">
+        <is>
+          <t>13/28</t>
+        </is>
+      </c>
+      <c r="I433" s="4" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="J433" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K433" t="n">
+        <v>36390324</v>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" s="2" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F434" t="n">
+        <v>3</v>
+      </c>
+      <c r="G434" t="n">
+        <v>18</v>
+      </c>
+      <c r="H434" t="inlineStr">
+        <is>
+          <t>3/18</t>
+        </is>
+      </c>
+      <c r="I434" s="4" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="J434" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K434" t="n">
+        <v>36928722</v>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" s="2" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F435" t="n">
+        <v>1</v>
+      </c>
+      <c r="G435" t="n">
+        <v>18</v>
+      </c>
+      <c r="H435" t="inlineStr">
+        <is>
+          <t>1/18</t>
+        </is>
+      </c>
+      <c r="I435" s="4" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="J435" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K435" t="n">
+        <v>36281127</v>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" s="2" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F436" t="n">
+        <v>9</v>
+      </c>
+      <c r="G436" t="n">
+        <v>28</v>
+      </c>
+      <c r="H436" t="inlineStr">
+        <is>
+          <t>9/28</t>
+        </is>
+      </c>
+      <c r="I436" s="4" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="J436" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K436" t="n">
+        <v>36280991</v>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" s="2" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F437" t="n">
+        <v>29</v>
+      </c>
+      <c r="G437" t="n">
+        <v>33</v>
+      </c>
+      <c r="H437" t="inlineStr">
+        <is>
+          <t>29/33</t>
+        </is>
+      </c>
+      <c r="I437" s="3" t="n">
+        <v>87.90000000000001</v>
+      </c>
+      <c r="J437" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K437" t="n">
+        <v>37873133</v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" s="2" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F438" t="n">
+        <v>17</v>
+      </c>
+      <c r="G438" t="n">
+        <v>28</v>
+      </c>
+      <c r="H438" t="inlineStr">
+        <is>
+          <t>17/28</t>
+        </is>
+      </c>
+      <c r="I438" s="5" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="J438" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K438" t="n">
+        <v>36929028</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K432"/>
+  <autoFilter ref="A1:K438"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
reset_seances.xlsx : refresh (régénéré par reset_scrape)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$438</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$443</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K438"/>
+  <dimension ref="A1:K443"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21061,8 +21061,243 @@
         <v>36929028</v>
       </c>
     </row>
+    <row r="439">
+      <c r="A439" s="2" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F439" t="n">
+        <v>5</v>
+      </c>
+      <c r="G439" t="n">
+        <v>28</v>
+      </c>
+      <c r="H439" t="inlineStr">
+        <is>
+          <t>5/28</t>
+        </is>
+      </c>
+      <c r="I439" s="4" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="J439" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K439" t="n">
+        <v>36321355</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" s="2" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F440" t="n">
+        <v>3</v>
+      </c>
+      <c r="G440" t="n">
+        <v>18</v>
+      </c>
+      <c r="H440" t="inlineStr">
+        <is>
+          <t>3/18</t>
+        </is>
+      </c>
+      <c r="I440" s="4" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="J440" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K440" t="n">
+        <v>36929154</v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" s="2" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F441" t="n">
+        <v>8</v>
+      </c>
+      <c r="G441" t="n">
+        <v>18</v>
+      </c>
+      <c r="H441" t="inlineStr">
+        <is>
+          <t>8/18</t>
+        </is>
+      </c>
+      <c r="I441" s="4" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="J441" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K441" t="n">
+        <v>36298234</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" s="2" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>Faustine CHOPIN</t>
+        </is>
+      </c>
+      <c r="F442" t="n">
+        <v>15</v>
+      </c>
+      <c r="G442" t="n">
+        <v>33</v>
+      </c>
+      <c r="H442" t="inlineStr">
+        <is>
+          <t>15/33</t>
+        </is>
+      </c>
+      <c r="I442" s="4" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="J442" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K442" t="n">
+        <v>36297679</v>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" s="2" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>RE-LAX  (English version)</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F443" t="n">
+        <v>29</v>
+      </c>
+      <c r="G443" t="n">
+        <v>33</v>
+      </c>
+      <c r="H443" t="inlineStr">
+        <is>
+          <t>29/33</t>
+        </is>
+      </c>
+      <c r="I443" s="3" t="n">
+        <v>87.90000000000001</v>
+      </c>
+      <c r="J443" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K443" t="n">
+        <v>36298041</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K438"/>
+  <autoFilter ref="A1:K443"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-06-05)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$443</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$457</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K443"/>
+  <dimension ref="A1:K457"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21296,8 +21296,666 @@
         <v>36298041</v>
       </c>
     </row>
+    <row r="444">
+      <c r="A444" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>alice dunoyer</t>
+        </is>
+      </c>
+      <c r="F444" t="n">
+        <v>15</v>
+      </c>
+      <c r="G444" t="n">
+        <v>33</v>
+      </c>
+      <c r="H444" t="inlineStr">
+        <is>
+          <t>15/33</t>
+        </is>
+      </c>
+      <c r="I444" s="4" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="J444" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K444" t="n">
+        <v>36321404</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F445" t="n">
+        <v>4</v>
+      </c>
+      <c r="G445" t="n">
+        <v>18</v>
+      </c>
+      <c r="H445" t="inlineStr">
+        <is>
+          <t>4/18</t>
+        </is>
+      </c>
+      <c r="I445" s="4" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="J445" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K445" t="n">
+        <v>36929286</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F446" t="n">
+        <v>6</v>
+      </c>
+      <c r="G446" t="n">
+        <v>18</v>
+      </c>
+      <c r="H446" t="inlineStr">
+        <is>
+          <t>6/18</t>
+        </is>
+      </c>
+      <c r="I446" s="4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J446" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K446" t="n">
+        <v>36298335</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>Pauline RAMON @pilatesbypops</t>
+        </is>
+      </c>
+      <c r="F447" t="n">
+        <v>32</v>
+      </c>
+      <c r="G447" t="n">
+        <v>33</v>
+      </c>
+      <c r="H447" t="inlineStr">
+        <is>
+          <t>32/33</t>
+        </is>
+      </c>
+      <c r="I447" s="3" t="n">
+        <v>97</v>
+      </c>
+      <c r="J447" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K447" t="n">
+        <v>36298376</v>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F448" t="n">
+        <v>23</v>
+      </c>
+      <c r="G448" t="n">
+        <v>33</v>
+      </c>
+      <c r="H448" t="inlineStr">
+        <is>
+          <t>23/33</t>
+        </is>
+      </c>
+      <c r="I448" s="5" t="n">
+        <v>69.7</v>
+      </c>
+      <c r="J448" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K448" t="n">
+        <v>36298573</v>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" s="2" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>07:45</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F449" t="n">
+        <v>5</v>
+      </c>
+      <c r="G449" t="n">
+        <v>28</v>
+      </c>
+      <c r="H449" t="inlineStr">
+        <is>
+          <t>5/28</t>
+        </is>
+      </c>
+      <c r="I449" s="4" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="J449" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K449" t="n">
+        <v>37090000</v>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" s="2" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F450" t="n">
+        <v>2</v>
+      </c>
+      <c r="G450" t="n">
+        <v>13</v>
+      </c>
+      <c r="H450" t="inlineStr">
+        <is>
+          <t>2/13</t>
+        </is>
+      </c>
+      <c r="I450" s="4" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="J450" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K450" t="n">
+        <v>37230108</v>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" s="2" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F451" t="n">
+        <v>0</v>
+      </c>
+      <c r="G451" t="n">
+        <v>13</v>
+      </c>
+      <c r="H451" t="inlineStr">
+        <is>
+          <t>0/13</t>
+        </is>
+      </c>
+      <c r="I451" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J451" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K451" t="n">
+        <v>37230144</v>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" s="2" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F452" t="n">
+        <v>5</v>
+      </c>
+      <c r="G452" t="n">
+        <v>13</v>
+      </c>
+      <c r="H452" t="inlineStr">
+        <is>
+          <t>5/13</t>
+        </is>
+      </c>
+      <c r="I452" s="4" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="J452" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K452" t="n">
+        <v>37090958</v>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" s="2" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F453" t="n">
+        <v>15</v>
+      </c>
+      <c r="G453" t="n">
+        <v>33</v>
+      </c>
+      <c r="H453" t="inlineStr">
+        <is>
+          <t>15/33</t>
+        </is>
+      </c>
+      <c r="I453" s="4" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="J453" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K453" t="n">
+        <v>36321555</v>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" s="2" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F454" t="n">
+        <v>6</v>
+      </c>
+      <c r="G454" t="n">
+        <v>18</v>
+      </c>
+      <c r="H454" t="inlineStr">
+        <is>
+          <t>6/18</t>
+        </is>
+      </c>
+      <c r="I454" s="4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J454" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K454" t="n">
+        <v>36929377</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" s="2" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F455" t="n">
+        <v>10</v>
+      </c>
+      <c r="G455" t="n">
+        <v>18</v>
+      </c>
+      <c r="H455" t="inlineStr">
+        <is>
+          <t>10/18</t>
+        </is>
+      </c>
+      <c r="I455" s="5" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="J455" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K455" t="n">
+        <v>36298750</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" s="2" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>Faustine CHOPIN</t>
+        </is>
+      </c>
+      <c r="F456" t="n">
+        <v>24</v>
+      </c>
+      <c r="G456" t="n">
+        <v>33</v>
+      </c>
+      <c r="H456" t="inlineStr">
+        <is>
+          <t>24/33</t>
+        </is>
+      </c>
+      <c r="I456" s="5" t="n">
+        <v>72.7</v>
+      </c>
+      <c r="J456" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K456" t="n">
+        <v>36298804</v>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" s="2" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F457" t="n">
+        <v>14</v>
+      </c>
+      <c r="G457" t="n">
+        <v>33</v>
+      </c>
+      <c r="H457" t="inlineStr">
+        <is>
+          <t>14/33</t>
+        </is>
+      </c>
+      <c r="I457" s="4" t="n">
+        <v>42.4</v>
+      </c>
+      <c r="J457" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K457" t="n">
+        <v>36298857</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K443"/>
+  <autoFilter ref="A1:K457"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ajout panneau META sur chaque dashboard (Méthode / Risque / État scrap)
- template_common.py : helper meta_panel_html(method, risk, freq, last_iso,
  n_rows) + bloc HTML 3 colonnes avec JS qui calcule la freshness
  ("Dernier scrap il y a X min/h/j") avec code couleur
- dashboard_meta.py : dict META par marque (banote/dna/le33foch/burningbar/
  senseclub/barrys/santroch/episod/anybuddy/snakeandtwist/reset +
  bsport_generic fallback)
- 12 scrapers patchés : injectent __META_PANEL__ après <div class="wrap">
  + computent le panneau dans write_html
- bsport_scrape + studio_scrape : utilisent cfg["key"] pour récupérer la
  meta de la marque courante

Affichage : juste sous le header, 3 colonnes
  ⚙️ Méthode : "API bsport directe", "Widget Mindbody", "Robot disparition"...
  ⚠️ Limites/risques : précision, throttle, capacité estimée...
  📡 État du scrap : "Dernier scrap il y a 4 min" + nb entrées + fréquence
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -14694,18 +14694,18 @@
         </is>
       </c>
       <c r="F303" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G303" t="n">
         <v>28</v>
       </c>
       <c r="H303" t="inlineStr">
         <is>
-          <t>29/28</t>
+          <t>28/28</t>
         </is>
       </c>
       <c r="I303" s="3" t="n">
-        <v>103.6</v>
+        <v>100</v>
       </c>
       <c r="J303" t="inlineStr">
         <is>
@@ -15775,18 +15775,18 @@
         </is>
       </c>
       <c r="F326" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G326" t="n">
         <v>28</v>
       </c>
       <c r="H326" t="inlineStr">
         <is>
-          <t>27/28</t>
+          <t>26/28</t>
         </is>
       </c>
       <c r="I326" s="3" t="n">
-        <v>96.40000000000001</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="J326" t="inlineStr">
         <is>
@@ -17232,22 +17232,22 @@
         </is>
       </c>
       <c r="F357" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G357" t="n">
         <v>28</v>
       </c>
       <c r="H357" t="inlineStr">
         <is>
-          <t>28/28</t>
+          <t>27/28</t>
         </is>
       </c>
       <c r="I357" s="3" t="n">
-        <v>100</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="J357" t="inlineStr">
         <is>
-          <t>oui</t>
+          <t>non</t>
         </is>
       </c>
       <c r="K357" t="n">

</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-06-06)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$457</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$464</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K457"/>
+  <dimension ref="A1:K464"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21954,8 +21954,337 @@
         <v>36298857</v>
       </c>
     </row>
+    <row r="458">
+      <c r="A458" s="2" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F458" t="n">
+        <v>10</v>
+      </c>
+      <c r="G458" t="n">
+        <v>32</v>
+      </c>
+      <c r="H458" t="inlineStr">
+        <is>
+          <t>10/32</t>
+        </is>
+      </c>
+      <c r="I458" s="4" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="J458" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K458" t="n">
+        <v>36319493</v>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" s="2" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F459" t="n">
+        <v>2</v>
+      </c>
+      <c r="G459" t="n">
+        <v>16</v>
+      </c>
+      <c r="H459" t="inlineStr">
+        <is>
+          <t>2/16</t>
+        </is>
+      </c>
+      <c r="I459" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="J459" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K459" t="n">
+        <v>36320651</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" s="2" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F460" t="n">
+        <v>7</v>
+      </c>
+      <c r="G460" t="n">
+        <v>16</v>
+      </c>
+      <c r="H460" t="inlineStr">
+        <is>
+          <t>7/16</t>
+        </is>
+      </c>
+      <c r="I460" s="4" t="n">
+        <v>43.8</v>
+      </c>
+      <c r="J460" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K460" t="n">
+        <v>36320050</v>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" s="2" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F461" t="n">
+        <v>10</v>
+      </c>
+      <c r="G461" t="n">
+        <v>33</v>
+      </c>
+      <c r="H461" t="inlineStr">
+        <is>
+          <t>10/33</t>
+        </is>
+      </c>
+      <c r="I461" s="4" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="J461" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K461" t="n">
+        <v>36320774</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" s="2" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F462" t="n">
+        <v>22</v>
+      </c>
+      <c r="G462" t="n">
+        <v>33</v>
+      </c>
+      <c r="H462" t="inlineStr">
+        <is>
+          <t>22/33</t>
+        </is>
+      </c>
+      <c r="I462" s="5" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J462" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K462" t="n">
+        <v>36320884</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" s="2" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F463" t="n">
+        <v>3</v>
+      </c>
+      <c r="G463" t="n">
+        <v>20</v>
+      </c>
+      <c r="H463" t="inlineStr">
+        <is>
+          <t>3/20</t>
+        </is>
+      </c>
+      <c r="I463" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="J463" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K463" t="n">
+        <v>36893821</v>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" s="2" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F464" t="n">
+        <v>14</v>
+      </c>
+      <c r="G464" t="n">
+        <v>20</v>
+      </c>
+      <c r="H464" t="inlineStr">
+        <is>
+          <t>14/20</t>
+        </is>
+      </c>
+      <c r="I464" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="J464" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K464" t="n">
+        <v>36893869</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K457"/>
+  <autoFilter ref="A1:K464"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-06-07)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$464</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$472</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K464"/>
+  <dimension ref="A1:K472"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -22283,8 +22283,384 @@
         <v>36893869</v>
       </c>
     </row>
+    <row r="465">
+      <c r="A465" s="2" t="n">
+        <v>46179</v>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F465" t="n">
+        <v>3</v>
+      </c>
+      <c r="G465" t="n">
+        <v>32</v>
+      </c>
+      <c r="H465" t="inlineStr">
+        <is>
+          <t>3/32</t>
+        </is>
+      </c>
+      <c r="I465" s="4" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="J465" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K465" t="n">
+        <v>36323268</v>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" s="2" t="n">
+        <v>46179</v>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F466" t="n">
+        <v>13</v>
+      </c>
+      <c r="G466" t="n">
+        <v>28</v>
+      </c>
+      <c r="H466" t="inlineStr">
+        <is>
+          <t>13/28</t>
+        </is>
+      </c>
+      <c r="I466" s="4" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="J466" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K466" t="n">
+        <v>36323114</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" s="2" t="n">
+        <v>46179</v>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F467" t="n">
+        <v>9</v>
+      </c>
+      <c r="G467" t="n">
+        <v>28</v>
+      </c>
+      <c r="H467" t="inlineStr">
+        <is>
+          <t>9/28</t>
+        </is>
+      </c>
+      <c r="I467" s="4" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="J467" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K467" t="n">
+        <v>38385551</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" s="2" t="n">
+        <v>46179</v>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F468" t="n">
+        <v>19</v>
+      </c>
+      <c r="G468" t="n">
+        <v>33</v>
+      </c>
+      <c r="H468" t="inlineStr">
+        <is>
+          <t>19/33</t>
+        </is>
+      </c>
+      <c r="I468" s="5" t="n">
+        <v>57.6</v>
+      </c>
+      <c r="J468" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K468" t="n">
+        <v>36329196</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" s="2" t="n">
+        <v>46179</v>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F469" t="n">
+        <v>21</v>
+      </c>
+      <c r="G469" t="n">
+        <v>36</v>
+      </c>
+      <c r="H469" t="inlineStr">
+        <is>
+          <t>21/36</t>
+        </is>
+      </c>
+      <c r="I469" s="5" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="J469" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K469" t="n">
+        <v>36329737</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" s="2" t="n">
+        <v>46179</v>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F470" t="n">
+        <v>28</v>
+      </c>
+      <c r="G470" t="n">
+        <v>33</v>
+      </c>
+      <c r="H470" t="inlineStr">
+        <is>
+          <t>28/33</t>
+        </is>
+      </c>
+      <c r="I470" s="5" t="n">
+        <v>84.8</v>
+      </c>
+      <c r="J470" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K470" t="n">
+        <v>36329961</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" s="2" t="n">
+        <v>46179</v>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F471" t="n">
+        <v>4</v>
+      </c>
+      <c r="G471" t="n">
+        <v>20</v>
+      </c>
+      <c r="H471" t="inlineStr">
+        <is>
+          <t>4/20</t>
+        </is>
+      </c>
+      <c r="I471" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J471" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K471" t="n">
+        <v>36935868</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" s="2" t="n">
+        <v>46179</v>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F472" t="n">
+        <v>10</v>
+      </c>
+      <c r="G472" t="n">
+        <v>20</v>
+      </c>
+      <c r="H472" t="inlineStr">
+        <is>
+          <t>10/20</t>
+        </is>
+      </c>
+      <c r="I472" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J472" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K472" t="n">
+        <v>36323853</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K464"/>
+  <autoFilter ref="A1:K472"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-06-08)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$472</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$479</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K472"/>
+  <dimension ref="A1:K479"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -22659,8 +22659,337 @@
         <v>36323853</v>
       </c>
     </row>
+    <row r="473">
+      <c r="A473" s="2" t="n">
+        <v>46180</v>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F473" t="n">
+        <v>7</v>
+      </c>
+      <c r="G473" t="n">
+        <v>36</v>
+      </c>
+      <c r="H473" t="inlineStr">
+        <is>
+          <t>7/36</t>
+        </is>
+      </c>
+      <c r="I473" s="4" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="J473" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K473" t="n">
+        <v>37240278</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" s="2" t="n">
+        <v>46180</v>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F474" t="n">
+        <v>25</v>
+      </c>
+      <c r="G474" t="n">
+        <v>33</v>
+      </c>
+      <c r="H474" t="inlineStr">
+        <is>
+          <t>25/33</t>
+        </is>
+      </c>
+      <c r="I474" s="5" t="n">
+        <v>75.8</v>
+      </c>
+      <c r="J474" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K474" t="n">
+        <v>36336024</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" s="2" t="n">
+        <v>46180</v>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F475" t="n">
+        <v>14</v>
+      </c>
+      <c r="G475" t="n">
+        <v>32</v>
+      </c>
+      <c r="H475" t="inlineStr">
+        <is>
+          <t>14/32</t>
+        </is>
+      </c>
+      <c r="I475" s="4" t="n">
+        <v>43.8</v>
+      </c>
+      <c r="J475" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K475" t="n">
+        <v>37240421</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" s="2" t="n">
+        <v>46180</v>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F476" t="n">
+        <v>24</v>
+      </c>
+      <c r="G476" t="n">
+        <v>32</v>
+      </c>
+      <c r="H476" t="inlineStr">
+        <is>
+          <t>24/32</t>
+        </is>
+      </c>
+      <c r="I476" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="J476" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K476" t="n">
+        <v>36892138</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" s="2" t="n">
+        <v>46180</v>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F477" t="n">
+        <v>27</v>
+      </c>
+      <c r="G477" t="n">
+        <v>33</v>
+      </c>
+      <c r="H477" t="inlineStr">
+        <is>
+          <t>27/33</t>
+        </is>
+      </c>
+      <c r="I477" s="5" t="n">
+        <v>81.8</v>
+      </c>
+      <c r="J477" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K477" t="n">
+        <v>36336239</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" s="2" t="n">
+        <v>46180</v>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F478" t="n">
+        <v>28</v>
+      </c>
+      <c r="G478" t="n">
+        <v>33</v>
+      </c>
+      <c r="H478" t="inlineStr">
+        <is>
+          <t>28/33</t>
+        </is>
+      </c>
+      <c r="I478" s="5" t="n">
+        <v>84.8</v>
+      </c>
+      <c r="J478" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K478" t="n">
+        <v>36692751</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" s="2" t="n">
+        <v>46180</v>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F479" t="n">
+        <v>21</v>
+      </c>
+      <c r="G479" t="n">
+        <v>36</v>
+      </c>
+      <c r="H479" t="inlineStr">
+        <is>
+          <t>21/36</t>
+        </is>
+      </c>
+      <c r="I479" s="5" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="J479" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K479" t="n">
+        <v>36892093</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K472"/>
+  <autoFilter ref="A1:K479"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-06-09)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$479</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$485</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K479"/>
+  <dimension ref="A1:K485"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2000,7 +2000,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Pauline RAMON @pilatesbypops</t>
+          <t>Pauline Ramon</t>
         </is>
       </c>
       <c r="F33" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Pauline RAMON @pilatesbypops</t>
+          <t>Pauline Ramon</t>
         </is>
       </c>
       <c r="F72" t="n">
@@ -5807,7 +5807,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Pauline RAMON @pilatesbypops</t>
+          <t>Pauline Ramon</t>
         </is>
       </c>
       <c r="F114" t="n">
@@ -8016,7 +8016,7 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>Pauline RAMON @pilatesbypops</t>
+          <t>Pauline Ramon</t>
         </is>
       </c>
       <c r="F161" t="n">
@@ -10131,7 +10131,7 @@
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>Pauline RAMON @pilatesbypops</t>
+          <t>Pauline Ramon</t>
         </is>
       </c>
       <c r="F206" t="n">
@@ -11165,7 +11165,7 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>Pauline RAMON @pilatesbypops</t>
+          <t>Pauline Ramon</t>
         </is>
       </c>
       <c r="F228" t="n">
@@ -12481,7 +12481,7 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>Pauline RAMON @pilatesbypops</t>
+          <t>Pauline Ramon</t>
         </is>
       </c>
       <c r="F256" t="n">
@@ -14878,7 +14878,7 @@
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>Pauline RAMON @pilatesbypops</t>
+          <t>Pauline Ramon</t>
         </is>
       </c>
       <c r="F307" t="n">
@@ -15536,7 +15536,7 @@
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>Pauline RAMON @pilatesbypops</t>
+          <t>Pauline Ramon</t>
         </is>
       </c>
       <c r="F321" t="n">
@@ -15912,7 +15912,7 @@
       </c>
       <c r="E329" t="inlineStr">
         <is>
-          <t>Pauline RAMON @pilatesbypops</t>
+          <t>Pauline Ramon</t>
         </is>
       </c>
       <c r="F329" t="n">
@@ -17181,7 +17181,7 @@
       </c>
       <c r="E356" t="inlineStr">
         <is>
-          <t>Pauline RAMON @pilatesbypops</t>
+          <t>Pauline Ramon</t>
         </is>
       </c>
       <c r="F356" t="n">
@@ -19484,7 +19484,7 @@
       </c>
       <c r="E405" t="inlineStr">
         <is>
-          <t>Pauline RAMON @pilatesbypops</t>
+          <t>Pauline Ramon</t>
         </is>
       </c>
       <c r="F405" t="n">
@@ -21458,7 +21458,7 @@
       </c>
       <c r="E447" t="inlineStr">
         <is>
-          <t>Pauline RAMON @pilatesbypops</t>
+          <t>Pauline Ramon</t>
         </is>
       </c>
       <c r="F447" t="n">
@@ -22988,8 +22988,290 @@
         <v>36892093</v>
       </c>
     </row>
+    <row r="480">
+      <c r="A480" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F480" t="n">
+        <v>12</v>
+      </c>
+      <c r="G480" t="n">
+        <v>28</v>
+      </c>
+      <c r="H480" t="inlineStr">
+        <is>
+          <t>12/28</t>
+        </is>
+      </c>
+      <c r="I480" s="4" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="J480" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K480" t="n">
+        <v>36390325</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F481" t="n">
+        <v>6</v>
+      </c>
+      <c r="G481" t="n">
+        <v>28</v>
+      </c>
+      <c r="H481" t="inlineStr">
+        <is>
+          <t>6/28</t>
+        </is>
+      </c>
+      <c r="I481" s="4" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="J481" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K481" t="n">
+        <v>36281128</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F482" t="n">
+        <v>6</v>
+      </c>
+      <c r="G482" t="n">
+        <v>18</v>
+      </c>
+      <c r="H482" t="inlineStr">
+        <is>
+          <t>6/18</t>
+        </is>
+      </c>
+      <c r="I482" s="4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J482" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K482" t="n">
+        <v>36928723</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F483" t="n">
+        <v>6</v>
+      </c>
+      <c r="G483" t="n">
+        <v>18</v>
+      </c>
+      <c r="H483" t="inlineStr">
+        <is>
+          <t>6/18</t>
+        </is>
+      </c>
+      <c r="I483" s="4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J483" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K483" t="n">
+        <v>38647189</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F484" t="n">
+        <v>19</v>
+      </c>
+      <c r="G484" t="n">
+        <v>33</v>
+      </c>
+      <c r="H484" t="inlineStr">
+        <is>
+          <t>19/33</t>
+        </is>
+      </c>
+      <c r="I484" s="5" t="n">
+        <v>57.6</v>
+      </c>
+      <c r="J484" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K484" t="n">
+        <v>36280992</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F485" t="n">
+        <v>22</v>
+      </c>
+      <c r="G485" t="n">
+        <v>33</v>
+      </c>
+      <c r="H485" t="inlineStr">
+        <is>
+          <t>22/33</t>
+        </is>
+      </c>
+      <c r="I485" s="5" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J485" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K485" t="n">
+        <v>37873134</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K479"/>
+  <autoFilter ref="A1:K485"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-06-10)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$485</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$491</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K485"/>
+  <dimension ref="A1:K491"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13472,18 +13472,18 @@
         </is>
       </c>
       <c r="F277" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G277" t="n">
         <v>12</v>
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>5/12</t>
+          <t>4/12</t>
         </is>
       </c>
       <c r="I277" s="4" t="n">
-        <v>41.7</v>
+        <v>33.3</v>
       </c>
       <c r="J277" t="inlineStr">
         <is>
@@ -23270,8 +23270,290 @@
         <v>37873134</v>
       </c>
     </row>
+    <row r="486">
+      <c r="A486" s="2" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F486" t="n">
+        <v>12</v>
+      </c>
+      <c r="G486" t="n">
+        <v>28</v>
+      </c>
+      <c r="H486" t="inlineStr">
+        <is>
+          <t>12/28</t>
+        </is>
+      </c>
+      <c r="I486" s="4" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="J486" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K486" t="n">
+        <v>36321356</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" s="2" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F487" t="n">
+        <v>6</v>
+      </c>
+      <c r="G487" t="n">
+        <v>18</v>
+      </c>
+      <c r="H487" t="inlineStr">
+        <is>
+          <t>6/18</t>
+        </is>
+      </c>
+      <c r="I487" s="4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J487" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K487" t="n">
+        <v>36298235</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" s="2" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F488" t="n">
+        <v>9</v>
+      </c>
+      <c r="G488" t="n">
+        <v>18</v>
+      </c>
+      <c r="H488" t="inlineStr">
+        <is>
+          <t>9/18</t>
+        </is>
+      </c>
+      <c r="I488" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J488" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K488" t="n">
+        <v>36929155</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" s="2" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F489" t="n">
+        <v>10</v>
+      </c>
+      <c r="G489" t="n">
+        <v>28</v>
+      </c>
+      <c r="H489" t="inlineStr">
+        <is>
+          <t>10/28</t>
+        </is>
+      </c>
+      <c r="I489" s="4" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="J489" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K489" t="n">
+        <v>36297680</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" s="2" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>RE-LAX  (English version)</t>
+        </is>
+      </c>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F490" t="n">
+        <v>20</v>
+      </c>
+      <c r="G490" t="n">
+        <v>28</v>
+      </c>
+      <c r="H490" t="inlineStr">
+        <is>
+          <t>20/28</t>
+        </is>
+      </c>
+      <c r="I490" s="5" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="J490" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K490" t="n">
+        <v>36298042</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" s="2" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F491" t="n">
+        <v>21</v>
+      </c>
+      <c r="G491" t="n">
+        <v>36</v>
+      </c>
+      <c r="H491" t="inlineStr">
+        <is>
+          <t>21/36</t>
+        </is>
+      </c>
+      <c r="I491" s="5" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="J491" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K491" t="n">
+        <v>38531841</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K485"/>
+  <autoFilter ref="A1:K491"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-06-11)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$491</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$496</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K491"/>
+  <dimension ref="A1:K496"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -23107,18 +23107,18 @@
         </is>
       </c>
       <c r="F482" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G482" t="n">
         <v>18</v>
       </c>
       <c r="H482" t="inlineStr">
         <is>
-          <t>6/18</t>
+          <t>5/18</t>
         </is>
       </c>
       <c r="I482" s="4" t="n">
-        <v>33.3</v>
+        <v>27.8</v>
       </c>
       <c r="J482" t="inlineStr">
         <is>
@@ -23552,8 +23552,243 @@
         <v>38531841</v>
       </c>
     </row>
+    <row r="492">
+      <c r="A492" s="2" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E492" t="inlineStr">
+        <is>
+          <t>alice dunoyer</t>
+        </is>
+      </c>
+      <c r="F492" t="n">
+        <v>10</v>
+      </c>
+      <c r="G492" t="n">
+        <v>33</v>
+      </c>
+      <c r="H492" t="inlineStr">
+        <is>
+          <t>10/33</t>
+        </is>
+      </c>
+      <c r="I492" s="4" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="J492" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K492" t="n">
+        <v>36321405</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" s="2" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F493" t="n">
+        <v>11</v>
+      </c>
+      <c r="G493" t="n">
+        <v>18</v>
+      </c>
+      <c r="H493" t="inlineStr">
+        <is>
+          <t>11/18</t>
+        </is>
+      </c>
+      <c r="I493" s="5" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="J493" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K493" t="n">
+        <v>36929287</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" s="2" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E494" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F494" t="n">
+        <v>10</v>
+      </c>
+      <c r="G494" t="n">
+        <v>18</v>
+      </c>
+      <c r="H494" t="inlineStr">
+        <is>
+          <t>10/18</t>
+        </is>
+      </c>
+      <c r="I494" s="5" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="J494" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K494" t="n">
+        <v>36298336</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" s="2" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>Pauline Ramon</t>
+        </is>
+      </c>
+      <c r="F495" t="n">
+        <v>28</v>
+      </c>
+      <c r="G495" t="n">
+        <v>33</v>
+      </c>
+      <c r="H495" t="inlineStr">
+        <is>
+          <t>28/33</t>
+        </is>
+      </c>
+      <c r="I495" s="5" t="n">
+        <v>84.8</v>
+      </c>
+      <c r="J495" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K495" t="n">
+        <v>36298377</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" s="2" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F496" t="n">
+        <v>31</v>
+      </c>
+      <c r="G496" t="n">
+        <v>33</v>
+      </c>
+      <c r="H496" t="inlineStr">
+        <is>
+          <t>31/33</t>
+        </is>
+      </c>
+      <c r="I496" s="3" t="n">
+        <v>93.90000000000001</v>
+      </c>
+      <c r="J496" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K496" t="n">
+        <v>36298574</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K491"/>
+  <autoFilter ref="A1:K496"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-06-12)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$496</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$505</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K496"/>
+  <dimension ref="A1:K505"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -23787,8 +23787,431 @@
         <v>36298574</v>
       </c>
     </row>
+    <row r="497">
+      <c r="A497" s="2" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>07:45</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F497" t="n">
+        <v>7</v>
+      </c>
+      <c r="G497" t="n">
+        <v>28</v>
+      </c>
+      <c r="H497" t="inlineStr">
+        <is>
+          <t>7/28</t>
+        </is>
+      </c>
+      <c r="I497" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="J497" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K497" t="n">
+        <v>37090001</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" s="2" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F498" t="n">
+        <v>1</v>
+      </c>
+      <c r="G498" t="n">
+        <v>13</v>
+      </c>
+      <c r="H498" t="inlineStr">
+        <is>
+          <t>1/13</t>
+        </is>
+      </c>
+      <c r="I498" s="4" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="J498" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K498" t="n">
+        <v>37230109</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" s="2" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F499" t="n">
+        <v>0</v>
+      </c>
+      <c r="G499" t="n">
+        <v>13</v>
+      </c>
+      <c r="H499" t="inlineStr">
+        <is>
+          <t>0/13</t>
+        </is>
+      </c>
+      <c r="I499" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J499" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K499" t="n">
+        <v>37230145</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" s="2" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F500" t="n">
+        <v>7</v>
+      </c>
+      <c r="G500" t="n">
+        <v>13</v>
+      </c>
+      <c r="H500" t="inlineStr">
+        <is>
+          <t>7/13</t>
+        </is>
+      </c>
+      <c r="I500" s="5" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="J500" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K500" t="n">
+        <v>37090959</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" s="2" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F501" t="n">
+        <v>16</v>
+      </c>
+      <c r="G501" t="n">
+        <v>28</v>
+      </c>
+      <c r="H501" t="inlineStr">
+        <is>
+          <t>16/28</t>
+        </is>
+      </c>
+      <c r="I501" s="5" t="n">
+        <v>57.1</v>
+      </c>
+      <c r="J501" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K501" t="n">
+        <v>36321556</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" s="2" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E502" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F502" t="n">
+        <v>6</v>
+      </c>
+      <c r="G502" t="n">
+        <v>18</v>
+      </c>
+      <c r="H502" t="inlineStr">
+        <is>
+          <t>6/18</t>
+        </is>
+      </c>
+      <c r="I502" s="4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J502" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K502" t="n">
+        <v>36929378</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" s="2" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E503" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F503" t="n">
+        <v>8</v>
+      </c>
+      <c r="G503" t="n">
+        <v>18</v>
+      </c>
+      <c r="H503" t="inlineStr">
+        <is>
+          <t>8/18</t>
+        </is>
+      </c>
+      <c r="I503" s="4" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="J503" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K503" t="n">
+        <v>36298751</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" s="2" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E504" t="inlineStr">
+        <is>
+          <t>Faustine CHOPIN</t>
+        </is>
+      </c>
+      <c r="F504" t="n">
+        <v>20</v>
+      </c>
+      <c r="G504" t="n">
+        <v>33</v>
+      </c>
+      <c r="H504" t="inlineStr">
+        <is>
+          <t>20/33</t>
+        </is>
+      </c>
+      <c r="I504" s="5" t="n">
+        <v>60.6</v>
+      </c>
+      <c r="J504" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K504" t="n">
+        <v>36298805</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" s="2" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E505" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F505" t="n">
+        <v>14</v>
+      </c>
+      <c r="G505" t="n">
+        <v>33</v>
+      </c>
+      <c r="H505" t="inlineStr">
+        <is>
+          <t>14/33</t>
+        </is>
+      </c>
+      <c r="I505" s="4" t="n">
+        <v>42.4</v>
+      </c>
+      <c r="J505" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K505" t="n">
+        <v>36298858</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K496"/>
+  <autoFilter ref="A1:K505"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-06-13)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$505</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$512</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K505"/>
+  <dimension ref="A1:K512"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -24000,18 +24000,18 @@
         </is>
       </c>
       <c r="F501" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G501" t="n">
         <v>28</v>
       </c>
       <c r="H501" t="inlineStr">
         <is>
-          <t>16/28</t>
+          <t>17/28</t>
         </is>
       </c>
       <c r="I501" s="5" t="n">
-        <v>57.1</v>
+        <v>60.7</v>
       </c>
       <c r="J501" t="inlineStr">
         <is>
@@ -24210,8 +24210,337 @@
         <v>36298858</v>
       </c>
     </row>
+    <row r="506">
+      <c r="A506" s="2" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E506" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F506" t="n">
+        <v>7</v>
+      </c>
+      <c r="G506" t="n">
+        <v>28</v>
+      </c>
+      <c r="H506" t="inlineStr">
+        <is>
+          <t>7/28</t>
+        </is>
+      </c>
+      <c r="I506" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="J506" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K506" t="n">
+        <v>36319494</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" s="2" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E507" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F507" t="n">
+        <v>3</v>
+      </c>
+      <c r="G507" t="n">
+        <v>16</v>
+      </c>
+      <c r="H507" t="inlineStr">
+        <is>
+          <t>3/16</t>
+        </is>
+      </c>
+      <c r="I507" s="4" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="J507" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K507" t="n">
+        <v>36320652</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" s="2" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E508" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F508" t="n">
+        <v>3</v>
+      </c>
+      <c r="G508" t="n">
+        <v>16</v>
+      </c>
+      <c r="H508" t="inlineStr">
+        <is>
+          <t>3/16</t>
+        </is>
+      </c>
+      <c r="I508" s="4" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="J508" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K508" t="n">
+        <v>36320051</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" s="2" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E509" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F509" t="n">
+        <v>28</v>
+      </c>
+      <c r="G509" t="n">
+        <v>33</v>
+      </c>
+      <c r="H509" t="inlineStr">
+        <is>
+          <t>28/33</t>
+        </is>
+      </c>
+      <c r="I509" s="5" t="n">
+        <v>84.8</v>
+      </c>
+      <c r="J509" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K509" t="n">
+        <v>36320775</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" s="2" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E510" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F510" t="n">
+        <v>30</v>
+      </c>
+      <c r="G510" t="n">
+        <v>33</v>
+      </c>
+      <c r="H510" t="inlineStr">
+        <is>
+          <t>30/33</t>
+        </is>
+      </c>
+      <c r="I510" s="3" t="n">
+        <v>90.90000000000001</v>
+      </c>
+      <c r="J510" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K510" t="n">
+        <v>36320885</v>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" s="2" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E511" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F511" t="n">
+        <v>12</v>
+      </c>
+      <c r="G511" t="n">
+        <v>20</v>
+      </c>
+      <c r="H511" t="inlineStr">
+        <is>
+          <t>12/20</t>
+        </is>
+      </c>
+      <c r="I511" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="J511" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K511" t="n">
+        <v>36893822</v>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" s="2" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E512" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F512" t="n">
+        <v>4</v>
+      </c>
+      <c r="G512" t="n">
+        <v>20</v>
+      </c>
+      <c r="H512" t="inlineStr">
+        <is>
+          <t>4/20</t>
+        </is>
+      </c>
+      <c r="I512" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J512" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K512" t="n">
+        <v>36893872</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K505"/>
+  <autoFilter ref="A1:K512"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-06-14)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$512</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$519</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K512"/>
+  <dimension ref="A1:K519"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -24539,8 +24539,337 @@
         <v>36893872</v>
       </c>
     </row>
+    <row r="513">
+      <c r="A513" s="2" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E513" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F513" t="n">
+        <v>4</v>
+      </c>
+      <c r="G513" t="n">
+        <v>32</v>
+      </c>
+      <c r="H513" t="inlineStr">
+        <is>
+          <t>4/32</t>
+        </is>
+      </c>
+      <c r="I513" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="J513" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K513" t="n">
+        <v>36323269</v>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" s="2" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>RE-BOOST  (English version)</t>
+        </is>
+      </c>
+      <c r="E514" t="inlineStr">
+        <is>
+          <t>alice dunoyer</t>
+        </is>
+      </c>
+      <c r="F514" t="n">
+        <v>6</v>
+      </c>
+      <c r="G514" t="n">
+        <v>33</v>
+      </c>
+      <c r="H514" t="inlineStr">
+        <is>
+          <t>6/33</t>
+        </is>
+      </c>
+      <c r="I514" s="4" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="J514" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K514" t="n">
+        <v>36323115</v>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" s="2" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E515" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F515" t="n">
+        <v>2</v>
+      </c>
+      <c r="G515" t="n">
+        <v>13</v>
+      </c>
+      <c r="H515" t="inlineStr">
+        <is>
+          <t>2/13</t>
+        </is>
+      </c>
+      <c r="I515" s="4" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="J515" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K515" t="n">
+        <v>38021838</v>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" s="2" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>13:45</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E516" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F516" t="n">
+        <v>2</v>
+      </c>
+      <c r="G516" t="n">
+        <v>13</v>
+      </c>
+      <c r="H516" t="inlineStr">
+        <is>
+          <t>2/13</t>
+        </is>
+      </c>
+      <c r="I516" s="4" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="J516" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K516" t="n">
+        <v>38021897</v>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" s="2" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E517" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F517" t="n">
+        <v>11</v>
+      </c>
+      <c r="G517" t="n">
+        <v>13</v>
+      </c>
+      <c r="H517" t="inlineStr">
+        <is>
+          <t>11/13</t>
+        </is>
+      </c>
+      <c r="I517" s="5" t="n">
+        <v>84.59999999999999</v>
+      </c>
+      <c r="J517" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K517" t="n">
+        <v>38021900</v>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" s="2" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E518" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F518" t="n">
+        <v>10</v>
+      </c>
+      <c r="G518" t="n">
+        <v>28</v>
+      </c>
+      <c r="H518" t="inlineStr">
+        <is>
+          <t>10/28</t>
+        </is>
+      </c>
+      <c r="I518" s="4" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="J518" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K518" t="n">
+        <v>36329738</v>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" s="2" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E519" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F519" t="n">
+        <v>20</v>
+      </c>
+      <c r="G519" t="n">
+        <v>28</v>
+      </c>
+      <c r="H519" t="inlineStr">
+        <is>
+          <t>20/28</t>
+        </is>
+      </c>
+      <c r="I519" s="5" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="J519" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K519" t="n">
+        <v>36329962</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K512"/>
+  <autoFilter ref="A1:K519"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-06-15)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$519</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$526</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K519"/>
+  <dimension ref="A1:K526"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -24868,8 +24868,337 @@
         <v>36329962</v>
       </c>
     </row>
+    <row r="520">
+      <c r="A520" s="2" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E520" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F520" t="n">
+        <v>8</v>
+      </c>
+      <c r="G520" t="n">
+        <v>36</v>
+      </c>
+      <c r="H520" t="inlineStr">
+        <is>
+          <t>8/36</t>
+        </is>
+      </c>
+      <c r="I520" s="4" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="J520" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K520" t="n">
+        <v>37240279</v>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" s="2" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E521" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F521" t="n">
+        <v>11</v>
+      </c>
+      <c r="G521" t="n">
+        <v>33</v>
+      </c>
+      <c r="H521" t="inlineStr">
+        <is>
+          <t>11/33</t>
+        </is>
+      </c>
+      <c r="I521" s="4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J521" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K521" t="n">
+        <v>36336025</v>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" s="2" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E522" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F522" t="n">
+        <v>6</v>
+      </c>
+      <c r="G522" t="n">
+        <v>28</v>
+      </c>
+      <c r="H522" t="inlineStr">
+        <is>
+          <t>6/28</t>
+        </is>
+      </c>
+      <c r="I522" s="4" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="J522" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K522" t="n">
+        <v>37240422</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" s="2" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E523" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F523" t="n">
+        <v>12</v>
+      </c>
+      <c r="G523" t="n">
+        <v>28</v>
+      </c>
+      <c r="H523" t="inlineStr">
+        <is>
+          <t>12/28</t>
+        </is>
+      </c>
+      <c r="I523" s="4" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="J523" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K523" t="n">
+        <v>36892139</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" s="2" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="D524" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E524" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F524" t="n">
+        <v>17</v>
+      </c>
+      <c r="G524" t="n">
+        <v>33</v>
+      </c>
+      <c r="H524" t="inlineStr">
+        <is>
+          <t>17/33</t>
+        </is>
+      </c>
+      <c r="I524" s="5" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="J524" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K524" t="n">
+        <v>36336240</v>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" s="2" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E525" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F525" t="n">
+        <v>15</v>
+      </c>
+      <c r="G525" t="n">
+        <v>33</v>
+      </c>
+      <c r="H525" t="inlineStr">
+        <is>
+          <t>15/33</t>
+        </is>
+      </c>
+      <c r="I525" s="4" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="J525" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K525" t="n">
+        <v>36692752</v>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" s="2" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E526" t="inlineStr">
+        <is>
+          <t>Free Flow session</t>
+        </is>
+      </c>
+      <c r="F526" t="n">
+        <v>22</v>
+      </c>
+      <c r="G526" t="n">
+        <v>36</v>
+      </c>
+      <c r="H526" t="inlineStr">
+        <is>
+          <t>22/36</t>
+        </is>
+      </c>
+      <c r="I526" s="5" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="J526" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K526" t="n">
+        <v>36892094</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K519"/>
+  <autoFilter ref="A1:K526"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-06-16)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$526</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$531</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K526"/>
+  <dimension ref="A1:K531"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1342,7 +1342,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F19" t="n">
@@ -1389,7 +1389,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F20" t="n">
@@ -1436,7 +1436,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F21" t="n">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F22" t="n">
@@ -1530,7 +1530,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F23" t="n">
@@ -1577,7 +1577,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F24" t="n">
@@ -1671,7 +1671,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F26" t="n">
@@ -1718,7 +1718,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F27" t="n">
@@ -1765,7 +1765,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F28" t="n">
@@ -1953,7 +1953,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F32" t="n">
@@ -2141,7 +2141,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F40" t="n">
@@ -2376,7 +2376,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F41" t="n">
@@ -2470,7 +2470,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F43" t="n">
@@ -2517,7 +2517,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F44" t="n">
@@ -2658,7 +2658,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F47" t="n">
@@ -2705,7 +2705,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F48" t="n">
@@ -2893,7 +2893,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F52" t="n">
@@ -2940,7 +2940,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F53" t="n">
@@ -2987,7 +2987,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F54" t="n">
@@ -3034,7 +3034,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F55" t="n">
@@ -3316,7 +3316,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F61" t="n">
@@ -3410,7 +3410,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F63" t="n">
@@ -3457,7 +3457,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F64" t="n">
@@ -3504,7 +3504,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F65" t="n">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F66" t="n">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F67" t="n">
@@ -3786,7 +3786,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F71" t="n">
@@ -3974,7 +3974,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F75" t="n">
@@ -4162,7 +4162,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F79" t="n">
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F80" t="n">
@@ -4303,7 +4303,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F82" t="n">
@@ -4350,7 +4350,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F83" t="n">
@@ -4491,7 +4491,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F86" t="n">
@@ -4538,7 +4538,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F87" t="n">
@@ -4726,7 +4726,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F91" t="n">
@@ -4773,7 +4773,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F92" t="n">
@@ -4820,7 +4820,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F93" t="n">
@@ -4867,7 +4867,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F94" t="n">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F95" t="n">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F97" t="n">
@@ -5055,7 +5055,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F98" t="n">
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F101" t="n">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F102" t="n">
@@ -5290,7 +5290,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F103" t="n">
@@ -5337,7 +5337,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F104" t="n">
@@ -5431,7 +5431,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F106" t="n">
@@ -5478,7 +5478,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F107" t="n">
@@ -5572,7 +5572,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F109" t="n">
@@ -5760,7 +5760,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F113" t="n">
@@ -5948,7 +5948,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F117" t="n">
@@ -6042,7 +6042,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F119" t="n">
@@ -6089,7 +6089,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F120" t="n">
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F122" t="n">
@@ -6230,7 +6230,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F123" t="n">
@@ -6324,7 +6324,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F125" t="n">
@@ -6371,7 +6371,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F126" t="n">
@@ -6512,7 +6512,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F129" t="n">
@@ -6559,7 +6559,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F130" t="n">
@@ -6606,7 +6606,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F131" t="n">
@@ -6841,7 +6841,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F136" t="n">
@@ -6888,7 +6888,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F137" t="n">
@@ -6935,7 +6935,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F138" t="n">
@@ -6982,7 +6982,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F139" t="n">
@@ -7076,7 +7076,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F141" t="n">
@@ -7123,7 +7123,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F142" t="n">
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F143" t="n">
@@ -7311,7 +7311,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F146" t="n">
@@ -7405,7 +7405,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F148" t="n">
@@ -7452,7 +7452,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F149" t="n">
@@ -7546,7 +7546,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F151" t="n">
@@ -7593,7 +7593,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F152" t="n">
@@ -7687,7 +7687,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F154" t="n">
@@ -7734,7 +7734,7 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F155" t="n">
@@ -7922,7 +7922,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F159" t="n">
@@ -7969,7 +7969,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F160" t="n">
@@ -8157,7 +8157,7 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F164" t="n">
@@ -8204,7 +8204,7 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F165" t="n">
@@ -8392,7 +8392,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F169" t="n">
@@ -8439,7 +8439,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F170" t="n">
@@ -8533,7 +8533,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F172" t="n">
@@ -8580,7 +8580,7 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F173" t="n">
@@ -8721,7 +8721,7 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F176" t="n">
@@ -8768,7 +8768,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F177" t="n">
@@ -8815,7 +8815,7 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F178" t="n">
@@ -8862,7 +8862,7 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F179" t="n">
@@ -9003,7 +9003,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F182" t="n">
@@ -9050,7 +9050,7 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F183" t="n">
@@ -9097,7 +9097,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F184" t="n">
@@ -9144,7 +9144,7 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F185" t="n">
@@ -9191,7 +9191,7 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F186" t="n">
@@ -9285,7 +9285,7 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F188" t="n">
@@ -9332,7 +9332,7 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F189" t="n">
@@ -9379,7 +9379,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F190" t="n">
@@ -9520,7 +9520,7 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F193" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F195" t="n">
@@ -9661,7 +9661,7 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F196" t="n">
@@ -9755,7 +9755,7 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F198" t="n">
@@ -9802,7 +9802,7 @@
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F199" t="n">
@@ -9896,7 +9896,7 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F201" t="n">
@@ -9943,7 +9943,7 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F202" t="n">
@@ -10272,7 +10272,7 @@
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F209" t="n">
@@ -10319,7 +10319,7 @@
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F210" t="n">
@@ -10366,7 +10366,7 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F211" t="n">
@@ -10460,7 +10460,7 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F213" t="n">
@@ -10507,7 +10507,7 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F214" t="n">
@@ -10742,7 +10742,7 @@
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F219" t="n">
@@ -10883,7 +10883,7 @@
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F222" t="n">
@@ -10930,7 +10930,7 @@
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F223" t="n">
@@ -10977,7 +10977,7 @@
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F224" t="n">
@@ -11118,7 +11118,7 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F227" t="n">
@@ -11212,7 +11212,7 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F229" t="n">
@@ -11259,7 +11259,7 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F230" t="n">
@@ -11306,7 +11306,7 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F231" t="n">
@@ -11353,7 +11353,7 @@
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F232" t="n">
@@ -11400,7 +11400,7 @@
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F233" t="n">
@@ -11447,7 +11447,7 @@
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F234" t="n">
@@ -11494,7 +11494,7 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F235" t="n">
@@ -11541,7 +11541,7 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F236" t="n">
@@ -11588,7 +11588,7 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F237" t="n">
@@ -11635,7 +11635,7 @@
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F238" t="n">
@@ -11682,7 +11682,7 @@
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F239" t="n">
@@ -11870,7 +11870,7 @@
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F243" t="n">
@@ -11917,7 +11917,7 @@
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F244" t="n">
@@ -12011,7 +12011,7 @@
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F246" t="n">
@@ -12058,7 +12058,7 @@
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F247" t="n">
@@ -12105,7 +12105,7 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F248" t="n">
@@ -12152,7 +12152,7 @@
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F249" t="n">
@@ -12199,7 +12199,7 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F250" t="n">
@@ -12387,7 +12387,7 @@
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F254" t="n">
@@ -12434,7 +12434,7 @@
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F255" t="n">
@@ -12575,7 +12575,7 @@
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F258" t="n">
@@ -12622,7 +12622,7 @@
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F259" t="n">
@@ -12669,7 +12669,7 @@
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F260" t="n">
@@ -12763,7 +12763,7 @@
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F262" t="n">
@@ -12810,7 +12810,7 @@
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F263" t="n">
@@ -12951,7 +12951,7 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F266" t="n">
@@ -12998,7 +12998,7 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F267" t="n">
@@ -13233,7 +13233,7 @@
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F272" t="n">
@@ -13280,7 +13280,7 @@
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F273" t="n">
@@ -13327,7 +13327,7 @@
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F274" t="n">
@@ -13421,7 +13421,7 @@
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F276" t="n">
@@ -13468,7 +13468,7 @@
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F277" t="n">
@@ -13515,7 +13515,7 @@
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F278" t="n">
@@ -13656,7 +13656,7 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F281" t="n">
@@ -13703,7 +13703,7 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F282" t="n">
@@ -13750,7 +13750,7 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F283" t="n">
@@ -13797,7 +13797,7 @@
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F284" t="n">
@@ -13844,7 +13844,7 @@
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F285" t="n">
@@ -13938,7 +13938,7 @@
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F287" t="n">
@@ -13985,7 +13985,7 @@
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F288" t="n">
@@ -14032,7 +14032,7 @@
       </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F289" t="n">
@@ -14173,7 +14173,7 @@
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F292" t="n">
@@ -14267,7 +14267,7 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F294" t="n">
@@ -14314,7 +14314,7 @@
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F295" t="n">
@@ -14408,7 +14408,7 @@
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F297" t="n">
@@ -14455,7 +14455,7 @@
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F298" t="n">
@@ -14549,7 +14549,7 @@
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F300" t="n">
@@ -14596,7 +14596,7 @@
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F301" t="n">
@@ -14784,7 +14784,7 @@
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F305" t="n">
@@ -14831,7 +14831,7 @@
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F306" t="n">
@@ -14972,7 +14972,7 @@
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F309" t="n">
@@ -15019,7 +15019,7 @@
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F310" t="n">
@@ -15113,7 +15113,7 @@
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F312" t="n">
@@ -15160,7 +15160,7 @@
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F313" t="n">
@@ -15207,7 +15207,7 @@
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F314" t="n">
@@ -15254,7 +15254,7 @@
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F315" t="n">
@@ -15442,7 +15442,7 @@
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F319" t="n">
@@ -15489,7 +15489,7 @@
       </c>
       <c r="E320" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F320" t="n">
@@ -15630,7 +15630,7 @@
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F323" t="n">
@@ -15677,7 +15677,7 @@
       </c>
       <c r="E324" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F324" t="n">
@@ -15724,7 +15724,7 @@
       </c>
       <c r="E325" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F325" t="n">
@@ -15959,7 +15959,7 @@
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F330" t="n">
@@ -16006,7 +16006,7 @@
       </c>
       <c r="E331" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F331" t="n">
@@ -16053,7 +16053,7 @@
       </c>
       <c r="E332" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F332" t="n">
@@ -16100,7 +16100,7 @@
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F333" t="n">
@@ -16147,7 +16147,7 @@
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F334" t="n">
@@ -16241,7 +16241,7 @@
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F336" t="n">
@@ -16288,7 +16288,7 @@
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F337" t="n">
@@ -16335,7 +16335,7 @@
       </c>
       <c r="E338" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F338" t="n">
@@ -16476,7 +16476,7 @@
       </c>
       <c r="E341" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F341" t="n">
@@ -16570,7 +16570,7 @@
       </c>
       <c r="E343" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F343" t="n">
@@ -16617,7 +16617,7 @@
       </c>
       <c r="E344" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F344" t="n">
@@ -16711,7 +16711,7 @@
       </c>
       <c r="E346" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F346" t="n">
@@ -16758,7 +16758,7 @@
       </c>
       <c r="E347" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F347" t="n">
@@ -16852,7 +16852,7 @@
       </c>
       <c r="E349" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F349" t="n">
@@ -16899,7 +16899,7 @@
       </c>
       <c r="E350" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F350" t="n">
@@ -17087,7 +17087,7 @@
       </c>
       <c r="E354" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F354" t="n">
@@ -17134,7 +17134,7 @@
       </c>
       <c r="E355" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F355" t="n">
@@ -17322,7 +17322,7 @@
       </c>
       <c r="E359" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F359" t="n">
@@ -17369,7 +17369,7 @@
       </c>
       <c r="E360" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F360" t="n">
@@ -17416,7 +17416,7 @@
       </c>
       <c r="E361" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F361" t="n">
@@ -17510,7 +17510,7 @@
       </c>
       <c r="E363" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F363" t="n">
@@ -17557,7 +17557,7 @@
       </c>
       <c r="E364" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F364" t="n">
@@ -17698,7 +17698,7 @@
       </c>
       <c r="E367" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F367" t="n">
@@ -17792,7 +17792,7 @@
       </c>
       <c r="E369" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F369" t="n">
@@ -17839,7 +17839,7 @@
       </c>
       <c r="E370" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F370" t="n">
@@ -17980,7 +17980,7 @@
       </c>
       <c r="E373" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F373" t="n">
@@ -18027,7 +18027,7 @@
       </c>
       <c r="E374" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F374" t="n">
@@ -18074,7 +18074,7 @@
       </c>
       <c r="E375" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F375" t="n">
@@ -18121,7 +18121,7 @@
       </c>
       <c r="E376" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F376" t="n">
@@ -18168,7 +18168,7 @@
       </c>
       <c r="E377" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F377" t="n">
@@ -18403,7 +18403,7 @@
       </c>
       <c r="E382" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F382" t="n">
@@ -18450,7 +18450,7 @@
       </c>
       <c r="E383" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F383" t="n">
@@ -18497,7 +18497,7 @@
       </c>
       <c r="E384" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F384" t="n">
@@ -18591,7 +18591,7 @@
       </c>
       <c r="E386" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F386" t="n">
@@ -18638,7 +18638,7 @@
       </c>
       <c r="E387" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F387" t="n">
@@ -18779,7 +18779,7 @@
       </c>
       <c r="E390" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F390" t="n">
@@ -18873,7 +18873,7 @@
       </c>
       <c r="E392" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F392" t="n">
@@ -18920,7 +18920,7 @@
       </c>
       <c r="E393" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F393" t="n">
@@ -19061,7 +19061,7 @@
       </c>
       <c r="E396" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F396" t="n">
@@ -19155,7 +19155,7 @@
       </c>
       <c r="E398" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F398" t="n">
@@ -19202,7 +19202,7 @@
       </c>
       <c r="E399" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F399" t="n">
@@ -19390,7 +19390,7 @@
       </c>
       <c r="E403" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F403" t="n">
@@ -19437,7 +19437,7 @@
       </c>
       <c r="E404" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F404" t="n">
@@ -19625,7 +19625,7 @@
       </c>
       <c r="E408" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F408" t="n">
@@ -19719,7 +19719,7 @@
       </c>
       <c r="E410" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F410" t="n">
@@ -19766,7 +19766,7 @@
       </c>
       <c r="E411" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F411" t="n">
@@ -19954,7 +19954,7 @@
       </c>
       <c r="E415" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F415" t="n">
@@ -20001,7 +20001,7 @@
       </c>
       <c r="E416" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F416" t="n">
@@ -20142,7 +20142,7 @@
       </c>
       <c r="E419" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F419" t="n">
@@ -20189,7 +20189,7 @@
       </c>
       <c r="E420" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F420" t="n">
@@ -20236,7 +20236,7 @@
       </c>
       <c r="E421" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F421" t="n">
@@ -20377,7 +20377,7 @@
       </c>
       <c r="E424" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F424" t="n">
@@ -20424,7 +20424,7 @@
       </c>
       <c r="E425" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F425" t="n">
@@ -20471,7 +20471,7 @@
       </c>
       <c r="E426" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F426" t="n">
@@ -20565,7 +20565,7 @@
       </c>
       <c r="E428" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F428" t="n">
@@ -20612,7 +20612,7 @@
       </c>
       <c r="E429" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F429" t="n">
@@ -20753,7 +20753,7 @@
       </c>
       <c r="E432" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F432" t="n">
@@ -20847,7 +20847,7 @@
       </c>
       <c r="E434" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F434" t="n">
@@ -20894,7 +20894,7 @@
       </c>
       <c r="E435" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F435" t="n">
@@ -21035,7 +21035,7 @@
       </c>
       <c r="E438" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F438" t="n">
@@ -21129,7 +21129,7 @@
       </c>
       <c r="E440" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F440" t="n">
@@ -21176,7 +21176,7 @@
       </c>
       <c r="E441" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F441" t="n">
@@ -21364,7 +21364,7 @@
       </c>
       <c r="E445" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F445" t="n">
@@ -21411,7 +21411,7 @@
       </c>
       <c r="E446" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F446" t="n">
@@ -21599,7 +21599,7 @@
       </c>
       <c r="E450" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F450" t="n">
@@ -21646,7 +21646,7 @@
       </c>
       <c r="E451" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F451" t="n">
@@ -21693,7 +21693,7 @@
       </c>
       <c r="E452" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F452" t="n">
@@ -21787,7 +21787,7 @@
       </c>
       <c r="E454" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F454" t="n">
@@ -21834,7 +21834,7 @@
       </c>
       <c r="E455" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F455" t="n">
@@ -21975,7 +21975,7 @@
       </c>
       <c r="E458" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F458" t="n">
@@ -22022,7 +22022,7 @@
       </c>
       <c r="E459" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F459" t="n">
@@ -22069,7 +22069,7 @@
       </c>
       <c r="E460" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F460" t="n">
@@ -22210,7 +22210,7 @@
       </c>
       <c r="E463" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F463" t="n">
@@ -22257,7 +22257,7 @@
       </c>
       <c r="E464" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F464" t="n">
@@ -22304,7 +22304,7 @@
       </c>
       <c r="E465" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F465" t="n">
@@ -22351,7 +22351,7 @@
       </c>
       <c r="E466" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F466" t="n">
@@ -22398,7 +22398,7 @@
       </c>
       <c r="E467" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F467" t="n">
@@ -22492,7 +22492,7 @@
       </c>
       <c r="E469" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F469" t="n">
@@ -22586,7 +22586,7 @@
       </c>
       <c r="E471" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F471" t="n">
@@ -22633,7 +22633,7 @@
       </c>
       <c r="E472" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F472" t="n">
@@ -22680,7 +22680,7 @@
       </c>
       <c r="E473" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F473" t="n">
@@ -22774,7 +22774,7 @@
       </c>
       <c r="E475" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F475" t="n">
@@ -22821,7 +22821,7 @@
       </c>
       <c r="E476" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F476" t="n">
@@ -22962,7 +22962,7 @@
       </c>
       <c r="E479" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F479" t="n">
@@ -23056,7 +23056,7 @@
       </c>
       <c r="E481" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F481" t="n">
@@ -23103,7 +23103,7 @@
       </c>
       <c r="E482" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F482" t="n">
@@ -23150,7 +23150,7 @@
       </c>
       <c r="E483" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F483" t="n">
@@ -23338,7 +23338,7 @@
       </c>
       <c r="E487" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F487" t="n">
@@ -23385,7 +23385,7 @@
       </c>
       <c r="E488" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F488" t="n">
@@ -23526,7 +23526,7 @@
       </c>
       <c r="E491" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F491" t="n">
@@ -23620,7 +23620,7 @@
       </c>
       <c r="E493" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F493" t="n">
@@ -23667,7 +23667,7 @@
       </c>
       <c r="E494" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F494" t="n">
@@ -23855,7 +23855,7 @@
       </c>
       <c r="E498" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F498" t="n">
@@ -23902,7 +23902,7 @@
       </c>
       <c r="E499" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F499" t="n">
@@ -23949,7 +23949,7 @@
       </c>
       <c r="E500" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F500" t="n">
@@ -24043,7 +24043,7 @@
       </c>
       <c r="E502" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F502" t="n">
@@ -24090,7 +24090,7 @@
       </c>
       <c r="E503" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F503" t="n">
@@ -24278,7 +24278,7 @@
       </c>
       <c r="E507" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F507" t="n">
@@ -24325,7 +24325,7 @@
       </c>
       <c r="E508" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F508" t="n">
@@ -24466,7 +24466,7 @@
       </c>
       <c r="E511" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F511" t="n">
@@ -24513,7 +24513,7 @@
       </c>
       <c r="E512" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F512" t="n">
@@ -24560,7 +24560,7 @@
       </c>
       <c r="E513" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F513" t="n">
@@ -24654,7 +24654,7 @@
       </c>
       <c r="E515" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F515" t="n">
@@ -24701,7 +24701,7 @@
       </c>
       <c r="E516" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F516" t="n">
@@ -24748,7 +24748,7 @@
       </c>
       <c r="E517" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F517" t="n">
@@ -24889,7 +24889,7 @@
       </c>
       <c r="E520" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F520" t="n">
@@ -24983,7 +24983,7 @@
       </c>
       <c r="E522" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F522" t="n">
@@ -25030,7 +25030,7 @@
       </c>
       <c r="E523" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F523" t="n">
@@ -25171,7 +25171,7 @@
       </c>
       <c r="E526" t="inlineStr">
         <is>
-          <t>Free Flow session</t>
+          <t>Free Flow session session</t>
         </is>
       </c>
       <c r="F526" t="n">
@@ -25197,8 +25197,243 @@
         <v>36892094</v>
       </c>
     </row>
+    <row r="527">
+      <c r="A527" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E527" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F527" t="n">
+        <v>9</v>
+      </c>
+      <c r="G527" t="n">
+        <v>28</v>
+      </c>
+      <c r="H527" t="inlineStr">
+        <is>
+          <t>9/28</t>
+        </is>
+      </c>
+      <c r="I527" s="4" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="J527" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K527" t="n">
+        <v>36390326</v>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="D528" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E528" t="inlineStr">
+        <is>
+          <t>Free Flow session session</t>
+        </is>
+      </c>
+      <c r="F528" t="n">
+        <v>4</v>
+      </c>
+      <c r="G528" t="n">
+        <v>28</v>
+      </c>
+      <c r="H528" t="inlineStr">
+        <is>
+          <t>4/28</t>
+        </is>
+      </c>
+      <c r="I528" s="4" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="J528" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K528" t="n">
+        <v>36281129</v>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="D529" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E529" t="inlineStr">
+        <is>
+          <t>Free Flow session session</t>
+        </is>
+      </c>
+      <c r="F529" t="n">
+        <v>9</v>
+      </c>
+      <c r="G529" t="n">
+        <v>32</v>
+      </c>
+      <c r="H529" t="inlineStr">
+        <is>
+          <t>9/32</t>
+        </is>
+      </c>
+      <c r="I529" s="4" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="J529" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K529" t="n">
+        <v>36928724</v>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D530" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E530" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F530" t="n">
+        <v>10</v>
+      </c>
+      <c r="G530" t="n">
+        <v>28</v>
+      </c>
+      <c r="H530" t="inlineStr">
+        <is>
+          <t>10/28</t>
+        </is>
+      </c>
+      <c r="I530" s="4" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="J530" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K530" t="n">
+        <v>36280993</v>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="D531" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E531" t="inlineStr">
+        <is>
+          <t>Free Flow session session</t>
+        </is>
+      </c>
+      <c r="F531" t="n">
+        <v>19</v>
+      </c>
+      <c r="G531" t="n">
+        <v>32</v>
+      </c>
+      <c r="H531" t="inlineStr">
+        <is>
+          <t>19/32</t>
+        </is>
+      </c>
+      <c r="I531" s="5" t="n">
+        <v>59.4</v>
+      </c>
+      <c r="J531" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K531" t="n">
+        <v>36929030</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K526"/>
+  <autoFilter ref="A1:K531"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-06-17)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$531</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$536</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K531"/>
+  <dimension ref="A1:K536"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -25432,8 +25432,243 @@
         <v>36929030</v>
       </c>
     </row>
+    <row r="532">
+      <c r="A532" s="2" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D532" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E532" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F532" t="n">
+        <v>13</v>
+      </c>
+      <c r="G532" t="n">
+        <v>33</v>
+      </c>
+      <c r="H532" t="inlineStr">
+        <is>
+          <t>13/33</t>
+        </is>
+      </c>
+      <c r="I532" s="4" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="J532" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K532" t="n">
+        <v>36321357</v>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" s="2" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D533" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E533" t="inlineStr">
+        <is>
+          <t>Free Flow session session</t>
+        </is>
+      </c>
+      <c r="F533" t="n">
+        <v>9</v>
+      </c>
+      <c r="G533" t="n">
+        <v>18</v>
+      </c>
+      <c r="H533" t="inlineStr">
+        <is>
+          <t>9/18</t>
+        </is>
+      </c>
+      <c r="I533" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J533" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K533" t="n">
+        <v>36929156</v>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" s="2" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D534" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E534" t="inlineStr">
+        <is>
+          <t>Free Flow session session</t>
+        </is>
+      </c>
+      <c r="F534" t="n">
+        <v>5</v>
+      </c>
+      <c r="G534" t="n">
+        <v>18</v>
+      </c>
+      <c r="H534" t="inlineStr">
+        <is>
+          <t>5/18</t>
+        </is>
+      </c>
+      <c r="I534" s="4" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="J534" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K534" t="n">
+        <v>36298236</v>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" s="2" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D535" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E535" t="inlineStr">
+        <is>
+          <t>Faustine CHOPIN</t>
+        </is>
+      </c>
+      <c r="F535" t="n">
+        <v>22</v>
+      </c>
+      <c r="G535" t="n">
+        <v>33</v>
+      </c>
+      <c r="H535" t="inlineStr">
+        <is>
+          <t>22/33</t>
+        </is>
+      </c>
+      <c r="I535" s="5" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J535" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K535" t="n">
+        <v>36297681</v>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" s="2" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D536" t="inlineStr">
+        <is>
+          <t>RE-LAX  (English version)</t>
+        </is>
+      </c>
+      <c r="E536" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F536" t="n">
+        <v>0</v>
+      </c>
+      <c r="G536" t="n">
+        <v>28</v>
+      </c>
+      <c r="H536" t="inlineStr">
+        <is>
+          <t>0/28</t>
+        </is>
+      </c>
+      <c r="I536" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J536" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K536" t="n">
+        <v>36298043</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K531"/>
+  <autoFilter ref="A1:K536"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-06-18)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$536</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$541</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K536"/>
+  <dimension ref="A1:K541"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1342,7 +1342,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F19" t="n">
@@ -1389,7 +1389,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F20" t="n">
@@ -1436,7 +1436,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F21" t="n">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F22" t="n">
@@ -1530,7 +1530,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F23" t="n">
@@ -1577,7 +1577,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F24" t="n">
@@ -1671,7 +1671,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F26" t="n">
@@ -1718,7 +1718,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F27" t="n">
@@ -1765,7 +1765,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F28" t="n">
@@ -1953,7 +1953,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F32" t="n">
@@ -2141,7 +2141,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F40" t="n">
@@ -2376,7 +2376,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F41" t="n">
@@ -2470,7 +2470,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F43" t="n">
@@ -2517,7 +2517,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F44" t="n">
@@ -2658,7 +2658,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F47" t="n">
@@ -2705,7 +2705,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F48" t="n">
@@ -2893,7 +2893,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F52" t="n">
@@ -2940,7 +2940,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F53" t="n">
@@ -2987,7 +2987,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F54" t="n">
@@ -3034,7 +3034,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F55" t="n">
@@ -3316,7 +3316,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F61" t="n">
@@ -3410,7 +3410,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F63" t="n">
@@ -3457,7 +3457,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F64" t="n">
@@ -3504,7 +3504,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F65" t="n">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F66" t="n">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F67" t="n">
@@ -3786,7 +3786,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F71" t="n">
@@ -3974,7 +3974,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F75" t="n">
@@ -4162,7 +4162,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F79" t="n">
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F80" t="n">
@@ -4303,7 +4303,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F82" t="n">
@@ -4350,7 +4350,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F83" t="n">
@@ -4491,7 +4491,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F86" t="n">
@@ -4538,7 +4538,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F87" t="n">
@@ -4726,7 +4726,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F91" t="n">
@@ -4773,7 +4773,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F92" t="n">
@@ -4820,7 +4820,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F93" t="n">
@@ -4867,7 +4867,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F94" t="n">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F95" t="n">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F97" t="n">
@@ -5055,7 +5055,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F98" t="n">
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F101" t="n">
@@ -5243,7 +5243,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F102" t="n">
@@ -5290,7 +5290,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F103" t="n">
@@ -5337,7 +5337,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F104" t="n">
@@ -5431,7 +5431,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F106" t="n">
@@ -5478,7 +5478,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F107" t="n">
@@ -5572,7 +5572,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F109" t="n">
@@ -5760,7 +5760,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F113" t="n">
@@ -5948,7 +5948,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F117" t="n">
@@ -6042,7 +6042,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F119" t="n">
@@ -6089,7 +6089,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F120" t="n">
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F122" t="n">
@@ -6230,7 +6230,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F123" t="n">
@@ -6324,7 +6324,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F125" t="n">
@@ -6371,7 +6371,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F126" t="n">
@@ -6512,7 +6512,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F129" t="n">
@@ -6559,7 +6559,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F130" t="n">
@@ -6606,7 +6606,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F131" t="n">
@@ -6841,7 +6841,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F136" t="n">
@@ -6888,7 +6888,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F137" t="n">
@@ -6935,7 +6935,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F138" t="n">
@@ -6982,7 +6982,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F139" t="n">
@@ -7076,7 +7076,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F141" t="n">
@@ -7123,7 +7123,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F142" t="n">
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F143" t="n">
@@ -7311,7 +7311,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F146" t="n">
@@ -7405,7 +7405,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F148" t="n">
@@ -7452,7 +7452,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F149" t="n">
@@ -7546,7 +7546,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F151" t="n">
@@ -7593,7 +7593,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F152" t="n">
@@ -7687,7 +7687,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F154" t="n">
@@ -7734,7 +7734,7 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F155" t="n">
@@ -7922,7 +7922,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F159" t="n">
@@ -7969,7 +7969,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F160" t="n">
@@ -8157,7 +8157,7 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F164" t="n">
@@ -8204,7 +8204,7 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F165" t="n">
@@ -8392,7 +8392,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F169" t="n">
@@ -8439,7 +8439,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F170" t="n">
@@ -8533,7 +8533,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F172" t="n">
@@ -8580,7 +8580,7 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F173" t="n">
@@ -8721,7 +8721,7 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F176" t="n">
@@ -8768,7 +8768,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F177" t="n">
@@ -8815,7 +8815,7 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F178" t="n">
@@ -8862,7 +8862,7 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F179" t="n">
@@ -9003,7 +9003,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F182" t="n">
@@ -9050,7 +9050,7 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F183" t="n">
@@ -9097,7 +9097,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F184" t="n">
@@ -9144,7 +9144,7 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F185" t="n">
@@ -9191,7 +9191,7 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F186" t="n">
@@ -9285,7 +9285,7 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F188" t="n">
@@ -9332,7 +9332,7 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F189" t="n">
@@ -9379,7 +9379,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F190" t="n">
@@ -9520,7 +9520,7 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F193" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F195" t="n">
@@ -9661,7 +9661,7 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F196" t="n">
@@ -9755,7 +9755,7 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F198" t="n">
@@ -9802,7 +9802,7 @@
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F199" t="n">
@@ -9896,7 +9896,7 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F201" t="n">
@@ -9943,7 +9943,7 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F202" t="n">
@@ -10272,7 +10272,7 @@
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F209" t="n">
@@ -10319,7 +10319,7 @@
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F210" t="n">
@@ -10366,7 +10366,7 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F211" t="n">
@@ -10460,7 +10460,7 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F213" t="n">
@@ -10507,7 +10507,7 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F214" t="n">
@@ -10742,7 +10742,7 @@
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F219" t="n">
@@ -10883,7 +10883,7 @@
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F222" t="n">
@@ -10930,7 +10930,7 @@
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F223" t="n">
@@ -10977,7 +10977,7 @@
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F224" t="n">
@@ -11118,7 +11118,7 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F227" t="n">
@@ -11212,7 +11212,7 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F229" t="n">
@@ -11259,7 +11259,7 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F230" t="n">
@@ -11306,7 +11306,7 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F231" t="n">
@@ -11353,7 +11353,7 @@
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F232" t="n">
@@ -11400,7 +11400,7 @@
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F233" t="n">
@@ -11447,7 +11447,7 @@
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F234" t="n">
@@ -11494,7 +11494,7 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F235" t="n">
@@ -11541,7 +11541,7 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F236" t="n">
@@ -11588,7 +11588,7 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F237" t="n">
@@ -11635,7 +11635,7 @@
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F238" t="n">
@@ -11682,7 +11682,7 @@
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F239" t="n">
@@ -11870,7 +11870,7 @@
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F243" t="n">
@@ -11917,7 +11917,7 @@
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F244" t="n">
@@ -12011,7 +12011,7 @@
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F246" t="n">
@@ -12058,7 +12058,7 @@
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F247" t="n">
@@ -12105,7 +12105,7 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F248" t="n">
@@ -12152,7 +12152,7 @@
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F249" t="n">
@@ -12199,7 +12199,7 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F250" t="n">
@@ -12387,7 +12387,7 @@
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F254" t="n">
@@ -12434,7 +12434,7 @@
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F255" t="n">
@@ -12575,7 +12575,7 @@
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F258" t="n">
@@ -12622,7 +12622,7 @@
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F259" t="n">
@@ -12669,7 +12669,7 @@
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F260" t="n">
@@ -12763,7 +12763,7 @@
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F262" t="n">
@@ -12810,7 +12810,7 @@
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F263" t="n">
@@ -12951,7 +12951,7 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F266" t="n">
@@ -12998,7 +12998,7 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F267" t="n">
@@ -13233,7 +13233,7 @@
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F272" t="n">
@@ -13280,7 +13280,7 @@
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F273" t="n">
@@ -13327,7 +13327,7 @@
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F274" t="n">
@@ -13421,7 +13421,7 @@
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F276" t="n">
@@ -13468,7 +13468,7 @@
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F277" t="n">
@@ -13515,7 +13515,7 @@
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F278" t="n">
@@ -13656,7 +13656,7 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F281" t="n">
@@ -13703,7 +13703,7 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F282" t="n">
@@ -13750,7 +13750,7 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F283" t="n">
@@ -13797,7 +13797,7 @@
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F284" t="n">
@@ -13844,7 +13844,7 @@
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F285" t="n">
@@ -13938,7 +13938,7 @@
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F287" t="n">
@@ -13985,7 +13985,7 @@
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F288" t="n">
@@ -14032,7 +14032,7 @@
       </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F289" t="n">
@@ -14173,7 +14173,7 @@
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F292" t="n">
@@ -14267,7 +14267,7 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F294" t="n">
@@ -14314,7 +14314,7 @@
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F295" t="n">
@@ -14408,7 +14408,7 @@
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F297" t="n">
@@ -14455,7 +14455,7 @@
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F298" t="n">
@@ -14549,7 +14549,7 @@
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F300" t="n">
@@ -14596,7 +14596,7 @@
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F301" t="n">
@@ -14784,7 +14784,7 @@
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F305" t="n">
@@ -14831,7 +14831,7 @@
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F306" t="n">
@@ -14972,7 +14972,7 @@
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F309" t="n">
@@ -15019,7 +15019,7 @@
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F310" t="n">
@@ -15113,7 +15113,7 @@
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F312" t="n">
@@ -15160,7 +15160,7 @@
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F313" t="n">
@@ -15207,7 +15207,7 @@
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F314" t="n">
@@ -15254,7 +15254,7 @@
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F315" t="n">
@@ -15442,7 +15442,7 @@
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F319" t="n">
@@ -15489,7 +15489,7 @@
       </c>
       <c r="E320" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F320" t="n">
@@ -15630,7 +15630,7 @@
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F323" t="n">
@@ -15677,7 +15677,7 @@
       </c>
       <c r="E324" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F324" t="n">
@@ -15724,7 +15724,7 @@
       </c>
       <c r="E325" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F325" t="n">
@@ -15959,7 +15959,7 @@
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F330" t="n">
@@ -16006,7 +16006,7 @@
       </c>
       <c r="E331" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F331" t="n">
@@ -16053,7 +16053,7 @@
       </c>
       <c r="E332" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F332" t="n">
@@ -16100,7 +16100,7 @@
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F333" t="n">
@@ -16147,7 +16147,7 @@
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F334" t="n">
@@ -16241,7 +16241,7 @@
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F336" t="n">
@@ -16288,7 +16288,7 @@
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F337" t="n">
@@ -16335,7 +16335,7 @@
       </c>
       <c r="E338" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F338" t="n">
@@ -16476,7 +16476,7 @@
       </c>
       <c r="E341" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F341" t="n">
@@ -16570,7 +16570,7 @@
       </c>
       <c r="E343" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F343" t="n">
@@ -16617,7 +16617,7 @@
       </c>
       <c r="E344" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F344" t="n">
@@ -16711,7 +16711,7 @@
       </c>
       <c r="E346" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F346" t="n">
@@ -16758,7 +16758,7 @@
       </c>
       <c r="E347" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F347" t="n">
@@ -16852,7 +16852,7 @@
       </c>
       <c r="E349" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F349" t="n">
@@ -16899,7 +16899,7 @@
       </c>
       <c r="E350" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F350" t="n">
@@ -17087,7 +17087,7 @@
       </c>
       <c r="E354" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F354" t="n">
@@ -17134,7 +17134,7 @@
       </c>
       <c r="E355" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F355" t="n">
@@ -17322,7 +17322,7 @@
       </c>
       <c r="E359" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F359" t="n">
@@ -17369,7 +17369,7 @@
       </c>
       <c r="E360" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F360" t="n">
@@ -17416,7 +17416,7 @@
       </c>
       <c r="E361" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F361" t="n">
@@ -17510,7 +17510,7 @@
       </c>
       <c r="E363" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F363" t="n">
@@ -17557,7 +17557,7 @@
       </c>
       <c r="E364" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F364" t="n">
@@ -17698,7 +17698,7 @@
       </c>
       <c r="E367" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F367" t="n">
@@ -17792,7 +17792,7 @@
       </c>
       <c r="E369" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F369" t="n">
@@ -17839,7 +17839,7 @@
       </c>
       <c r="E370" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F370" t="n">
@@ -17980,7 +17980,7 @@
       </c>
       <c r="E373" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F373" t="n">
@@ -18027,7 +18027,7 @@
       </c>
       <c r="E374" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F374" t="n">
@@ -18074,7 +18074,7 @@
       </c>
       <c r="E375" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F375" t="n">
@@ -18121,7 +18121,7 @@
       </c>
       <c r="E376" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F376" t="n">
@@ -18168,7 +18168,7 @@
       </c>
       <c r="E377" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F377" t="n">
@@ -18403,7 +18403,7 @@
       </c>
       <c r="E382" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F382" t="n">
@@ -18450,7 +18450,7 @@
       </c>
       <c r="E383" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F383" t="n">
@@ -18497,7 +18497,7 @@
       </c>
       <c r="E384" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F384" t="n">
@@ -18591,7 +18591,7 @@
       </c>
       <c r="E386" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F386" t="n">
@@ -18638,7 +18638,7 @@
       </c>
       <c r="E387" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F387" t="n">
@@ -18779,7 +18779,7 @@
       </c>
       <c r="E390" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F390" t="n">
@@ -18873,7 +18873,7 @@
       </c>
       <c r="E392" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F392" t="n">
@@ -18920,7 +18920,7 @@
       </c>
       <c r="E393" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F393" t="n">
@@ -19061,7 +19061,7 @@
       </c>
       <c r="E396" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F396" t="n">
@@ -19155,7 +19155,7 @@
       </c>
       <c r="E398" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F398" t="n">
@@ -19202,7 +19202,7 @@
       </c>
       <c r="E399" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F399" t="n">
@@ -19390,7 +19390,7 @@
       </c>
       <c r="E403" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F403" t="n">
@@ -19437,7 +19437,7 @@
       </c>
       <c r="E404" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F404" t="n">
@@ -19625,7 +19625,7 @@
       </c>
       <c r="E408" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F408" t="n">
@@ -19719,7 +19719,7 @@
       </c>
       <c r="E410" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F410" t="n">
@@ -19766,7 +19766,7 @@
       </c>
       <c r="E411" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F411" t="n">
@@ -19954,7 +19954,7 @@
       </c>
       <c r="E415" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F415" t="n">
@@ -20001,7 +20001,7 @@
       </c>
       <c r="E416" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F416" t="n">
@@ -20142,7 +20142,7 @@
       </c>
       <c r="E419" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F419" t="n">
@@ -20189,7 +20189,7 @@
       </c>
       <c r="E420" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F420" t="n">
@@ -20236,7 +20236,7 @@
       </c>
       <c r="E421" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F421" t="n">
@@ -20377,7 +20377,7 @@
       </c>
       <c r="E424" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F424" t="n">
@@ -20424,7 +20424,7 @@
       </c>
       <c r="E425" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F425" t="n">
@@ -20471,7 +20471,7 @@
       </c>
       <c r="E426" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F426" t="n">
@@ -20565,7 +20565,7 @@
       </c>
       <c r="E428" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F428" t="n">
@@ -20612,7 +20612,7 @@
       </c>
       <c r="E429" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F429" t="n">
@@ -20753,7 +20753,7 @@
       </c>
       <c r="E432" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F432" t="n">
@@ -20847,7 +20847,7 @@
       </c>
       <c r="E434" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F434" t="n">
@@ -20894,7 +20894,7 @@
       </c>
       <c r="E435" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F435" t="n">
@@ -21035,7 +21035,7 @@
       </c>
       <c r="E438" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F438" t="n">
@@ -21129,7 +21129,7 @@
       </c>
       <c r="E440" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F440" t="n">
@@ -21176,7 +21176,7 @@
       </c>
       <c r="E441" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F441" t="n">
@@ -21364,7 +21364,7 @@
       </c>
       <c r="E445" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F445" t="n">
@@ -21411,7 +21411,7 @@
       </c>
       <c r="E446" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F446" t="n">
@@ -21599,7 +21599,7 @@
       </c>
       <c r="E450" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F450" t="n">
@@ -21646,7 +21646,7 @@
       </c>
       <c r="E451" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F451" t="n">
@@ -21693,7 +21693,7 @@
       </c>
       <c r="E452" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F452" t="n">
@@ -21787,7 +21787,7 @@
       </c>
       <c r="E454" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F454" t="n">
@@ -21834,7 +21834,7 @@
       </c>
       <c r="E455" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F455" t="n">
@@ -21975,7 +21975,7 @@
       </c>
       <c r="E458" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F458" t="n">
@@ -22022,7 +22022,7 @@
       </c>
       <c r="E459" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F459" t="n">
@@ -22069,7 +22069,7 @@
       </c>
       <c r="E460" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F460" t="n">
@@ -22210,7 +22210,7 @@
       </c>
       <c r="E463" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F463" t="n">
@@ -22257,7 +22257,7 @@
       </c>
       <c r="E464" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F464" t="n">
@@ -22304,7 +22304,7 @@
       </c>
       <c r="E465" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F465" t="n">
@@ -22351,7 +22351,7 @@
       </c>
       <c r="E466" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F466" t="n">
@@ -22398,7 +22398,7 @@
       </c>
       <c r="E467" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F467" t="n">
@@ -22492,7 +22492,7 @@
       </c>
       <c r="E469" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F469" t="n">
@@ -22586,7 +22586,7 @@
       </c>
       <c r="E471" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F471" t="n">
@@ -22633,7 +22633,7 @@
       </c>
       <c r="E472" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F472" t="n">
@@ -22680,7 +22680,7 @@
       </c>
       <c r="E473" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F473" t="n">
@@ -22774,7 +22774,7 @@
       </c>
       <c r="E475" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F475" t="n">
@@ -22821,7 +22821,7 @@
       </c>
       <c r="E476" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F476" t="n">
@@ -22962,7 +22962,7 @@
       </c>
       <c r="E479" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F479" t="n">
@@ -23056,7 +23056,7 @@
       </c>
       <c r="E481" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F481" t="n">
@@ -23103,7 +23103,7 @@
       </c>
       <c r="E482" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F482" t="n">
@@ -23150,7 +23150,7 @@
       </c>
       <c r="E483" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F483" t="n">
@@ -23338,7 +23338,7 @@
       </c>
       <c r="E487" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F487" t="n">
@@ -23385,7 +23385,7 @@
       </c>
       <c r="E488" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F488" t="n">
@@ -23526,7 +23526,7 @@
       </c>
       <c r="E491" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F491" t="n">
@@ -23620,7 +23620,7 @@
       </c>
       <c r="E493" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F493" t="n">
@@ -23667,7 +23667,7 @@
       </c>
       <c r="E494" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F494" t="n">
@@ -23855,7 +23855,7 @@
       </c>
       <c r="E498" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F498" t="n">
@@ -23902,7 +23902,7 @@
       </c>
       <c r="E499" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F499" t="n">
@@ -23949,7 +23949,7 @@
       </c>
       <c r="E500" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F500" t="n">
@@ -24043,7 +24043,7 @@
       </c>
       <c r="E502" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F502" t="n">
@@ -24090,7 +24090,7 @@
       </c>
       <c r="E503" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F503" t="n">
@@ -24278,7 +24278,7 @@
       </c>
       <c r="E507" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F507" t="n">
@@ -24325,7 +24325,7 @@
       </c>
       <c r="E508" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F508" t="n">
@@ -24466,7 +24466,7 @@
       </c>
       <c r="E511" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F511" t="n">
@@ -24513,7 +24513,7 @@
       </c>
       <c r="E512" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F512" t="n">
@@ -24560,7 +24560,7 @@
       </c>
       <c r="E513" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F513" t="n">
@@ -24654,7 +24654,7 @@
       </c>
       <c r="E515" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F515" t="n">
@@ -24701,7 +24701,7 @@
       </c>
       <c r="E516" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F516" t="n">
@@ -24748,7 +24748,7 @@
       </c>
       <c r="E517" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F517" t="n">
@@ -24889,7 +24889,7 @@
       </c>
       <c r="E520" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F520" t="n">
@@ -24983,7 +24983,7 @@
       </c>
       <c r="E522" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F522" t="n">
@@ -25030,7 +25030,7 @@
       </c>
       <c r="E523" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F523" t="n">
@@ -25171,7 +25171,7 @@
       </c>
       <c r="E526" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F526" t="n">
@@ -25265,7 +25265,7 @@
       </c>
       <c r="E528" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F528" t="n">
@@ -25312,7 +25312,7 @@
       </c>
       <c r="E529" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F529" t="n">
@@ -25406,7 +25406,7 @@
       </c>
       <c r="E531" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F531" t="n">
@@ -25500,7 +25500,7 @@
       </c>
       <c r="E533" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F533" t="n">
@@ -25547,7 +25547,7 @@
       </c>
       <c r="E534" t="inlineStr">
         <is>
-          <t>Free Flow session session</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F534" t="n">
@@ -25667,8 +25667,243 @@
         <v>36298043</v>
       </c>
     </row>
+    <row r="537">
+      <c r="A537" s="2" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D537" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E537" t="inlineStr">
+        <is>
+          <t>alice dunoyer</t>
+        </is>
+      </c>
+      <c r="F537" t="n">
+        <v>8</v>
+      </c>
+      <c r="G537" t="n">
+        <v>33</v>
+      </c>
+      <c r="H537" t="inlineStr">
+        <is>
+          <t>8/33</t>
+        </is>
+      </c>
+      <c r="I537" s="4" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="J537" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K537" t="n">
+        <v>36321406</v>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" s="2" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D538" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E538" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F538" t="n">
+        <v>5</v>
+      </c>
+      <c r="G538" t="n">
+        <v>18</v>
+      </c>
+      <c r="H538" t="inlineStr">
+        <is>
+          <t>5/18</t>
+        </is>
+      </c>
+      <c r="I538" s="4" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="J538" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K538" t="n">
+        <v>36929288</v>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" s="2" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D539" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E539" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F539" t="n">
+        <v>6</v>
+      </c>
+      <c r="G539" t="n">
+        <v>18</v>
+      </c>
+      <c r="H539" t="inlineStr">
+        <is>
+          <t>6/18</t>
+        </is>
+      </c>
+      <c r="I539" s="4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J539" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K539" t="n">
+        <v>36298337</v>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" s="2" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D540" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E540" t="inlineStr">
+        <is>
+          <t>Pauline Ramon</t>
+        </is>
+      </c>
+      <c r="F540" t="n">
+        <v>21</v>
+      </c>
+      <c r="G540" t="n">
+        <v>33</v>
+      </c>
+      <c r="H540" t="inlineStr">
+        <is>
+          <t>21/33</t>
+        </is>
+      </c>
+      <c r="I540" s="5" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="J540" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K540" t="n">
+        <v>36298378</v>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" s="2" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D541" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E541" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F541" t="n">
+        <v>25</v>
+      </c>
+      <c r="G541" t="n">
+        <v>33</v>
+      </c>
+      <c r="H541" t="inlineStr">
+        <is>
+          <t>25/33</t>
+        </is>
+      </c>
+      <c r="I541" s="5" t="n">
+        <v>75.8</v>
+      </c>
+      <c r="J541" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K541" t="n">
+        <v>36298575</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K536"/>
+  <autoFilter ref="A1:K541"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-06-19)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$541</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$550</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K541"/>
+  <dimension ref="A1:K550"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -25902,8 +25902,431 @@
         <v>36298575</v>
       </c>
     </row>
+    <row r="542">
+      <c r="A542" s="2" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>07:45</t>
+        </is>
+      </c>
+      <c r="D542" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E542" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F542" t="n">
+        <v>10</v>
+      </c>
+      <c r="G542" t="n">
+        <v>28</v>
+      </c>
+      <c r="H542" t="inlineStr">
+        <is>
+          <t>10/28</t>
+        </is>
+      </c>
+      <c r="I542" s="4" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="J542" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K542" t="n">
+        <v>37090002</v>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" s="2" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D543" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E543" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F543" t="n">
+        <v>4</v>
+      </c>
+      <c r="G543" t="n">
+        <v>13</v>
+      </c>
+      <c r="H543" t="inlineStr">
+        <is>
+          <t>4/13</t>
+        </is>
+      </c>
+      <c r="I543" s="4" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="J543" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K543" t="n">
+        <v>37230110</v>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" s="2" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="D544" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E544" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F544" t="n">
+        <v>0</v>
+      </c>
+      <c r="G544" t="n">
+        <v>13</v>
+      </c>
+      <c r="H544" t="inlineStr">
+        <is>
+          <t>0/13</t>
+        </is>
+      </c>
+      <c r="I544" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J544" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K544" t="n">
+        <v>37230146</v>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" s="2" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D545" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E545" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F545" t="n">
+        <v>3</v>
+      </c>
+      <c r="G545" t="n">
+        <v>13</v>
+      </c>
+      <c r="H545" t="inlineStr">
+        <is>
+          <t>3/13</t>
+        </is>
+      </c>
+      <c r="I545" s="4" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="J545" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K545" t="n">
+        <v>37090960</v>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" s="2" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E546" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F546" t="n">
+        <v>12</v>
+      </c>
+      <c r="G546" t="n">
+        <v>33</v>
+      </c>
+      <c r="H546" t="inlineStr">
+        <is>
+          <t>12/33</t>
+        </is>
+      </c>
+      <c r="I546" s="4" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="J546" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K546" t="n">
+        <v>36321557</v>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" s="2" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E547" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F547" t="n">
+        <v>0</v>
+      </c>
+      <c r="G547" t="n">
+        <v>18</v>
+      </c>
+      <c r="H547" t="inlineStr">
+        <is>
+          <t>0/18</t>
+        </is>
+      </c>
+      <c r="I547" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J547" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K547" t="n">
+        <v>36929379</v>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" s="2" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D548" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E548" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F548" t="n">
+        <v>11</v>
+      </c>
+      <c r="G548" t="n">
+        <v>18</v>
+      </c>
+      <c r="H548" t="inlineStr">
+        <is>
+          <t>11/18</t>
+        </is>
+      </c>
+      <c r="I548" s="5" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="J548" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K548" t="n">
+        <v>36298752</v>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" s="2" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D549" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E549" t="inlineStr">
+        <is>
+          <t>Faustine CHOPIN</t>
+        </is>
+      </c>
+      <c r="F549" t="n">
+        <v>16</v>
+      </c>
+      <c r="G549" t="n">
+        <v>33</v>
+      </c>
+      <c r="H549" t="inlineStr">
+        <is>
+          <t>16/33</t>
+        </is>
+      </c>
+      <c r="I549" s="4" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="J549" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K549" t="n">
+        <v>36298806</v>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" s="2" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D550" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E550" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F550" t="n">
+        <v>21</v>
+      </c>
+      <c r="G550" t="n">
+        <v>33</v>
+      </c>
+      <c r="H550" t="inlineStr">
+        <is>
+          <t>21/33</t>
+        </is>
+      </c>
+      <c r="I550" s="5" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="J550" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K550" t="n">
+        <v>36298859</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K541"/>
+  <autoFilter ref="A1:K550"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-06-20)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$550</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$557</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K550"/>
+  <dimension ref="A1:K557"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -26325,8 +26325,337 @@
         <v>36298859</v>
       </c>
     </row>
+    <row r="551">
+      <c r="A551" s="2" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D551" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E551" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F551" t="n">
+        <v>4</v>
+      </c>
+      <c r="G551" t="n">
+        <v>33</v>
+      </c>
+      <c r="H551" t="inlineStr">
+        <is>
+          <t>4/33</t>
+        </is>
+      </c>
+      <c r="I551" s="4" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="J551" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K551" t="n">
+        <v>36319495</v>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" s="2" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D552" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E552" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F552" t="n">
+        <v>2</v>
+      </c>
+      <c r="G552" t="n">
+        <v>16</v>
+      </c>
+      <c r="H552" t="inlineStr">
+        <is>
+          <t>2/16</t>
+        </is>
+      </c>
+      <c r="I552" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="J552" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K552" t="n">
+        <v>36320653</v>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" s="2" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D553" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E553" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F553" t="n">
+        <v>4</v>
+      </c>
+      <c r="G553" t="n">
+        <v>16</v>
+      </c>
+      <c r="H553" t="inlineStr">
+        <is>
+          <t>4/16</t>
+        </is>
+      </c>
+      <c r="I553" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="J553" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K553" t="n">
+        <v>36320052</v>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" s="2" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E554" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F554" t="n">
+        <v>21</v>
+      </c>
+      <c r="G554" t="n">
+        <v>33</v>
+      </c>
+      <c r="H554" t="inlineStr">
+        <is>
+          <t>21/33</t>
+        </is>
+      </c>
+      <c r="I554" s="5" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="J554" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K554" t="n">
+        <v>36320776</v>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" s="2" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E555" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F555" t="n">
+        <v>17</v>
+      </c>
+      <c r="G555" t="n">
+        <v>33</v>
+      </c>
+      <c r="H555" t="inlineStr">
+        <is>
+          <t>17/33</t>
+        </is>
+      </c>
+      <c r="I555" s="5" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="J555" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K555" t="n">
+        <v>36320886</v>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" s="2" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D556" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E556" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F556" t="n">
+        <v>13</v>
+      </c>
+      <c r="G556" t="n">
+        <v>20</v>
+      </c>
+      <c r="H556" t="inlineStr">
+        <is>
+          <t>13/20</t>
+        </is>
+      </c>
+      <c r="I556" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="J556" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K556" t="n">
+        <v>36893823</v>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" s="2" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E557" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F557" t="n">
+        <v>7</v>
+      </c>
+      <c r="G557" t="n">
+        <v>20</v>
+      </c>
+      <c r="H557" t="inlineStr">
+        <is>
+          <t>7/20</t>
+        </is>
+      </c>
+      <c r="I557" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="J557" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K557" t="n">
+        <v>36893874</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K550"/>
+  <autoFilter ref="A1:K557"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-06-21)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$557</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$565</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K557"/>
+  <dimension ref="A1:K565"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -26654,8 +26654,384 @@
         <v>36893874</v>
       </c>
     </row>
+    <row r="558">
+      <c r="A558" s="2" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E558" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F558" t="n">
+        <v>8</v>
+      </c>
+      <c r="G558" t="n">
+        <v>32</v>
+      </c>
+      <c r="H558" t="inlineStr">
+        <is>
+          <t>8/32</t>
+        </is>
+      </c>
+      <c r="I558" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="J558" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K558" t="n">
+        <v>36323270</v>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" s="2" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D559" t="inlineStr">
+        <is>
+          <t>RE-BOOST  (English version)</t>
+        </is>
+      </c>
+      <c r="E559" t="inlineStr">
+        <is>
+          <t>alice dunoyer</t>
+        </is>
+      </c>
+      <c r="F559" t="n">
+        <v>16</v>
+      </c>
+      <c r="G559" t="n">
+        <v>33</v>
+      </c>
+      <c r="H559" t="inlineStr">
+        <is>
+          <t>16/33</t>
+        </is>
+      </c>
+      <c r="I559" s="4" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="J559" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K559" t="n">
+        <v>36323116</v>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" s="2" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E560" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F560" t="n">
+        <v>9</v>
+      </c>
+      <c r="G560" t="n">
+        <v>32</v>
+      </c>
+      <c r="H560" t="inlineStr">
+        <is>
+          <t>9/32</t>
+        </is>
+      </c>
+      <c r="I560" s="4" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="J560" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K560" t="n">
+        <v>38771768</v>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" s="2" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E561" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F561" t="n">
+        <v>25</v>
+      </c>
+      <c r="G561" t="n">
+        <v>33</v>
+      </c>
+      <c r="H561" t="inlineStr">
+        <is>
+          <t>25/33</t>
+        </is>
+      </c>
+      <c r="I561" s="5" t="n">
+        <v>75.8</v>
+      </c>
+      <c r="J561" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K561" t="n">
+        <v>36329198</v>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" s="2" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="D562" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E562" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F562" t="n">
+        <v>21</v>
+      </c>
+      <c r="G562" t="n">
+        <v>32</v>
+      </c>
+      <c r="H562" t="inlineStr">
+        <is>
+          <t>21/32</t>
+        </is>
+      </c>
+      <c r="I562" s="5" t="n">
+        <v>65.59999999999999</v>
+      </c>
+      <c r="J562" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K562" t="n">
+        <v>38771868</v>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" s="2" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E563" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F563" t="n">
+        <v>14</v>
+      </c>
+      <c r="G563" t="n">
+        <v>31</v>
+      </c>
+      <c r="H563" t="inlineStr">
+        <is>
+          <t>14/31</t>
+        </is>
+      </c>
+      <c r="I563" s="4" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="J563" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K563" t="n">
+        <v>36329963</v>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" s="2" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D564" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E564" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F564" t="n">
+        <v>0</v>
+      </c>
+      <c r="G564" t="n">
+        <v>20</v>
+      </c>
+      <c r="H564" t="inlineStr">
+        <is>
+          <t>0/20</t>
+        </is>
+      </c>
+      <c r="I564" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J564" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K564" t="n">
+        <v>36935870</v>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" s="2" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="D565" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E565" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F565" t="n">
+        <v>0</v>
+      </c>
+      <c r="G565" t="n">
+        <v>20</v>
+      </c>
+      <c r="H565" t="inlineStr">
+        <is>
+          <t>0/20</t>
+        </is>
+      </c>
+      <c r="I565" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J565" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K565" t="n">
+        <v>36323855</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K557"/>
+  <autoFilter ref="A1:K565"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-06-22)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$565</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$572</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K565"/>
+  <dimension ref="A1:K572"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -27030,8 +27030,337 @@
         <v>36323855</v>
       </c>
     </row>
+    <row r="566">
+      <c r="A566" s="2" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D566" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E566" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F566" t="n">
+        <v>8</v>
+      </c>
+      <c r="G566" t="n">
+        <v>36</v>
+      </c>
+      <c r="H566" t="inlineStr">
+        <is>
+          <t>8/36</t>
+        </is>
+      </c>
+      <c r="I566" s="4" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="J566" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K566" t="n">
+        <v>37240280</v>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" s="2" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E567" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F567" t="n">
+        <v>7</v>
+      </c>
+      <c r="G567" t="n">
+        <v>33</v>
+      </c>
+      <c r="H567" t="inlineStr">
+        <is>
+          <t>7/33</t>
+        </is>
+      </c>
+      <c r="I567" s="4" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="J567" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K567" t="n">
+        <v>36336026</v>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" s="2" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E568" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F568" t="n">
+        <v>6</v>
+      </c>
+      <c r="G568" t="n">
+        <v>28</v>
+      </c>
+      <c r="H568" t="inlineStr">
+        <is>
+          <t>6/28</t>
+        </is>
+      </c>
+      <c r="I568" s="4" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="J568" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K568" t="n">
+        <v>37240423</v>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" s="2" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E569" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F569" t="n">
+        <v>19</v>
+      </c>
+      <c r="G569" t="n">
+        <v>28</v>
+      </c>
+      <c r="H569" t="inlineStr">
+        <is>
+          <t>19/28</t>
+        </is>
+      </c>
+      <c r="I569" s="5" t="n">
+        <v>67.90000000000001</v>
+      </c>
+      <c r="J569" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K569" t="n">
+        <v>36892140</v>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" s="2" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E570" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F570" t="n">
+        <v>16</v>
+      </c>
+      <c r="G570" t="n">
+        <v>32</v>
+      </c>
+      <c r="H570" t="inlineStr">
+        <is>
+          <t>16/32</t>
+        </is>
+      </c>
+      <c r="I570" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J570" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K570" t="n">
+        <v>36336241</v>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" s="2" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E571" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F571" t="n">
+        <v>16</v>
+      </c>
+      <c r="G571" t="n">
+        <v>28</v>
+      </c>
+      <c r="H571" t="inlineStr">
+        <is>
+          <t>16/28</t>
+        </is>
+      </c>
+      <c r="I571" s="5" t="n">
+        <v>57.1</v>
+      </c>
+      <c r="J571" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K571" t="n">
+        <v>36692753</v>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" s="2" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="D572" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E572" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F572" t="n">
+        <v>13</v>
+      </c>
+      <c r="G572" t="n">
+        <v>36</v>
+      </c>
+      <c r="H572" t="inlineStr">
+        <is>
+          <t>13/36</t>
+        </is>
+      </c>
+      <c r="I572" s="4" t="n">
+        <v>36.1</v>
+      </c>
+      <c r="J572" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K572" t="n">
+        <v>36892095</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K565"/>
+  <autoFilter ref="A1:K572"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-06-23)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$572</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$579</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K572"/>
+  <dimension ref="A1:K579"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -27359,8 +27359,337 @@
         <v>36892095</v>
       </c>
     </row>
+    <row r="573">
+      <c r="A573" s="2" t="n">
+        <v>46195</v>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D573" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E573" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F573" t="n">
+        <v>11</v>
+      </c>
+      <c r="G573" t="n">
+        <v>28</v>
+      </c>
+      <c r="H573" t="inlineStr">
+        <is>
+          <t>11/28</t>
+        </is>
+      </c>
+      <c r="I573" s="4" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="J573" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K573" t="n">
+        <v>36390327</v>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" s="2" t="n">
+        <v>46195</v>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E574" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F574" t="n">
+        <v>6</v>
+      </c>
+      <c r="G574" t="n">
+        <v>28</v>
+      </c>
+      <c r="H574" t="inlineStr">
+        <is>
+          <t>6/28</t>
+        </is>
+      </c>
+      <c r="I574" s="4" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="J574" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K574" t="n">
+        <v>36281130</v>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" s="2" t="n">
+        <v>46195</v>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E575" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F575" t="n">
+        <v>5</v>
+      </c>
+      <c r="G575" t="n">
+        <v>18</v>
+      </c>
+      <c r="H575" t="inlineStr">
+        <is>
+          <t>5/18</t>
+        </is>
+      </c>
+      <c r="I575" s="4" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="J575" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K575" t="n">
+        <v>38531906</v>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" s="2" t="n">
+        <v>46195</v>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D576" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E576" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F576" t="n">
+        <v>5</v>
+      </c>
+      <c r="G576" t="n">
+        <v>18</v>
+      </c>
+      <c r="H576" t="inlineStr">
+        <is>
+          <t>5/18</t>
+        </is>
+      </c>
+      <c r="I576" s="4" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="J576" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K576" t="n">
+        <v>36928725</v>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" s="2" t="n">
+        <v>46195</v>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E577" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F577" t="n">
+        <v>8</v>
+      </c>
+      <c r="G577" t="n">
+        <v>28</v>
+      </c>
+      <c r="H577" t="inlineStr">
+        <is>
+          <t>8/28</t>
+        </is>
+      </c>
+      <c r="I577" s="4" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="J577" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K577" t="n">
+        <v>36280994</v>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" s="2" t="n">
+        <v>46195</v>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="D578" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E578" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F578" t="n">
+        <v>11</v>
+      </c>
+      <c r="G578" t="n">
+        <v>28</v>
+      </c>
+      <c r="H578" t="inlineStr">
+        <is>
+          <t>11/28</t>
+        </is>
+      </c>
+      <c r="I578" s="4" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="J578" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K578" t="n">
+        <v>37873136</v>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" s="2" t="n">
+        <v>46195</v>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D579" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E579" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F579" t="n">
+        <v>13</v>
+      </c>
+      <c r="G579" t="n">
+        <v>32</v>
+      </c>
+      <c r="H579" t="inlineStr">
+        <is>
+          <t>13/32</t>
+        </is>
+      </c>
+      <c r="I579" s="4" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="J579" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K579" t="n">
+        <v>36929031</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K572"/>
+  <autoFilter ref="A1:K579"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-06-24)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$579</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$584</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K579"/>
+  <dimension ref="A1:K584"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -27688,8 +27688,243 @@
         <v>36929031</v>
       </c>
     </row>
+    <row r="580">
+      <c r="A580" s="2" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D580" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E580" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F580" t="n">
+        <v>9</v>
+      </c>
+      <c r="G580" t="n">
+        <v>33</v>
+      </c>
+      <c r="H580" t="inlineStr">
+        <is>
+          <t>9/33</t>
+        </is>
+      </c>
+      <c r="I580" s="4" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="J580" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K580" t="n">
+        <v>36321358</v>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" s="2" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D581" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E581" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F581" t="n">
+        <v>5</v>
+      </c>
+      <c r="G581" t="n">
+        <v>18</v>
+      </c>
+      <c r="H581" t="inlineStr">
+        <is>
+          <t>5/18</t>
+        </is>
+      </c>
+      <c r="I581" s="4" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="J581" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K581" t="n">
+        <v>36929157</v>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" s="2" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D582" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E582" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F582" t="n">
+        <v>16</v>
+      </c>
+      <c r="G582" t="n">
+        <v>18</v>
+      </c>
+      <c r="H582" t="inlineStr">
+        <is>
+          <t>16/18</t>
+        </is>
+      </c>
+      <c r="I582" s="3" t="n">
+        <v>88.90000000000001</v>
+      </c>
+      <c r="J582" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K582" t="n">
+        <v>36298237</v>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" s="2" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D583" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E583" t="inlineStr">
+        <is>
+          <t>Faustine CHOPIN</t>
+        </is>
+      </c>
+      <c r="F583" t="n">
+        <v>30</v>
+      </c>
+      <c r="G583" t="n">
+        <v>28</v>
+      </c>
+      <c r="H583" t="inlineStr">
+        <is>
+          <t>30/28</t>
+        </is>
+      </c>
+      <c r="I583" s="3" t="n">
+        <v>107.1</v>
+      </c>
+      <c r="J583" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K583" t="n">
+        <v>36297682</v>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" s="2" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D584" t="inlineStr">
+        <is>
+          <t>RE-LAX  (English version)</t>
+        </is>
+      </c>
+      <c r="E584" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F584" t="n">
+        <v>22</v>
+      </c>
+      <c r="G584" t="n">
+        <v>28</v>
+      </c>
+      <c r="H584" t="inlineStr">
+        <is>
+          <t>22/28</t>
+        </is>
+      </c>
+      <c r="I584" s="5" t="n">
+        <v>78.59999999999999</v>
+      </c>
+      <c r="J584" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K584" t="n">
+        <v>36298044</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K579"/>
+  <autoFilter ref="A1:K584"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-06-25)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$584</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$589</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K584"/>
+  <dimension ref="A1:K589"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -27923,8 +27923,243 @@
         <v>36298044</v>
       </c>
     </row>
+    <row r="585">
+      <c r="A585" s="2" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D585" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E585" t="inlineStr">
+        <is>
+          <t>alice dunoyer</t>
+        </is>
+      </c>
+      <c r="F585" t="n">
+        <v>17</v>
+      </c>
+      <c r="G585" t="n">
+        <v>33</v>
+      </c>
+      <c r="H585" t="inlineStr">
+        <is>
+          <t>17/33</t>
+        </is>
+      </c>
+      <c r="I585" s="5" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="J585" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K585" t="n">
+        <v>36321407</v>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" s="2" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D586" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E586" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F586" t="n">
+        <v>4</v>
+      </c>
+      <c r="G586" t="n">
+        <v>18</v>
+      </c>
+      <c r="H586" t="inlineStr">
+        <is>
+          <t>4/18</t>
+        </is>
+      </c>
+      <c r="I586" s="4" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="J586" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K586" t="n">
+        <v>36929289</v>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" s="2" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D587" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E587" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F587" t="n">
+        <v>10</v>
+      </c>
+      <c r="G587" t="n">
+        <v>18</v>
+      </c>
+      <c r="H587" t="inlineStr">
+        <is>
+          <t>10/18</t>
+        </is>
+      </c>
+      <c r="I587" s="5" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="J587" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K587" t="n">
+        <v>36298338</v>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" s="2" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D588" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E588" t="inlineStr">
+        <is>
+          <t>Pauline Ramon</t>
+        </is>
+      </c>
+      <c r="F588" t="n">
+        <v>23</v>
+      </c>
+      <c r="G588" t="n">
+        <v>33</v>
+      </c>
+      <c r="H588" t="inlineStr">
+        <is>
+          <t>23/33</t>
+        </is>
+      </c>
+      <c r="I588" s="5" t="n">
+        <v>69.7</v>
+      </c>
+      <c r="J588" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K588" t="n">
+        <v>36298379</v>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" s="2" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D589" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E589" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F589" t="n">
+        <v>20</v>
+      </c>
+      <c r="G589" t="n">
+        <v>33</v>
+      </c>
+      <c r="H589" t="inlineStr">
+        <is>
+          <t>20/33</t>
+        </is>
+      </c>
+      <c r="I589" s="5" t="n">
+        <v>60.6</v>
+      </c>
+      <c r="J589" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K589" t="n">
+        <v>36298576</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K584"/>
+  <autoFilter ref="A1:K589"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-06-26)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$589</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$594</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K589"/>
+  <dimension ref="A1:K594"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -28158,8 +28158,243 @@
         <v>36298576</v>
       </c>
     </row>
+    <row r="590">
+      <c r="A590" s="2" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D590" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E590" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F590" t="n">
+        <v>15</v>
+      </c>
+      <c r="G590" t="n">
+        <v>33</v>
+      </c>
+      <c r="H590" t="inlineStr">
+        <is>
+          <t>15/33</t>
+        </is>
+      </c>
+      <c r="I590" s="4" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="J590" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K590" t="n">
+        <v>36321558</v>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" s="2" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D591" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E591" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F591" t="n">
+        <v>8</v>
+      </c>
+      <c r="G591" t="n">
+        <v>18</v>
+      </c>
+      <c r="H591" t="inlineStr">
+        <is>
+          <t>8/18</t>
+        </is>
+      </c>
+      <c r="I591" s="4" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="J591" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K591" t="n">
+        <v>36929380</v>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" s="2" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D592" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E592" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F592" t="n">
+        <v>6</v>
+      </c>
+      <c r="G592" t="n">
+        <v>18</v>
+      </c>
+      <c r="H592" t="inlineStr">
+        <is>
+          <t>6/18</t>
+        </is>
+      </c>
+      <c r="I592" s="4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J592" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K592" t="n">
+        <v>36298753</v>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" s="2" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D593" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E593" t="inlineStr">
+        <is>
+          <t>Faustine CHOPIN</t>
+        </is>
+      </c>
+      <c r="F593" t="n">
+        <v>19</v>
+      </c>
+      <c r="G593" t="n">
+        <v>33</v>
+      </c>
+      <c r="H593" t="inlineStr">
+        <is>
+          <t>19/33</t>
+        </is>
+      </c>
+      <c r="I593" s="5" t="n">
+        <v>57.6</v>
+      </c>
+      <c r="J593" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K593" t="n">
+        <v>36298807</v>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" s="2" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D594" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E594" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F594" t="n">
+        <v>21</v>
+      </c>
+      <c r="G594" t="n">
+        <v>33</v>
+      </c>
+      <c r="H594" t="inlineStr">
+        <is>
+          <t>21/33</t>
+        </is>
+      </c>
+      <c r="I594" s="5" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="J594" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K594" t="n">
+        <v>36298860</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K589"/>
+  <autoFilter ref="A1:K594"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-06-27)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$594</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$601</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K594"/>
+  <dimension ref="A1:K601"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -28393,8 +28393,337 @@
         <v>36298860</v>
       </c>
     </row>
+    <row r="595">
+      <c r="A595" s="2" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D595" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E595" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F595" t="n">
+        <v>9</v>
+      </c>
+      <c r="G595" t="n">
+        <v>33</v>
+      </c>
+      <c r="H595" t="inlineStr">
+        <is>
+          <t>9/33</t>
+        </is>
+      </c>
+      <c r="I595" s="4" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="J595" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K595" t="n">
+        <v>36319496</v>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" s="2" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D596" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E596" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F596" t="n">
+        <v>7</v>
+      </c>
+      <c r="G596" t="n">
+        <v>16</v>
+      </c>
+      <c r="H596" t="inlineStr">
+        <is>
+          <t>7/16</t>
+        </is>
+      </c>
+      <c r="I596" s="4" t="n">
+        <v>43.8</v>
+      </c>
+      <c r="J596" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K596" t="n">
+        <v>36320654</v>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" s="2" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D597" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E597" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F597" t="n">
+        <v>7</v>
+      </c>
+      <c r="G597" t="n">
+        <v>16</v>
+      </c>
+      <c r="H597" t="inlineStr">
+        <is>
+          <t>7/16</t>
+        </is>
+      </c>
+      <c r="I597" s="4" t="n">
+        <v>43.8</v>
+      </c>
+      <c r="J597" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K597" t="n">
+        <v>36320053</v>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" s="2" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D598" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E598" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F598" t="n">
+        <v>11</v>
+      </c>
+      <c r="G598" t="n">
+        <v>33</v>
+      </c>
+      <c r="H598" t="inlineStr">
+        <is>
+          <t>11/33</t>
+        </is>
+      </c>
+      <c r="I598" s="4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J598" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K598" t="n">
+        <v>36320777</v>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" s="2" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D599" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E599" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F599" t="n">
+        <v>27</v>
+      </c>
+      <c r="G599" t="n">
+        <v>33</v>
+      </c>
+      <c r="H599" t="inlineStr">
+        <is>
+          <t>27/33</t>
+        </is>
+      </c>
+      <c r="I599" s="5" t="n">
+        <v>81.8</v>
+      </c>
+      <c r="J599" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K599" t="n">
+        <v>36320887</v>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" s="2" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D600" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E600" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F600" t="n">
+        <v>12</v>
+      </c>
+      <c r="G600" t="n">
+        <v>20</v>
+      </c>
+      <c r="H600" t="inlineStr">
+        <is>
+          <t>12/20</t>
+        </is>
+      </c>
+      <c r="I600" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="J600" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K600" t="n">
+        <v>36893824</v>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" s="2" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D601" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E601" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F601" t="n">
+        <v>9</v>
+      </c>
+      <c r="G601" t="n">
+        <v>20</v>
+      </c>
+      <c r="H601" t="inlineStr">
+        <is>
+          <t>9/20</t>
+        </is>
+      </c>
+      <c r="I601" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="J601" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K601" t="n">
+        <v>36893876</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K594"/>
+  <autoFilter ref="A1:K601"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-06-28)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$601</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$607</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K601"/>
+  <dimension ref="A1:K607"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -28722,8 +28722,290 @@
         <v>36893876</v>
       </c>
     </row>
+    <row r="602">
+      <c r="A602" s="2" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D602" t="inlineStr">
+        <is>
+          <t>Aufguss Sauna Festival - Jan &amp; Sigrid</t>
+        </is>
+      </c>
+      <c r="E602" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F602" t="n">
+        <v>11</v>
+      </c>
+      <c r="G602" t="n">
+        <v>35</v>
+      </c>
+      <c r="H602" t="inlineStr">
+        <is>
+          <t>11/35</t>
+        </is>
+      </c>
+      <c r="I602" s="4" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="J602" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K602" t="n">
+        <v>39014126</v>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" s="2" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D603" t="inlineStr">
+        <is>
+          <t>Aufguss Sauna Festival - Laura + Sigrid &amp; Job</t>
+        </is>
+      </c>
+      <c r="E603" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F603" t="n">
+        <v>17</v>
+      </c>
+      <c r="G603" t="n">
+        <v>35</v>
+      </c>
+      <c r="H603" t="inlineStr">
+        <is>
+          <t>17/35</t>
+        </is>
+      </c>
+      <c r="I603" s="4" t="n">
+        <v>48.6</v>
+      </c>
+      <c r="J603" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K603" t="n">
+        <v>39014222</v>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" s="2" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D604" t="inlineStr">
+        <is>
+          <t>Aufguss Sauna Festival - Adrien + Jean-Louis</t>
+        </is>
+      </c>
+      <c r="E604" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F604" t="n">
+        <v>7</v>
+      </c>
+      <c r="G604" t="n">
+        <v>35</v>
+      </c>
+      <c r="H604" t="inlineStr">
+        <is>
+          <t>7/35</t>
+        </is>
+      </c>
+      <c r="I604" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J604" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K604" t="n">
+        <v>39015567</v>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" s="2" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="D605" t="inlineStr">
+        <is>
+          <t>Aufguss Sauna Festival - Simon + Job</t>
+        </is>
+      </c>
+      <c r="E605" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F605" t="n">
+        <v>27</v>
+      </c>
+      <c r="G605" t="n">
+        <v>35</v>
+      </c>
+      <c r="H605" t="inlineStr">
+        <is>
+          <t>27/35</t>
+        </is>
+      </c>
+      <c r="I605" s="5" t="n">
+        <v>77.09999999999999</v>
+      </c>
+      <c r="J605" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K605" t="n">
+        <v>39015912</v>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" s="2" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D606" t="inlineStr">
+        <is>
+          <t>Aufguss Sauna Festival - Jan + Laura</t>
+        </is>
+      </c>
+      <c r="E606" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F606" t="n">
+        <v>30</v>
+      </c>
+      <c r="G606" t="n">
+        <v>35</v>
+      </c>
+      <c r="H606" t="inlineStr">
+        <is>
+          <t>30/35</t>
+        </is>
+      </c>
+      <c r="I606" s="3" t="n">
+        <v>85.7</v>
+      </c>
+      <c r="J606" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K606" t="n">
+        <v>39016270</v>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" s="2" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="D607" t="inlineStr">
+        <is>
+          <t>Aufguss Sauna Festival - Jean-Louis + Sigrid</t>
+        </is>
+      </c>
+      <c r="E607" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F607" t="n">
+        <v>15</v>
+      </c>
+      <c r="G607" t="n">
+        <v>35</v>
+      </c>
+      <c r="H607" t="inlineStr">
+        <is>
+          <t>15/35</t>
+        </is>
+      </c>
+      <c r="I607" s="4" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="J607" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K607" t="n">
+        <v>39016548</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K601"/>
+  <autoFilter ref="A1:K607"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-06-29)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$607</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$613</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K607"/>
+  <dimension ref="A1:K613"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -28841,18 +28841,18 @@
         </is>
       </c>
       <c r="F604" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G604" t="n">
         <v>35</v>
       </c>
       <c r="H604" t="inlineStr">
         <is>
-          <t>7/35</t>
+          <t>6/35</t>
         </is>
       </c>
       <c r="I604" s="4" t="n">
-        <v>20</v>
+        <v>17.1</v>
       </c>
       <c r="J604" t="inlineStr">
         <is>
@@ -29004,8 +29004,290 @@
         <v>39016548</v>
       </c>
     </row>
+    <row r="608">
+      <c r="A608" s="2" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D608" t="inlineStr">
+        <is>
+          <t>Aufguss Sauna Festival - Simon + Laura</t>
+        </is>
+      </c>
+      <c r="E608" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F608" t="n">
+        <v>7</v>
+      </c>
+      <c r="G608" t="n">
+        <v>35</v>
+      </c>
+      <c r="H608" t="inlineStr">
+        <is>
+          <t>7/35</t>
+        </is>
+      </c>
+      <c r="I608" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J608" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K608" t="n">
+        <v>39016575</v>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" s="2" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D609" t="inlineStr">
+        <is>
+          <t>Aufguss Sauna Festival - Jan + Sigrid / Job / Laura</t>
+        </is>
+      </c>
+      <c r="E609" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F609" t="n">
+        <v>15</v>
+      </c>
+      <c r="G609" t="n">
+        <v>35</v>
+      </c>
+      <c r="H609" t="inlineStr">
+        <is>
+          <t>15/35</t>
+        </is>
+      </c>
+      <c r="I609" s="4" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="J609" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K609" t="n">
+        <v>39016601</v>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" s="2" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D610" t="inlineStr">
+        <is>
+          <t>Aufguss Sauna Festival - Simon + Jean-Louis</t>
+        </is>
+      </c>
+      <c r="E610" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F610" t="n">
+        <v>11</v>
+      </c>
+      <c r="G610" t="n">
+        <v>35</v>
+      </c>
+      <c r="H610" t="inlineStr">
+        <is>
+          <t>11/35</t>
+        </is>
+      </c>
+      <c r="I610" s="4" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="J610" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K610" t="n">
+        <v>39016605</v>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" s="2" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="D611" t="inlineStr">
+        <is>
+          <t>Aufguss Sauna Festival - Adrien + Jean-Louis</t>
+        </is>
+      </c>
+      <c r="E611" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F611" t="n">
+        <v>29</v>
+      </c>
+      <c r="G611" t="n">
+        <v>35</v>
+      </c>
+      <c r="H611" t="inlineStr">
+        <is>
+          <t>29/35</t>
+        </is>
+      </c>
+      <c r="I611" s="5" t="n">
+        <v>82.90000000000001</v>
+      </c>
+      <c r="J611" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K611" t="n">
+        <v>39016633</v>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" s="2" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="D612" t="inlineStr">
+        <is>
+          <t>Aufguss Sauna Festival - Jan + Adrien</t>
+        </is>
+      </c>
+      <c r="E612" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F612" t="n">
+        <v>28</v>
+      </c>
+      <c r="G612" t="n">
+        <v>35</v>
+      </c>
+      <c r="H612" t="inlineStr">
+        <is>
+          <t>28/35</t>
+        </is>
+      </c>
+      <c r="I612" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="J612" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K612" t="n">
+        <v>39016637</v>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" s="2" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F613" t="n">
+        <v>36</v>
+      </c>
+      <c r="G613" t="n">
+        <v>36</v>
+      </c>
+      <c r="H613" t="inlineStr">
+        <is>
+          <t>36/36</t>
+        </is>
+      </c>
+      <c r="I613" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J613" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K613" t="n">
+        <v>36892096</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K607"/>
+  <autoFilter ref="A1:K613"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-06-30)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$613</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$620</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K613"/>
+  <dimension ref="A1:K620"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29286,8 +29286,337 @@
         <v>36892096</v>
       </c>
     </row>
+    <row r="614">
+      <c r="A614" s="2" t="n">
+        <v>46202</v>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E614" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F614" t="n">
+        <v>11</v>
+      </c>
+      <c r="G614" t="n">
+        <v>28</v>
+      </c>
+      <c r="H614" t="inlineStr">
+        <is>
+          <t>11/28</t>
+        </is>
+      </c>
+      <c r="I614" s="4" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="J614" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K614" t="n">
+        <v>36390328</v>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" s="2" t="n">
+        <v>46202</v>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E615" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F615" t="n">
+        <v>10</v>
+      </c>
+      <c r="G615" t="n">
+        <v>28</v>
+      </c>
+      <c r="H615" t="inlineStr">
+        <is>
+          <t>10/28</t>
+        </is>
+      </c>
+      <c r="I615" s="4" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="J615" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K615" t="n">
+        <v>36281131</v>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" s="2" t="n">
+        <v>46202</v>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F616" t="n">
+        <v>2</v>
+      </c>
+      <c r="G616" t="n">
+        <v>18</v>
+      </c>
+      <c r="H616" t="inlineStr">
+        <is>
+          <t>2/18</t>
+        </is>
+      </c>
+      <c r="I616" s="4" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="J616" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K616" t="n">
+        <v>38531907</v>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" s="2" t="n">
+        <v>46202</v>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F617" t="n">
+        <v>1</v>
+      </c>
+      <c r="G617" t="n">
+        <v>18</v>
+      </c>
+      <c r="H617" t="inlineStr">
+        <is>
+          <t>1/18</t>
+        </is>
+      </c>
+      <c r="I617" s="4" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="J617" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K617" t="n">
+        <v>36928726</v>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" s="2" t="n">
+        <v>46202</v>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D618" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E618" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F618" t="n">
+        <v>13</v>
+      </c>
+      <c r="G618" t="n">
+        <v>28</v>
+      </c>
+      <c r="H618" t="inlineStr">
+        <is>
+          <t>13/28</t>
+        </is>
+      </c>
+      <c r="I618" s="4" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="J618" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K618" t="n">
+        <v>36280995</v>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" s="2" t="n">
+        <v>46202</v>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="D619" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E619" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F619" t="n">
+        <v>18</v>
+      </c>
+      <c r="G619" t="n">
+        <v>28</v>
+      </c>
+      <c r="H619" t="inlineStr">
+        <is>
+          <t>18/28</t>
+        </is>
+      </c>
+      <c r="I619" s="5" t="n">
+        <v>64.3</v>
+      </c>
+      <c r="J619" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K619" t="n">
+        <v>37873137</v>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" s="2" t="n">
+        <v>46202</v>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D620" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E620" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F620" t="n">
+        <v>15</v>
+      </c>
+      <c r="G620" t="n">
+        <v>32</v>
+      </c>
+      <c r="H620" t="inlineStr">
+        <is>
+          <t>15/32</t>
+        </is>
+      </c>
+      <c r="I620" s="4" t="n">
+        <v>46.9</v>
+      </c>
+      <c r="J620" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K620" t="n">
+        <v>36929032</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K613"/>
+  <autoFilter ref="A1:K620"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-07-01)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$620</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$626</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K620"/>
+  <dimension ref="A1:K626"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29615,8 +29615,290 @@
         <v>36929032</v>
       </c>
     </row>
+    <row r="621">
+      <c r="A621" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E621" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F621" t="n">
+        <v>11</v>
+      </c>
+      <c r="G621" t="n">
+        <v>33</v>
+      </c>
+      <c r="H621" t="inlineStr">
+        <is>
+          <t>11/33</t>
+        </is>
+      </c>
+      <c r="I621" s="4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J621" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K621" t="n">
+        <v>36321359</v>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D622" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E622" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F622" t="n">
+        <v>9</v>
+      </c>
+      <c r="G622" t="n">
+        <v>18</v>
+      </c>
+      <c r="H622" t="inlineStr">
+        <is>
+          <t>9/18</t>
+        </is>
+      </c>
+      <c r="I622" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J622" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K622" t="n">
+        <v>36929158</v>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D623" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F623" t="n">
+        <v>8</v>
+      </c>
+      <c r="G623" t="n">
+        <v>18</v>
+      </c>
+      <c r="H623" t="inlineStr">
+        <is>
+          <t>8/18</t>
+        </is>
+      </c>
+      <c r="I623" s="4" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="J623" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K623" t="n">
+        <v>36298238</v>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D624" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F624" t="n">
+        <v>16</v>
+      </c>
+      <c r="G624" t="n">
+        <v>28</v>
+      </c>
+      <c r="H624" t="inlineStr">
+        <is>
+          <t>16/28</t>
+        </is>
+      </c>
+      <c r="I624" s="5" t="n">
+        <v>57.1</v>
+      </c>
+      <c r="J624" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K624" t="n">
+        <v>36297683</v>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="D625" t="inlineStr">
+        <is>
+          <t>RE-LAX  (English version)</t>
+        </is>
+      </c>
+      <c r="E625" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F625" t="n">
+        <v>13</v>
+      </c>
+      <c r="G625" t="n">
+        <v>28</v>
+      </c>
+      <c r="H625" t="inlineStr">
+        <is>
+          <t>13/28</t>
+        </is>
+      </c>
+      <c r="I625" s="4" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="J625" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K625" t="n">
+        <v>36298045</v>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D626" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E626" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F626" t="n">
+        <v>13</v>
+      </c>
+      <c r="G626" t="n">
+        <v>32</v>
+      </c>
+      <c r="H626" t="inlineStr">
+        <is>
+          <t>13/32</t>
+        </is>
+      </c>
+      <c r="I626" s="4" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="J626" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K626" t="n">
+        <v>38946307</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K620"/>
+  <autoFilter ref="A1:K626"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-07-02)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$626</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$631</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K626"/>
+  <dimension ref="A1:K631"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29897,8 +29897,243 @@
         <v>38946307</v>
       </c>
     </row>
+    <row r="627">
+      <c r="A627" s="2" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D627" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E627" t="inlineStr">
+        <is>
+          <t>alice dunoyer</t>
+        </is>
+      </c>
+      <c r="F627" t="n">
+        <v>14</v>
+      </c>
+      <c r="G627" t="n">
+        <v>33</v>
+      </c>
+      <c r="H627" t="inlineStr">
+        <is>
+          <t>14/33</t>
+        </is>
+      </c>
+      <c r="I627" s="4" t="n">
+        <v>42.4</v>
+      </c>
+      <c r="J627" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K627" t="n">
+        <v>36321408</v>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" s="2" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D628" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F628" t="n">
+        <v>4</v>
+      </c>
+      <c r="G628" t="n">
+        <v>18</v>
+      </c>
+      <c r="H628" t="inlineStr">
+        <is>
+          <t>4/18</t>
+        </is>
+      </c>
+      <c r="I628" s="4" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="J628" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K628" t="n">
+        <v>36929290</v>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" s="2" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D629" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E629" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F629" t="n">
+        <v>4</v>
+      </c>
+      <c r="G629" t="n">
+        <v>18</v>
+      </c>
+      <c r="H629" t="inlineStr">
+        <is>
+          <t>4/18</t>
+        </is>
+      </c>
+      <c r="I629" s="4" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="J629" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K629" t="n">
+        <v>36298339</v>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" s="2" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D630" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E630" t="inlineStr">
+        <is>
+          <t>Pauline Ramon</t>
+        </is>
+      </c>
+      <c r="F630" t="n">
+        <v>10</v>
+      </c>
+      <c r="G630" t="n">
+        <v>33</v>
+      </c>
+      <c r="H630" t="inlineStr">
+        <is>
+          <t>10/33</t>
+        </is>
+      </c>
+      <c r="I630" s="4" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="J630" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K630" t="n">
+        <v>36298380</v>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" s="2" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D631" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E631" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F631" t="n">
+        <v>16</v>
+      </c>
+      <c r="G631" t="n">
+        <v>33</v>
+      </c>
+      <c r="H631" t="inlineStr">
+        <is>
+          <t>16/33</t>
+        </is>
+      </c>
+      <c r="I631" s="4" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="J631" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K631" t="n">
+        <v>36298577</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K626"/>
+  <autoFilter ref="A1:K631"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-07-03)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$631</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$640</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K631"/>
+  <dimension ref="A1:K640"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30132,8 +30132,431 @@
         <v>36298577</v>
       </c>
     </row>
+    <row r="632">
+      <c r="A632" s="2" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>07:45</t>
+        </is>
+      </c>
+      <c r="D632" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E632" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F632" t="n">
+        <v>8</v>
+      </c>
+      <c r="G632" t="n">
+        <v>28</v>
+      </c>
+      <c r="H632" t="inlineStr">
+        <is>
+          <t>8/28</t>
+        </is>
+      </c>
+      <c r="I632" s="4" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="J632" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K632" t="n">
+        <v>37090004</v>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" s="2" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D633" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E633" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F633" t="n">
+        <v>3</v>
+      </c>
+      <c r="G633" t="n">
+        <v>13</v>
+      </c>
+      <c r="H633" t="inlineStr">
+        <is>
+          <t>3/13</t>
+        </is>
+      </c>
+      <c r="I633" s="4" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="J633" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K633" t="n">
+        <v>37230112</v>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" s="2" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="D634" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E634" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F634" t="n">
+        <v>2</v>
+      </c>
+      <c r="G634" t="n">
+        <v>13</v>
+      </c>
+      <c r="H634" t="inlineStr">
+        <is>
+          <t>2/13</t>
+        </is>
+      </c>
+      <c r="I634" s="4" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="J634" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K634" t="n">
+        <v>37230148</v>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" s="2" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E635" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F635" t="n">
+        <v>1</v>
+      </c>
+      <c r="G635" t="n">
+        <v>13</v>
+      </c>
+      <c r="H635" t="inlineStr">
+        <is>
+          <t>1/13</t>
+        </is>
+      </c>
+      <c r="I635" s="4" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="J635" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K635" t="n">
+        <v>37090962</v>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" s="2" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E636" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F636" t="n">
+        <v>13</v>
+      </c>
+      <c r="G636" t="n">
+        <v>33</v>
+      </c>
+      <c r="H636" t="inlineStr">
+        <is>
+          <t>13/33</t>
+        </is>
+      </c>
+      <c r="I636" s="4" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="J636" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K636" t="n">
+        <v>36321559</v>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" s="2" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D637" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F637" t="n">
+        <v>8</v>
+      </c>
+      <c r="G637" t="n">
+        <v>18</v>
+      </c>
+      <c r="H637" t="inlineStr">
+        <is>
+          <t>8/18</t>
+        </is>
+      </c>
+      <c r="I637" s="4" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="J637" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K637" t="n">
+        <v>36929381</v>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" s="2" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F638" t="n">
+        <v>4</v>
+      </c>
+      <c r="G638" t="n">
+        <v>18</v>
+      </c>
+      <c r="H638" t="inlineStr">
+        <is>
+          <t>4/18</t>
+        </is>
+      </c>
+      <c r="I638" s="4" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="J638" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K638" t="n">
+        <v>36298754</v>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" s="2" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E639" t="inlineStr">
+        <is>
+          <t>Faustine CHOPIN</t>
+        </is>
+      </c>
+      <c r="F639" t="n">
+        <v>15</v>
+      </c>
+      <c r="G639" t="n">
+        <v>33</v>
+      </c>
+      <c r="H639" t="inlineStr">
+        <is>
+          <t>15/33</t>
+        </is>
+      </c>
+      <c r="I639" s="4" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="J639" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K639" t="n">
+        <v>36298808</v>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" s="2" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D640" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E640" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F640" t="n">
+        <v>27</v>
+      </c>
+      <c r="G640" t="n">
+        <v>33</v>
+      </c>
+      <c r="H640" t="inlineStr">
+        <is>
+          <t>27/33</t>
+        </is>
+      </c>
+      <c r="I640" s="5" t="n">
+        <v>81.8</v>
+      </c>
+      <c r="J640" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K640" t="n">
+        <v>36298861</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K631"/>
+  <autoFilter ref="A1:K640"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-07-04)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$640</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$648</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K640"/>
+  <dimension ref="A1:K648"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30555,8 +30555,384 @@
         <v>36298861</v>
       </c>
     </row>
+    <row r="641">
+      <c r="A641" s="2" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="D641" t="inlineStr">
+        <is>
+          <t>Session 1 - Formation founding coachs</t>
+        </is>
+      </c>
+      <c r="E641" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F641" t="n">
+        <v>4</v>
+      </c>
+      <c r="G641" t="n">
+        <v>28</v>
+      </c>
+      <c r="H641" t="inlineStr">
+        <is>
+          <t>4/28</t>
+        </is>
+      </c>
+      <c r="I641" s="4" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="J641" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K641" t="n">
+        <v>39406900</v>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" s="2" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D642" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E642" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F642" t="n">
+        <v>12</v>
+      </c>
+      <c r="G642" t="n">
+        <v>33</v>
+      </c>
+      <c r="H642" t="inlineStr">
+        <is>
+          <t>12/33</t>
+        </is>
+      </c>
+      <c r="I642" s="4" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="J642" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K642" t="n">
+        <v>36319497</v>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" s="2" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D643" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E643" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F643" t="n">
+        <v>4</v>
+      </c>
+      <c r="G643" t="n">
+        <v>16</v>
+      </c>
+      <c r="H643" t="inlineStr">
+        <is>
+          <t>4/16</t>
+        </is>
+      </c>
+      <c r="I643" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="J643" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K643" t="n">
+        <v>36320655</v>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" s="2" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D644" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E644" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F644" t="n">
+        <v>2</v>
+      </c>
+      <c r="G644" t="n">
+        <v>16</v>
+      </c>
+      <c r="H644" t="inlineStr">
+        <is>
+          <t>2/16</t>
+        </is>
+      </c>
+      <c r="I644" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="J644" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K644" t="n">
+        <v>36320054</v>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" s="2" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D645" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E645" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F645" t="n">
+        <v>17</v>
+      </c>
+      <c r="G645" t="n">
+        <v>33</v>
+      </c>
+      <c r="H645" t="inlineStr">
+        <is>
+          <t>17/33</t>
+        </is>
+      </c>
+      <c r="I645" s="5" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="J645" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K645" t="n">
+        <v>36320778</v>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" s="2" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D646" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F646" t="n">
+        <v>11</v>
+      </c>
+      <c r="G646" t="n">
+        <v>33</v>
+      </c>
+      <c r="H646" t="inlineStr">
+        <is>
+          <t>11/33</t>
+        </is>
+      </c>
+      <c r="I646" s="4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J646" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K646" t="n">
+        <v>36320888</v>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" s="2" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F647" t="n">
+        <v>12</v>
+      </c>
+      <c r="G647" t="n">
+        <v>12</v>
+      </c>
+      <c r="H647" t="inlineStr">
+        <is>
+          <t>12/12</t>
+        </is>
+      </c>
+      <c r="I647" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J647" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K647" t="n">
+        <v>36893825</v>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" s="2" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F648" t="n">
+        <v>4</v>
+      </c>
+      <c r="G648" t="n">
+        <v>8</v>
+      </c>
+      <c r="H648" t="inlineStr">
+        <is>
+          <t>4/8</t>
+        </is>
+      </c>
+      <c r="I648" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J648" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K648" t="n">
+        <v>36893878</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K640"/>
+  <autoFilter ref="A1:K648"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-07-05)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$648</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$656</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K648"/>
+  <dimension ref="A1:K656"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30931,8 +30931,384 @@
         <v>36893878</v>
       </c>
     </row>
+    <row r="649">
+      <c r="A649" s="2" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F649" t="n">
+        <v>13</v>
+      </c>
+      <c r="G649" t="n">
+        <v>32</v>
+      </c>
+      <c r="H649" t="inlineStr">
+        <is>
+          <t>13/32</t>
+        </is>
+      </c>
+      <c r="I649" s="4" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="J649" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K649" t="n">
+        <v>36323272</v>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" s="2" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>alice dunoyer</t>
+        </is>
+      </c>
+      <c r="F650" t="n">
+        <v>4</v>
+      </c>
+      <c r="G650" t="n">
+        <v>33</v>
+      </c>
+      <c r="H650" t="inlineStr">
+        <is>
+          <t>4/33</t>
+        </is>
+      </c>
+      <c r="I650" s="4" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="J650" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K650" t="n">
+        <v>36323118</v>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" s="2" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F651" t="n">
+        <v>10</v>
+      </c>
+      <c r="G651" t="n">
+        <v>32</v>
+      </c>
+      <c r="H651" t="inlineStr">
+        <is>
+          <t>10/32</t>
+        </is>
+      </c>
+      <c r="I651" s="4" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="J651" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K651" t="n">
+        <v>38771770</v>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" s="2" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F652" t="n">
+        <v>7</v>
+      </c>
+      <c r="G652" t="n">
+        <v>33</v>
+      </c>
+      <c r="H652" t="inlineStr">
+        <is>
+          <t>7/33</t>
+        </is>
+      </c>
+      <c r="I652" s="4" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="J652" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K652" t="n">
+        <v>36329200</v>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" s="2" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E653" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F653" t="n">
+        <v>7</v>
+      </c>
+      <c r="G653" t="n">
+        <v>32</v>
+      </c>
+      <c r="H653" t="inlineStr">
+        <is>
+          <t>7/32</t>
+        </is>
+      </c>
+      <c r="I653" s="4" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="J653" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K653" t="n">
+        <v>38771870</v>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" s="2" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E654" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F654" t="n">
+        <v>9</v>
+      </c>
+      <c r="G654" t="n">
+        <v>33</v>
+      </c>
+      <c r="H654" t="inlineStr">
+        <is>
+          <t>9/33</t>
+        </is>
+      </c>
+      <c r="I654" s="4" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="J654" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K654" t="n">
+        <v>36329965</v>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" s="2" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F655" t="n">
+        <v>0</v>
+      </c>
+      <c r="G655" t="n">
+        <v>20</v>
+      </c>
+      <c r="H655" t="inlineStr">
+        <is>
+          <t>0/20</t>
+        </is>
+      </c>
+      <c r="I655" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J655" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K655" t="n">
+        <v>36935872</v>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" s="2" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E656" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F656" t="n">
+        <v>0</v>
+      </c>
+      <c r="G656" t="n">
+        <v>20</v>
+      </c>
+      <c r="H656" t="inlineStr">
+        <is>
+          <t>0/20</t>
+        </is>
+      </c>
+      <c r="I656" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J656" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K656" t="n">
+        <v>36323857</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K648"/>
+  <autoFilter ref="A1:K656"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-07-06)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$656</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$663</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K656"/>
+  <dimension ref="A1:K663"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -31307,8 +31307,337 @@
         <v>36323857</v>
       </c>
     </row>
+    <row r="657">
+      <c r="A657" s="2" t="n">
+        <v>46208</v>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D657" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F657" t="n">
+        <v>6</v>
+      </c>
+      <c r="G657" t="n">
+        <v>36</v>
+      </c>
+      <c r="H657" t="inlineStr">
+        <is>
+          <t>6/36</t>
+        </is>
+      </c>
+      <c r="I657" s="4" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="J657" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K657" t="n">
+        <v>37240282</v>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" s="2" t="n">
+        <v>46208</v>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F658" t="n">
+        <v>19</v>
+      </c>
+      <c r="G658" t="n">
+        <v>33</v>
+      </c>
+      <c r="H658" t="inlineStr">
+        <is>
+          <t>19/33</t>
+        </is>
+      </c>
+      <c r="I658" s="5" t="n">
+        <v>57.6</v>
+      </c>
+      <c r="J658" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K658" t="n">
+        <v>36336028</v>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" s="2" t="n">
+        <v>46208</v>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F659" t="n">
+        <v>12</v>
+      </c>
+      <c r="G659" t="n">
+        <v>28</v>
+      </c>
+      <c r="H659" t="inlineStr">
+        <is>
+          <t>12/28</t>
+        </is>
+      </c>
+      <c r="I659" s="4" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="J659" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K659" t="n">
+        <v>37240425</v>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" s="2" t="n">
+        <v>46208</v>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D660" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E660" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F660" t="n">
+        <v>17</v>
+      </c>
+      <c r="G660" t="n">
+        <v>28</v>
+      </c>
+      <c r="H660" t="inlineStr">
+        <is>
+          <t>17/28</t>
+        </is>
+      </c>
+      <c r="I660" s="5" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="J660" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K660" t="n">
+        <v>36892142</v>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" s="2" t="n">
+        <v>46208</v>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="D661" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E661" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F661" t="n">
+        <v>17</v>
+      </c>
+      <c r="G661" t="n">
+        <v>33</v>
+      </c>
+      <c r="H661" t="inlineStr">
+        <is>
+          <t>17/33</t>
+        </is>
+      </c>
+      <c r="I661" s="5" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="J661" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K661" t="n">
+        <v>36336243</v>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" s="2" t="n">
+        <v>46208</v>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="D662" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F662" t="n">
+        <v>28</v>
+      </c>
+      <c r="G662" t="n">
+        <v>33</v>
+      </c>
+      <c r="H662" t="inlineStr">
+        <is>
+          <t>28/33</t>
+        </is>
+      </c>
+      <c r="I662" s="5" t="n">
+        <v>84.8</v>
+      </c>
+      <c r="J662" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K662" t="n">
+        <v>36692755</v>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" s="2" t="n">
+        <v>46208</v>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F663" t="n">
+        <v>9</v>
+      </c>
+      <c r="G663" t="n">
+        <v>36</v>
+      </c>
+      <c r="H663" t="inlineStr">
+        <is>
+          <t>9/36</t>
+        </is>
+      </c>
+      <c r="I663" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="J663" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K663" t="n">
+        <v>36892097</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K656"/>
+  <autoFilter ref="A1:K663"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-07-07)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$663</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$669</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K663"/>
+  <dimension ref="A1:K669"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -31636,8 +31636,290 @@
         <v>36892097</v>
       </c>
     </row>
+    <row r="664">
+      <c r="A664" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D664" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F664" t="n">
+        <v>7</v>
+      </c>
+      <c r="G664" t="n">
+        <v>28</v>
+      </c>
+      <c r="H664" t="inlineStr">
+        <is>
+          <t>7/28</t>
+        </is>
+      </c>
+      <c r="I664" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="J664" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K664" t="n">
+        <v>36390329</v>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F665" t="n">
+        <v>8</v>
+      </c>
+      <c r="G665" t="n">
+        <v>18</v>
+      </c>
+      <c r="H665" t="inlineStr">
+        <is>
+          <t>8/18</t>
+        </is>
+      </c>
+      <c r="I665" s="4" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="J665" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K665" t="n">
+        <v>38531908</v>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F666" t="n">
+        <v>4</v>
+      </c>
+      <c r="G666" t="n">
+        <v>18</v>
+      </c>
+      <c r="H666" t="inlineStr">
+        <is>
+          <t>4/18</t>
+        </is>
+      </c>
+      <c r="I666" s="4" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="J666" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K666" t="n">
+        <v>36928727</v>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F667" t="n">
+        <v>25</v>
+      </c>
+      <c r="G667" t="n">
+        <v>28</v>
+      </c>
+      <c r="H667" t="inlineStr">
+        <is>
+          <t>25/28</t>
+        </is>
+      </c>
+      <c r="I667" s="3" t="n">
+        <v>89.3</v>
+      </c>
+      <c r="J667" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K667" t="n">
+        <v>36280996</v>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F668" t="n">
+        <v>15</v>
+      </c>
+      <c r="G668" t="n">
+        <v>28</v>
+      </c>
+      <c r="H668" t="inlineStr">
+        <is>
+          <t>15/28</t>
+        </is>
+      </c>
+      <c r="I668" s="5" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="J668" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K668" t="n">
+        <v>37873138</v>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F669" t="n">
+        <v>5</v>
+      </c>
+      <c r="G669" t="n">
+        <v>32</v>
+      </c>
+      <c r="H669" t="inlineStr">
+        <is>
+          <t>5/32</t>
+        </is>
+      </c>
+      <c r="I669" s="4" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="J669" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K669" t="n">
+        <v>36929033</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K663"/>
+  <autoFilter ref="A1:K669"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-07-08)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$669</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$675</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K669"/>
+  <dimension ref="A1:K675"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -31918,8 +31918,290 @@
         <v>36929033</v>
       </c>
     </row>
+    <row r="670">
+      <c r="A670" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F670" t="n">
+        <v>11</v>
+      </c>
+      <c r="G670" t="n">
+        <v>28</v>
+      </c>
+      <c r="H670" t="inlineStr">
+        <is>
+          <t>11/28</t>
+        </is>
+      </c>
+      <c r="I670" s="4" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="J670" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K670" t="n">
+        <v>36321360</v>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F671" t="n">
+        <v>6</v>
+      </c>
+      <c r="G671" t="n">
+        <v>18</v>
+      </c>
+      <c r="H671" t="inlineStr">
+        <is>
+          <t>6/18</t>
+        </is>
+      </c>
+      <c r="I671" s="4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J671" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K671" t="n">
+        <v>36929159</v>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F672" t="n">
+        <v>9</v>
+      </c>
+      <c r="G672" t="n">
+        <v>18</v>
+      </c>
+      <c r="H672" t="inlineStr">
+        <is>
+          <t>9/18</t>
+        </is>
+      </c>
+      <c r="I672" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J672" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K672" t="n">
+        <v>36298239</v>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr">
+        <is>
+          <t>Faustine CHOPIN</t>
+        </is>
+      </c>
+      <c r="F673" t="n">
+        <v>14</v>
+      </c>
+      <c r="G673" t="n">
+        <v>28</v>
+      </c>
+      <c r="H673" t="inlineStr">
+        <is>
+          <t>14/28</t>
+        </is>
+      </c>
+      <c r="I673" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J673" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K673" t="n">
+        <v>36297684</v>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="D674" t="inlineStr">
+        <is>
+          <t>RE-LAX  (English version)</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F674" t="n">
+        <v>11</v>
+      </c>
+      <c r="G674" t="n">
+        <v>28</v>
+      </c>
+      <c r="H674" t="inlineStr">
+        <is>
+          <t>11/28</t>
+        </is>
+      </c>
+      <c r="I674" s="4" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="J674" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K674" t="n">
+        <v>36298046</v>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" s="2" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D675" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F675" t="n">
+        <v>13</v>
+      </c>
+      <c r="G675" t="n">
+        <v>32</v>
+      </c>
+      <c r="H675" t="inlineStr">
+        <is>
+          <t>13/32</t>
+        </is>
+      </c>
+      <c r="I675" s="4" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="J675" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K675" t="n">
+        <v>38946656</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K669"/>
+  <autoFilter ref="A1:K675"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-07-09)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$675</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$680</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K675"/>
+  <dimension ref="A1:K680"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -32200,8 +32200,243 @@
         <v>38946656</v>
       </c>
     </row>
+    <row r="676">
+      <c r="A676" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>alice dunoyer</t>
+        </is>
+      </c>
+      <c r="F676" t="n">
+        <v>19</v>
+      </c>
+      <c r="G676" t="n">
+        <v>33</v>
+      </c>
+      <c r="H676" t="inlineStr">
+        <is>
+          <t>19/33</t>
+        </is>
+      </c>
+      <c r="I676" s="5" t="n">
+        <v>57.6</v>
+      </c>
+      <c r="J676" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K676" t="n">
+        <v>36321409</v>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F677" t="n">
+        <v>2</v>
+      </c>
+      <c r="G677" t="n">
+        <v>18</v>
+      </c>
+      <c r="H677" t="inlineStr">
+        <is>
+          <t>2/18</t>
+        </is>
+      </c>
+      <c r="I677" s="4" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="J677" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K677" t="n">
+        <v>36929291</v>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F678" t="n">
+        <v>10</v>
+      </c>
+      <c r="G678" t="n">
+        <v>18</v>
+      </c>
+      <c r="H678" t="inlineStr">
+        <is>
+          <t>10/18</t>
+        </is>
+      </c>
+      <c r="I678" s="5" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="J678" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K678" t="n">
+        <v>36298340</v>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr">
+        <is>
+          <t>Pauline Ramon</t>
+        </is>
+      </c>
+      <c r="F679" t="n">
+        <v>16</v>
+      </c>
+      <c r="G679" t="n">
+        <v>33</v>
+      </c>
+      <c r="H679" t="inlineStr">
+        <is>
+          <t>16/33</t>
+        </is>
+      </c>
+      <c r="I679" s="4" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="J679" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K679" t="n">
+        <v>36298381</v>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F680" t="n">
+        <v>16</v>
+      </c>
+      <c r="G680" t="n">
+        <v>33</v>
+      </c>
+      <c r="H680" t="inlineStr">
+        <is>
+          <t>16/33</t>
+        </is>
+      </c>
+      <c r="I680" s="4" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="J680" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K680" t="n">
+        <v>36298578</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K675"/>
+  <autoFilter ref="A1:K680"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-07-10)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$680</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$685</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K680"/>
+  <dimension ref="A1:K685"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -590,7 +590,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>alice dunoyer</t>
+          <t>Alice Dunoyer</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -1201,7 +1201,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>alice dunoyer</t>
+          <t>Alice Dunoyer</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -2752,7 +2752,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>alice dunoyer</t>
+          <t>Alice Dunoyer</t>
         </is>
       </c>
       <c r="F49" t="n">
@@ -3128,7 +3128,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>alice dunoyer</t>
+          <t>Alice Dunoyer</t>
         </is>
       </c>
       <c r="F57" t="n">
@@ -3269,7 +3269,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>alice dunoyer</t>
+          <t>Alice Dunoyer</t>
         </is>
       </c>
       <c r="F60" t="n">
@@ -3739,7 +3739,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>alice dunoyer</t>
+          <t>Alice Dunoyer</t>
         </is>
       </c>
       <c r="F70" t="n">
@@ -4585,7 +4585,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>alice dunoyer</t>
+          <t>Alice Dunoyer</t>
         </is>
       </c>
       <c r="F88" t="n">
@@ -5713,7 +5713,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>alice dunoyer</t>
+          <t>Alice Dunoyer</t>
         </is>
       </c>
       <c r="F112" t="n">
@@ -10084,7 +10084,7 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>alice dunoyer</t>
+          <t>Alice Dunoyer</t>
         </is>
       </c>
       <c r="F205" t="n">
@@ -10695,7 +10695,7 @@
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>alice dunoyer</t>
+          <t>Alice Dunoyer</t>
         </is>
       </c>
       <c r="F218" t="n">
@@ -11024,7 +11024,7 @@
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>alice dunoyer</t>
+          <t>Alice Dunoyer</t>
         </is>
       </c>
       <c r="F225" t="n">
@@ -12340,7 +12340,7 @@
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t>alice dunoyer</t>
+          <t>Alice Dunoyer</t>
         </is>
       </c>
       <c r="F253" t="n">
@@ -13374,7 +13374,7 @@
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>alice dunoyer</t>
+          <t>Alice Dunoyer</t>
         </is>
       </c>
       <c r="F275" t="n">
@@ -15771,7 +15771,7 @@
       </c>
       <c r="E326" t="inlineStr">
         <is>
-          <t>alice dunoyer</t>
+          <t>Alice Dunoyer</t>
         </is>
       </c>
       <c r="F326" t="n">
@@ -17040,7 +17040,7 @@
       </c>
       <c r="E353" t="inlineStr">
         <is>
-          <t>alice dunoyer</t>
+          <t>Alice Dunoyer</t>
         </is>
       </c>
       <c r="F353" t="n">
@@ -20283,7 +20283,7 @@
       </c>
       <c r="E422" t="inlineStr">
         <is>
-          <t>alice dunoyer</t>
+          <t>Alice Dunoyer</t>
         </is>
       </c>
       <c r="F422" t="n">
@@ -21317,7 +21317,7 @@
       </c>
       <c r="E444" t="inlineStr">
         <is>
-          <t>alice dunoyer</t>
+          <t>Alice Dunoyer</t>
         </is>
       </c>
       <c r="F444" t="n">
@@ -23573,7 +23573,7 @@
       </c>
       <c r="E492" t="inlineStr">
         <is>
-          <t>alice dunoyer</t>
+          <t>Alice Dunoyer</t>
         </is>
       </c>
       <c r="F492" t="n">
@@ -24607,7 +24607,7 @@
       </c>
       <c r="E514" t="inlineStr">
         <is>
-          <t>alice dunoyer</t>
+          <t>Alice Dunoyer</t>
         </is>
       </c>
       <c r="F514" t="n">
@@ -25688,7 +25688,7 @@
       </c>
       <c r="E537" t="inlineStr">
         <is>
-          <t>alice dunoyer</t>
+          <t>Alice Dunoyer</t>
         </is>
       </c>
       <c r="F537" t="n">
@@ -26722,7 +26722,7 @@
       </c>
       <c r="E559" t="inlineStr">
         <is>
-          <t>alice dunoyer</t>
+          <t>Alice Dunoyer</t>
         </is>
       </c>
       <c r="F559" t="n">
@@ -27944,7 +27944,7 @@
       </c>
       <c r="E585" t="inlineStr">
         <is>
-          <t>alice dunoyer</t>
+          <t>Alice Dunoyer</t>
         </is>
       </c>
       <c r="F585" t="n">
@@ -29918,7 +29918,7 @@
       </c>
       <c r="E627" t="inlineStr">
         <is>
-          <t>alice dunoyer</t>
+          <t>Alice Dunoyer</t>
         </is>
       </c>
       <c r="F627" t="n">
@@ -30999,7 +30999,7 @@
       </c>
       <c r="E650" t="inlineStr">
         <is>
-          <t>alice dunoyer</t>
+          <t>Alice Dunoyer</t>
         </is>
       </c>
       <c r="F650" t="n">
@@ -32221,7 +32221,7 @@
       </c>
       <c r="E676" t="inlineStr">
         <is>
-          <t>alice dunoyer</t>
+          <t>Alice Dunoyer</t>
         </is>
       </c>
       <c r="F676" t="n">
@@ -32435,8 +32435,243 @@
         <v>36298578</v>
       </c>
     </row>
+    <row r="681">
+      <c r="A681" s="2" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F681" t="n">
+        <v>15</v>
+      </c>
+      <c r="G681" t="n">
+        <v>33</v>
+      </c>
+      <c r="H681" t="inlineStr">
+        <is>
+          <t>15/33</t>
+        </is>
+      </c>
+      <c r="I681" s="4" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="J681" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K681" t="n">
+        <v>36321560</v>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" s="2" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F682" t="n">
+        <v>9</v>
+      </c>
+      <c r="G682" t="n">
+        <v>18</v>
+      </c>
+      <c r="H682" t="inlineStr">
+        <is>
+          <t>9/18</t>
+        </is>
+      </c>
+      <c r="I682" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J682" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K682" t="n">
+        <v>36929382</v>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" s="2" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F683" t="n">
+        <v>4</v>
+      </c>
+      <c r="G683" t="n">
+        <v>18</v>
+      </c>
+      <c r="H683" t="inlineStr">
+        <is>
+          <t>4/18</t>
+        </is>
+      </c>
+      <c r="I683" s="4" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="J683" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K683" t="n">
+        <v>36298755</v>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" s="2" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D684" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>Faustine CHOPIN</t>
+        </is>
+      </c>
+      <c r="F684" t="n">
+        <v>20</v>
+      </c>
+      <c r="G684" t="n">
+        <v>33</v>
+      </c>
+      <c r="H684" t="inlineStr">
+        <is>
+          <t>20/33</t>
+        </is>
+      </c>
+      <c r="I684" s="5" t="n">
+        <v>60.6</v>
+      </c>
+      <c r="J684" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K684" t="n">
+        <v>36298809</v>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" s="2" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D685" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F685" t="n">
+        <v>18</v>
+      </c>
+      <c r="G685" t="n">
+        <v>33</v>
+      </c>
+      <c r="H685" t="inlineStr">
+        <is>
+          <t>18/33</t>
+        </is>
+      </c>
+      <c r="I685" s="5" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="J685" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K685" t="n">
+        <v>36298862</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K680"/>
+  <autoFilter ref="A1:K685"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-07-11)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$685</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$690</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K685"/>
+  <dimension ref="A1:K690"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -32670,8 +32670,243 @@
         <v>36298862</v>
       </c>
     </row>
+    <row r="686">
+      <c r="A686" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D686" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E686" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F686" t="n">
+        <v>6</v>
+      </c>
+      <c r="G686" t="n">
+        <v>33</v>
+      </c>
+      <c r="H686" t="inlineStr">
+        <is>
+          <t>6/33</t>
+        </is>
+      </c>
+      <c r="I686" s="4" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="J686" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K686" t="n">
+        <v>36319498</v>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D687" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F687" t="n">
+        <v>8</v>
+      </c>
+      <c r="G687" t="n">
+        <v>16</v>
+      </c>
+      <c r="H687" t="inlineStr">
+        <is>
+          <t>8/16</t>
+        </is>
+      </c>
+      <c r="I687" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J687" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K687" t="n">
+        <v>36320055</v>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D688" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F688" t="n">
+        <v>5</v>
+      </c>
+      <c r="G688" t="n">
+        <v>32</v>
+      </c>
+      <c r="H688" t="inlineStr">
+        <is>
+          <t>5/32</t>
+        </is>
+      </c>
+      <c r="I688" s="4" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="J688" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K688" t="n">
+        <v>36320779</v>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D689" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E689" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F689" t="n">
+        <v>23</v>
+      </c>
+      <c r="G689" t="n">
+        <v>33</v>
+      </c>
+      <c r="H689" t="inlineStr">
+        <is>
+          <t>23/33</t>
+        </is>
+      </c>
+      <c r="I689" s="5" t="n">
+        <v>69.7</v>
+      </c>
+      <c r="J689" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K689" t="n">
+        <v>36320889</v>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D690" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E690" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F690" t="n">
+        <v>22</v>
+      </c>
+      <c r="G690" t="n">
+        <v>20</v>
+      </c>
+      <c r="H690" t="inlineStr">
+        <is>
+          <t>22/20</t>
+        </is>
+      </c>
+      <c r="I690" s="3" t="n">
+        <v>110</v>
+      </c>
+      <c r="J690" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K690" t="n">
+        <v>36893826</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K685"/>
+  <autoFilter ref="A1:K690"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-07-12)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$690</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$696</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K690"/>
+  <dimension ref="A1:K696"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10981,18 +10981,18 @@
         </is>
       </c>
       <c r="F224" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G224" t="n">
         <v>32</v>
       </c>
       <c r="H224" t="inlineStr">
         <is>
-          <t>20/32</t>
+          <t>18/32</t>
         </is>
       </c>
       <c r="I224" s="5" t="n">
-        <v>62.5</v>
+        <v>56.2</v>
       </c>
       <c r="J224" t="inlineStr">
         <is>
@@ -12579,18 +12579,18 @@
         </is>
       </c>
       <c r="F258" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G258" t="n">
         <v>13</v>
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>4/13</t>
+          <t>3/13</t>
         </is>
       </c>
       <c r="I258" s="4" t="n">
-        <v>30.8</v>
+        <v>23.1</v>
       </c>
       <c r="J258" t="inlineStr">
         <is>
@@ -21603,18 +21603,18 @@
         </is>
       </c>
       <c r="F450" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G450" t="n">
         <v>13</v>
       </c>
       <c r="H450" t="inlineStr">
         <is>
-          <t>2/13</t>
+          <t>1/13</t>
         </is>
       </c>
       <c r="I450" s="4" t="n">
-        <v>15.4</v>
+        <v>7.7</v>
       </c>
       <c r="J450" t="inlineStr">
         <is>
@@ -22684,18 +22684,18 @@
         </is>
       </c>
       <c r="F473" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G473" t="n">
         <v>36</v>
       </c>
       <c r="H473" t="inlineStr">
         <is>
-          <t>7/36</t>
+          <t>6/36</t>
         </is>
       </c>
       <c r="I473" s="4" t="n">
-        <v>19.4</v>
+        <v>16.7</v>
       </c>
       <c r="J473" t="inlineStr">
         <is>
@@ -32905,8 +32905,290 @@
         <v>36893826</v>
       </c>
     </row>
+    <row r="691">
+      <c r="A691" s="2" t="n">
+        <v>46214</v>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D691" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F691" t="n">
+        <v>8</v>
+      </c>
+      <c r="G691" t="n">
+        <v>32</v>
+      </c>
+      <c r="H691" t="inlineStr">
+        <is>
+          <t>8/32</t>
+        </is>
+      </c>
+      <c r="I691" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="J691" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K691" t="n">
+        <v>36323273</v>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" s="2" t="n">
+        <v>46214</v>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D692" t="inlineStr">
+        <is>
+          <t>RE-BOOST  (English version)</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr">
+        <is>
+          <t>Alice Dunoyer</t>
+        </is>
+      </c>
+      <c r="F692" t="n">
+        <v>12</v>
+      </c>
+      <c r="G692" t="n">
+        <v>33</v>
+      </c>
+      <c r="H692" t="inlineStr">
+        <is>
+          <t>12/33</t>
+        </is>
+      </c>
+      <c r="I692" s="4" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="J692" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K692" t="n">
+        <v>36323119</v>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" s="2" t="n">
+        <v>46214</v>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D693" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F693" t="n">
+        <v>9</v>
+      </c>
+      <c r="G693" t="n">
+        <v>32</v>
+      </c>
+      <c r="H693" t="inlineStr">
+        <is>
+          <t>9/32</t>
+        </is>
+      </c>
+      <c r="I693" s="4" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="J693" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K693" t="n">
+        <v>38771771</v>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" s="2" t="n">
+        <v>46214</v>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D694" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E694" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F694" t="n">
+        <v>10</v>
+      </c>
+      <c r="G694" t="n">
+        <v>33</v>
+      </c>
+      <c r="H694" t="inlineStr">
+        <is>
+          <t>10/33</t>
+        </is>
+      </c>
+      <c r="I694" s="4" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="J694" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K694" t="n">
+        <v>36329201</v>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" s="2" t="n">
+        <v>46214</v>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="D695" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F695" t="n">
+        <v>37</v>
+      </c>
+      <c r="G695" t="n">
+        <v>32</v>
+      </c>
+      <c r="H695" t="inlineStr">
+        <is>
+          <t>37/32</t>
+        </is>
+      </c>
+      <c r="I695" s="3" t="n">
+        <v>115.6</v>
+      </c>
+      <c r="J695" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K695" t="n">
+        <v>38771871</v>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" s="2" t="n">
+        <v>46214</v>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D696" t="inlineStr">
+        <is>
+          <t>RE-LAX  (English version)</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>Sigga Daregard</t>
+        </is>
+      </c>
+      <c r="F696" t="n">
+        <v>28</v>
+      </c>
+      <c r="G696" t="n">
+        <v>28</v>
+      </c>
+      <c r="H696" t="inlineStr">
+        <is>
+          <t>28/28</t>
+        </is>
+      </c>
+      <c r="I696" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J696" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K696" t="n">
+        <v>36329966</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K690"/>
+  <autoFilter ref="A1:K696"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-07-13)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$696</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$702</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K696"/>
+  <dimension ref="A1:K702"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -33187,8 +33187,290 @@
         <v>36329966</v>
       </c>
     </row>
+    <row r="697">
+      <c r="A697" s="2" t="n">
+        <v>46215</v>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D697" t="inlineStr">
+        <is>
+          <t>RE-LAX  (English version)</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>Sigga Daregard</t>
+        </is>
+      </c>
+      <c r="F697" t="n">
+        <v>23</v>
+      </c>
+      <c r="G697" t="n">
+        <v>28</v>
+      </c>
+      <c r="H697" t="inlineStr">
+        <is>
+          <t>23/28</t>
+        </is>
+      </c>
+      <c r="I697" s="5" t="n">
+        <v>82.09999999999999</v>
+      </c>
+      <c r="J697" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K697" t="n">
+        <v>36336029</v>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" s="2" t="n">
+        <v>46215</v>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D698" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F698" t="n">
+        <v>10</v>
+      </c>
+      <c r="G698" t="n">
+        <v>28</v>
+      </c>
+      <c r="H698" t="inlineStr">
+        <is>
+          <t>10/28</t>
+        </is>
+      </c>
+      <c r="I698" s="4" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="J698" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K698" t="n">
+        <v>37240426</v>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" s="2" t="n">
+        <v>46215</v>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D699" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E699" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F699" t="n">
+        <v>20</v>
+      </c>
+      <c r="G699" t="n">
+        <v>28</v>
+      </c>
+      <c r="H699" t="inlineStr">
+        <is>
+          <t>20/28</t>
+        </is>
+      </c>
+      <c r="I699" s="5" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="J699" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K699" t="n">
+        <v>36892143</v>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" s="2" t="n">
+        <v>46215</v>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="D700" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E700" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F700" t="n">
+        <v>23</v>
+      </c>
+      <c r="G700" t="n">
+        <v>33</v>
+      </c>
+      <c r="H700" t="inlineStr">
+        <is>
+          <t>23/33</t>
+        </is>
+      </c>
+      <c r="I700" s="5" t="n">
+        <v>69.7</v>
+      </c>
+      <c r="J700" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K700" t="n">
+        <v>36336244</v>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" s="2" t="n">
+        <v>46215</v>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="D701" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E701" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F701" t="n">
+        <v>24</v>
+      </c>
+      <c r="G701" t="n">
+        <v>32</v>
+      </c>
+      <c r="H701" t="inlineStr">
+        <is>
+          <t>24/32</t>
+        </is>
+      </c>
+      <c r="I701" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="J701" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K701" t="n">
+        <v>36692756</v>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" s="2" t="n">
+        <v>46215</v>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="D702" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E702" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F702" t="n">
+        <v>13</v>
+      </c>
+      <c r="G702" t="n">
+        <v>36</v>
+      </c>
+      <c r="H702" t="inlineStr">
+        <is>
+          <t>13/36</t>
+        </is>
+      </c>
+      <c r="I702" s="4" t="n">
+        <v>36.1</v>
+      </c>
+      <c r="J702" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K702" t="n">
+        <v>36892098</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K696"/>
+  <autoFilter ref="A1:K702"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-07-14)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$702</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$708</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K702"/>
+  <dimension ref="A1:K708"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -33469,8 +33469,290 @@
         <v>36892098</v>
       </c>
     </row>
+    <row r="703">
+      <c r="A703" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D703" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr">
+        <is>
+          <t>Alice Dunoyer</t>
+        </is>
+      </c>
+      <c r="F703" t="n">
+        <v>16</v>
+      </c>
+      <c r="G703" t="n">
+        <v>28</v>
+      </c>
+      <c r="H703" t="inlineStr">
+        <is>
+          <t>16/28</t>
+        </is>
+      </c>
+      <c r="I703" s="5" t="n">
+        <v>57.1</v>
+      </c>
+      <c r="J703" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K703" t="n">
+        <v>36390330</v>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D704" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E704" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F704" t="n">
+        <v>7</v>
+      </c>
+      <c r="G704" t="n">
+        <v>18</v>
+      </c>
+      <c r="H704" t="inlineStr">
+        <is>
+          <t>7/18</t>
+        </is>
+      </c>
+      <c r="I704" s="4" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="J704" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K704" t="n">
+        <v>38531909</v>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D705" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E705" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F705" t="n">
+        <v>12</v>
+      </c>
+      <c r="G705" t="n">
+        <v>18</v>
+      </c>
+      <c r="H705" t="inlineStr">
+        <is>
+          <t>12/18</t>
+        </is>
+      </c>
+      <c r="I705" s="5" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J705" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K705" t="n">
+        <v>36928728</v>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D706" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E706" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F706" t="n">
+        <v>5</v>
+      </c>
+      <c r="G706" t="n">
+        <v>28</v>
+      </c>
+      <c r="H706" t="inlineStr">
+        <is>
+          <t>5/28</t>
+        </is>
+      </c>
+      <c r="I706" s="4" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="J706" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K706" t="n">
+        <v>36280997</v>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="D707" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F707" t="n">
+        <v>6</v>
+      </c>
+      <c r="G707" t="n">
+        <v>28</v>
+      </c>
+      <c r="H707" t="inlineStr">
+        <is>
+          <t>6/28</t>
+        </is>
+      </c>
+      <c r="I707" s="4" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="J707" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K707" t="n">
+        <v>37873139</v>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D708" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E708" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F708" t="n">
+        <v>13</v>
+      </c>
+      <c r="G708" t="n">
+        <v>32</v>
+      </c>
+      <c r="H708" t="inlineStr">
+        <is>
+          <t>13/32</t>
+        </is>
+      </c>
+      <c r="I708" s="4" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="J708" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K708" t="n">
+        <v>36929034</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K702"/>
+  <autoFilter ref="A1:K708"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-07-15)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$708</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$713</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K708"/>
+  <dimension ref="A1:K713"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -33673,12 +33673,12 @@
       </c>
       <c r="D707" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Quiet Free-Flow</t>
         </is>
       </c>
       <c r="E707" t="inlineStr">
         <is>
-          <t>Leonore Chapin</t>
+          <t>Free Flow</t>
         </is>
       </c>
       <c r="F707" t="n">
@@ -33751,8 +33751,243 @@
         <v>36929034</v>
       </c>
     </row>
+    <row r="709">
+      <c r="A709" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="D709" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E709" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F709" t="n">
+        <v>9</v>
+      </c>
+      <c r="G709" t="n">
+        <v>33</v>
+      </c>
+      <c r="H709" t="inlineStr">
+        <is>
+          <t>9/33</t>
+        </is>
+      </c>
+      <c r="I709" s="4" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="J709" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K709" t="n">
+        <v>36321361</v>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D710" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E710" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F710" t="n">
+        <v>14</v>
+      </c>
+      <c r="G710" t="n">
+        <v>32</v>
+      </c>
+      <c r="H710" t="inlineStr">
+        <is>
+          <t>14/32</t>
+        </is>
+      </c>
+      <c r="I710" s="4" t="n">
+        <v>43.8</v>
+      </c>
+      <c r="J710" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K710" t="n">
+        <v>36298240</v>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="D711" t="inlineStr">
+        <is>
+          <t>RE-LAX  (English version)</t>
+        </is>
+      </c>
+      <c r="E711" t="inlineStr">
+        <is>
+          <t>Sigga Daregard</t>
+        </is>
+      </c>
+      <c r="F711" t="n">
+        <v>7</v>
+      </c>
+      <c r="G711" t="n">
+        <v>33</v>
+      </c>
+      <c r="H711" t="inlineStr">
+        <is>
+          <t>7/33</t>
+        </is>
+      </c>
+      <c r="I711" s="4" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="J711" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K711" t="n">
+        <v>36298047</v>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D712" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E712" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F712" t="n">
+        <v>34</v>
+      </c>
+      <c r="G712" t="n">
+        <v>32</v>
+      </c>
+      <c r="H712" t="inlineStr">
+        <is>
+          <t>34/32</t>
+        </is>
+      </c>
+      <c r="I712" s="3" t="n">
+        <v>106.2</v>
+      </c>
+      <c r="J712" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K712" t="n">
+        <v>36929160</v>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="D713" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E713" t="inlineStr">
+        <is>
+          <t>Faustine CHOPIN</t>
+        </is>
+      </c>
+      <c r="F713" t="n">
+        <v>33</v>
+      </c>
+      <c r="G713" t="n">
+        <v>33</v>
+      </c>
+      <c r="H713" t="inlineStr">
+        <is>
+          <t>33/33</t>
+        </is>
+      </c>
+      <c r="I713" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J713" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K713" t="n">
+        <v>36297685</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K708"/>
+  <autoFilter ref="A1:K713"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-07-16)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$713</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$718</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K713"/>
+  <dimension ref="A1:K718"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -33986,8 +33986,243 @@
         <v>36297685</v>
       </c>
     </row>
+    <row r="714">
+      <c r="A714" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D714" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E714" t="inlineStr">
+        <is>
+          <t>Alice Dunoyer</t>
+        </is>
+      </c>
+      <c r="F714" t="n">
+        <v>8</v>
+      </c>
+      <c r="G714" t="n">
+        <v>33</v>
+      </c>
+      <c r="H714" t="inlineStr">
+        <is>
+          <t>8/33</t>
+        </is>
+      </c>
+      <c r="I714" s="4" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="J714" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K714" t="n">
+        <v>36321410</v>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D715" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E715" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F715" t="n">
+        <v>9</v>
+      </c>
+      <c r="G715" t="n">
+        <v>18</v>
+      </c>
+      <c r="H715" t="inlineStr">
+        <is>
+          <t>9/18</t>
+        </is>
+      </c>
+      <c r="I715" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J715" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K715" t="n">
+        <v>36929292</v>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D716" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E716" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F716" t="n">
+        <v>7</v>
+      </c>
+      <c r="G716" t="n">
+        <v>18</v>
+      </c>
+      <c r="H716" t="inlineStr">
+        <is>
+          <t>7/18</t>
+        </is>
+      </c>
+      <c r="I716" s="4" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="J716" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K716" t="n">
+        <v>36298341</v>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D717" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E717" t="inlineStr">
+        <is>
+          <t>Pauline Ramon</t>
+        </is>
+      </c>
+      <c r="F717" t="n">
+        <v>25</v>
+      </c>
+      <c r="G717" t="n">
+        <v>28</v>
+      </c>
+      <c r="H717" t="inlineStr">
+        <is>
+          <t>25/28</t>
+        </is>
+      </c>
+      <c r="I717" s="3" t="n">
+        <v>89.3</v>
+      </c>
+      <c r="J717" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K717" t="n">
+        <v>36298382</v>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D718" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E718" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F718" t="n">
+        <v>20</v>
+      </c>
+      <c r="G718" t="n">
+        <v>33</v>
+      </c>
+      <c r="H718" t="inlineStr">
+        <is>
+          <t>20/33</t>
+        </is>
+      </c>
+      <c r="I718" s="5" t="n">
+        <v>60.6</v>
+      </c>
+      <c r="J718" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K718" t="n">
+        <v>36298579</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K713"/>
+  <autoFilter ref="A1:K718"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-07-17)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$718</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$727</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K718"/>
+  <dimension ref="A1:K727"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -34221,8 +34221,431 @@
         <v>36298579</v>
       </c>
     </row>
+    <row r="719">
+      <c r="A719" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>07:45</t>
+        </is>
+      </c>
+      <c r="D719" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E719" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F719" t="n">
+        <v>4</v>
+      </c>
+      <c r="G719" t="n">
+        <v>28</v>
+      </c>
+      <c r="H719" t="inlineStr">
+        <is>
+          <t>4/28</t>
+        </is>
+      </c>
+      <c r="I719" s="4" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="J719" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K719" t="n">
+        <v>37090006</v>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D720" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E720" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F720" t="n">
+        <v>3</v>
+      </c>
+      <c r="G720" t="n">
+        <v>13</v>
+      </c>
+      <c r="H720" t="inlineStr">
+        <is>
+          <t>3/13</t>
+        </is>
+      </c>
+      <c r="I720" s="4" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="J720" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K720" t="n">
+        <v>37230114</v>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="D721" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E721" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F721" t="n">
+        <v>1</v>
+      </c>
+      <c r="G721" t="n">
+        <v>13</v>
+      </c>
+      <c r="H721" t="inlineStr">
+        <is>
+          <t>1/13</t>
+        </is>
+      </c>
+      <c r="I721" s="4" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="J721" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K721" t="n">
+        <v>37230150</v>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D722" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E722" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F722" t="n">
+        <v>4</v>
+      </c>
+      <c r="G722" t="n">
+        <v>13</v>
+      </c>
+      <c r="H722" t="inlineStr">
+        <is>
+          <t>4/13</t>
+        </is>
+      </c>
+      <c r="I722" s="4" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="J722" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K722" t="n">
+        <v>37090964</v>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D723" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E723" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F723" t="n">
+        <v>6</v>
+      </c>
+      <c r="G723" t="n">
+        <v>33</v>
+      </c>
+      <c r="H723" t="inlineStr">
+        <is>
+          <t>6/33</t>
+        </is>
+      </c>
+      <c r="I723" s="4" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="J723" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K723" t="n">
+        <v>36321561</v>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D724" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E724" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F724" t="n">
+        <v>9</v>
+      </c>
+      <c r="G724" t="n">
+        <v>18</v>
+      </c>
+      <c r="H724" t="inlineStr">
+        <is>
+          <t>9/18</t>
+        </is>
+      </c>
+      <c r="I724" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J724" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K724" t="n">
+        <v>36929383</v>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C725" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D725" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E725" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F725" t="n">
+        <v>9</v>
+      </c>
+      <c r="G725" t="n">
+        <v>18</v>
+      </c>
+      <c r="H725" t="inlineStr">
+        <is>
+          <t>9/18</t>
+        </is>
+      </c>
+      <c r="I725" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J725" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K725" t="n">
+        <v>36298756</v>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D726" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E726" t="inlineStr">
+        <is>
+          <t>Faustine CHOPIN</t>
+        </is>
+      </c>
+      <c r="F726" t="n">
+        <v>18</v>
+      </c>
+      <c r="G726" t="n">
+        <v>33</v>
+      </c>
+      <c r="H726" t="inlineStr">
+        <is>
+          <t>18/33</t>
+        </is>
+      </c>
+      <c r="I726" s="5" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="J726" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K726" t="n">
+        <v>36298810</v>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D727" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E727" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F727" t="n">
+        <v>22</v>
+      </c>
+      <c r="G727" t="n">
+        <v>33</v>
+      </c>
+      <c r="H727" t="inlineStr">
+        <is>
+          <t>22/33</t>
+        </is>
+      </c>
+      <c r="I727" s="5" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J727" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K727" t="n">
+        <v>36298863</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K718"/>
+  <autoFilter ref="A1:K727"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-07-18)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$727</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$734</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K727"/>
+  <dimension ref="A1:K734"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -34644,8 +34644,337 @@
         <v>36298863</v>
       </c>
     </row>
+    <row r="728">
+      <c r="A728" s="2" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D728" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E728" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F728" t="n">
+        <v>11</v>
+      </c>
+      <c r="G728" t="n">
+        <v>32</v>
+      </c>
+      <c r="H728" t="inlineStr">
+        <is>
+          <t>11/32</t>
+        </is>
+      </c>
+      <c r="I728" s="4" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="J728" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K728" t="n">
+        <v>36319499</v>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" s="2" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C729" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D729" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E729" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F729" t="n">
+        <v>1</v>
+      </c>
+      <c r="G729" t="n">
+        <v>16</v>
+      </c>
+      <c r="H729" t="inlineStr">
+        <is>
+          <t>1/16</t>
+        </is>
+      </c>
+      <c r="I729" s="4" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="J729" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K729" t="n">
+        <v>36320657</v>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" s="2" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D730" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E730" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F730" t="n">
+        <v>4</v>
+      </c>
+      <c r="G730" t="n">
+        <v>16</v>
+      </c>
+      <c r="H730" t="inlineStr">
+        <is>
+          <t>4/16</t>
+        </is>
+      </c>
+      <c r="I730" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="J730" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K730" t="n">
+        <v>36320056</v>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" s="2" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D731" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E731" t="inlineStr">
+        <is>
+          <t>Sigga Daregard</t>
+        </is>
+      </c>
+      <c r="F731" t="n">
+        <v>9</v>
+      </c>
+      <c r="G731" t="n">
+        <v>33</v>
+      </c>
+      <c r="H731" t="inlineStr">
+        <is>
+          <t>9/33</t>
+        </is>
+      </c>
+      <c r="I731" s="4" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="J731" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K731" t="n">
+        <v>36320780</v>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" s="2" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D732" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E732" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F732" t="n">
+        <v>16</v>
+      </c>
+      <c r="G732" t="n">
+        <v>33</v>
+      </c>
+      <c r="H732" t="inlineStr">
+        <is>
+          <t>16/33</t>
+        </is>
+      </c>
+      <c r="I732" s="4" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="J732" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K732" t="n">
+        <v>36320890</v>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" s="2" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D733" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E733" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F733" t="n">
+        <v>17</v>
+      </c>
+      <c r="G733" t="n">
+        <v>20</v>
+      </c>
+      <c r="H733" t="inlineStr">
+        <is>
+          <t>17/20</t>
+        </is>
+      </c>
+      <c r="I733" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="J733" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K733" t="n">
+        <v>36893827</v>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" s="2" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D734" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E734" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F734" t="n">
+        <v>9</v>
+      </c>
+      <c r="G734" t="n">
+        <v>20</v>
+      </c>
+      <c r="H734" t="inlineStr">
+        <is>
+          <t>9/20</t>
+        </is>
+      </c>
+      <c r="I734" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="J734" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K734" t="n">
+        <v>36893882</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K727"/>
+  <autoFilter ref="A1:K734"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-07-19)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$734</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$740</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K734"/>
+  <dimension ref="A1:K740"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -34973,8 +34973,290 @@
         <v>36893882</v>
       </c>
     </row>
+    <row r="735">
+      <c r="A735" s="2" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D735" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E735" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F735" t="n">
+        <v>8</v>
+      </c>
+      <c r="G735" t="n">
+        <v>32</v>
+      </c>
+      <c r="H735" t="inlineStr">
+        <is>
+          <t>8/32</t>
+        </is>
+      </c>
+      <c r="I735" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="J735" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K735" t="n">
+        <v>36323274</v>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" s="2" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D736" t="inlineStr">
+        <is>
+          <t>RE-BOOST  (English version)</t>
+        </is>
+      </c>
+      <c r="E736" t="inlineStr">
+        <is>
+          <t>Alice Dunoyer</t>
+        </is>
+      </c>
+      <c r="F736" t="n">
+        <v>8</v>
+      </c>
+      <c r="G736" t="n">
+        <v>33</v>
+      </c>
+      <c r="H736" t="inlineStr">
+        <is>
+          <t>8/33</t>
+        </is>
+      </c>
+      <c r="I736" s="4" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="J736" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K736" t="n">
+        <v>36323120</v>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" s="2" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D737" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E737" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F737" t="n">
+        <v>14</v>
+      </c>
+      <c r="G737" t="n">
+        <v>32</v>
+      </c>
+      <c r="H737" t="inlineStr">
+        <is>
+          <t>14/32</t>
+        </is>
+      </c>
+      <c r="I737" s="4" t="n">
+        <v>43.8</v>
+      </c>
+      <c r="J737" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K737" t="n">
+        <v>38771772</v>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" s="2" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D738" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E738" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F738" t="n">
+        <v>13</v>
+      </c>
+      <c r="G738" t="n">
+        <v>33</v>
+      </c>
+      <c r="H738" t="inlineStr">
+        <is>
+          <t>13/33</t>
+        </is>
+      </c>
+      <c r="I738" s="4" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="J738" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K738" t="n">
+        <v>36329202</v>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" s="2" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="D739" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E739" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F739" t="n">
+        <v>12</v>
+      </c>
+      <c r="G739" t="n">
+        <v>32</v>
+      </c>
+      <c r="H739" t="inlineStr">
+        <is>
+          <t>12/32</t>
+        </is>
+      </c>
+      <c r="I739" s="4" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="J739" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K739" t="n">
+        <v>38771872</v>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" s="2" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D740" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E740" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F740" t="n">
+        <v>13</v>
+      </c>
+      <c r="G740" t="n">
+        <v>33</v>
+      </c>
+      <c r="H740" t="inlineStr">
+        <is>
+          <t>13/33</t>
+        </is>
+      </c>
+      <c r="I740" s="4" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="J740" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K740" t="n">
+        <v>36329967</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K734"/>
+  <autoFilter ref="A1:K740"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-07-20)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$740</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$746</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K740"/>
+  <dimension ref="A1:K746"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -35255,8 +35255,290 @@
         <v>36329967</v>
       </c>
     </row>
+    <row r="741">
+      <c r="A741" s="2" t="n">
+        <v>46222</v>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C741" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D741" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E741" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F741" t="n">
+        <v>13</v>
+      </c>
+      <c r="G741" t="n">
+        <v>36</v>
+      </c>
+      <c r="H741" t="inlineStr">
+        <is>
+          <t>13/36</t>
+        </is>
+      </c>
+      <c r="I741" s="4" t="n">
+        <v>36.1</v>
+      </c>
+      <c r="J741" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K741" t="n">
+        <v>37240284</v>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" s="2" t="n">
+        <v>46222</v>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D742" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E742" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F742" t="n">
+        <v>23</v>
+      </c>
+      <c r="G742" t="n">
+        <v>33</v>
+      </c>
+      <c r="H742" t="inlineStr">
+        <is>
+          <t>23/33</t>
+        </is>
+      </c>
+      <c r="I742" s="5" t="n">
+        <v>69.7</v>
+      </c>
+      <c r="J742" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K742" t="n">
+        <v>36336030</v>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" s="2" t="n">
+        <v>46222</v>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D743" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E743" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F743" t="n">
+        <v>9</v>
+      </c>
+      <c r="G743" t="n">
+        <v>28</v>
+      </c>
+      <c r="H743" t="inlineStr">
+        <is>
+          <t>9/28</t>
+        </is>
+      </c>
+      <c r="I743" s="4" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="J743" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K743" t="n">
+        <v>37240427</v>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" s="2" t="n">
+        <v>46222</v>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="D744" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E744" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F744" t="n">
+        <v>21</v>
+      </c>
+      <c r="G744" t="n">
+        <v>28</v>
+      </c>
+      <c r="H744" t="inlineStr">
+        <is>
+          <t>21/28</t>
+        </is>
+      </c>
+      <c r="I744" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="J744" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K744" t="n">
+        <v>36892144</v>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" s="2" t="n">
+        <v>46222</v>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="D745" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E745" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F745" t="n">
+        <v>31</v>
+      </c>
+      <c r="G745" t="n">
+        <v>33</v>
+      </c>
+      <c r="H745" t="inlineStr">
+        <is>
+          <t>31/33</t>
+        </is>
+      </c>
+      <c r="I745" s="3" t="n">
+        <v>93.90000000000001</v>
+      </c>
+      <c r="J745" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K745" t="n">
+        <v>36336245</v>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" s="2" t="n">
+        <v>46222</v>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="D746" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E746" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F746" t="n">
+        <v>27</v>
+      </c>
+      <c r="G746" t="n">
+        <v>33</v>
+      </c>
+      <c r="H746" t="inlineStr">
+        <is>
+          <t>27/33</t>
+        </is>
+      </c>
+      <c r="I746" s="5" t="n">
+        <v>81.8</v>
+      </c>
+      <c r="J746" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K746" t="n">
+        <v>36692757</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K740"/>
+  <autoFilter ref="A1:K746"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-07-21)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$746</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$752</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K746"/>
+  <dimension ref="A1:K752"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -35537,8 +35537,290 @@
         <v>36692757</v>
       </c>
     </row>
+    <row r="747">
+      <c r="A747" s="2" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D747" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E747" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F747" t="n">
+        <v>18</v>
+      </c>
+      <c r="G747" t="n">
+        <v>28</v>
+      </c>
+      <c r="H747" t="inlineStr">
+        <is>
+          <t>18/28</t>
+        </is>
+      </c>
+      <c r="I747" s="5" t="n">
+        <v>64.3</v>
+      </c>
+      <c r="J747" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K747" t="n">
+        <v>36390331</v>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" s="2" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D748" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E748" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F748" t="n">
+        <v>5</v>
+      </c>
+      <c r="G748" t="n">
+        <v>18</v>
+      </c>
+      <c r="H748" t="inlineStr">
+        <is>
+          <t>5/18</t>
+        </is>
+      </c>
+      <c r="I748" s="4" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="J748" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K748" t="n">
+        <v>38531910</v>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" s="2" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D749" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E749" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F749" t="n">
+        <v>1</v>
+      </c>
+      <c r="G749" t="n">
+        <v>18</v>
+      </c>
+      <c r="H749" t="inlineStr">
+        <is>
+          <t>1/18</t>
+        </is>
+      </c>
+      <c r="I749" s="4" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="J749" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K749" t="n">
+        <v>36928729</v>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" s="2" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D750" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E750" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F750" t="n">
+        <v>8</v>
+      </c>
+      <c r="G750" t="n">
+        <v>28</v>
+      </c>
+      <c r="H750" t="inlineStr">
+        <is>
+          <t>8/28</t>
+        </is>
+      </c>
+      <c r="I750" s="4" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="J750" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K750" t="n">
+        <v>36280998</v>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" s="2" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="D751" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E751" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F751" t="n">
+        <v>25</v>
+      </c>
+      <c r="G751" t="n">
+        <v>28</v>
+      </c>
+      <c r="H751" t="inlineStr">
+        <is>
+          <t>25/28</t>
+        </is>
+      </c>
+      <c r="I751" s="3" t="n">
+        <v>89.3</v>
+      </c>
+      <c r="J751" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K751" t="n">
+        <v>37873140</v>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" s="2" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D752" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E752" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F752" t="n">
+        <v>5</v>
+      </c>
+      <c r="G752" t="n">
+        <v>32</v>
+      </c>
+      <c r="H752" t="inlineStr">
+        <is>
+          <t>5/32</t>
+        </is>
+      </c>
+      <c r="I752" s="4" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="J752" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K752" t="n">
+        <v>36929035</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K746"/>
+  <autoFilter ref="A1:K752"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-07-22)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$752</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$758</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K752"/>
+  <dimension ref="A1:K758"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -35819,8 +35819,290 @@
         <v>36929035</v>
       </c>
     </row>
+    <row r="753">
+      <c r="A753" s="2" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D753" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E753" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F753" t="n">
+        <v>14</v>
+      </c>
+      <c r="G753" t="n">
+        <v>33</v>
+      </c>
+      <c r="H753" t="inlineStr">
+        <is>
+          <t>14/33</t>
+        </is>
+      </c>
+      <c r="I753" s="4" t="n">
+        <v>42.4</v>
+      </c>
+      <c r="J753" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K753" t="n">
+        <v>36321362</v>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" s="2" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D754" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E754" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F754" t="n">
+        <v>7</v>
+      </c>
+      <c r="G754" t="n">
+        <v>18</v>
+      </c>
+      <c r="H754" t="inlineStr">
+        <is>
+          <t>7/18</t>
+        </is>
+      </c>
+      <c r="I754" s="4" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="J754" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K754" t="n">
+        <v>36929161</v>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" s="2" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D755" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E755" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F755" t="n">
+        <v>4</v>
+      </c>
+      <c r="G755" t="n">
+        <v>18</v>
+      </c>
+      <c r="H755" t="inlineStr">
+        <is>
+          <t>4/18</t>
+        </is>
+      </c>
+      <c r="I755" s="4" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="J755" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K755" t="n">
+        <v>36298241</v>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" s="2" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C756" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D756" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E756" t="inlineStr">
+        <is>
+          <t>Faustine CHOPIN</t>
+        </is>
+      </c>
+      <c r="F756" t="n">
+        <v>13</v>
+      </c>
+      <c r="G756" t="n">
+        <v>28</v>
+      </c>
+      <c r="H756" t="inlineStr">
+        <is>
+          <t>13/28</t>
+        </is>
+      </c>
+      <c r="I756" s="4" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="J756" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K756" t="n">
+        <v>36297686</v>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" s="2" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C757" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="D757" t="inlineStr">
+        <is>
+          <t>RE-LAX  (English version)</t>
+        </is>
+      </c>
+      <c r="E757" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F757" t="n">
+        <v>15</v>
+      </c>
+      <c r="G757" t="n">
+        <v>28</v>
+      </c>
+      <c r="H757" t="inlineStr">
+        <is>
+          <t>15/28</t>
+        </is>
+      </c>
+      <c r="I757" s="5" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="J757" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K757" t="n">
+        <v>36298048</v>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" s="2" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B758" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C758" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D758" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E758" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F758" t="n">
+        <v>19</v>
+      </c>
+      <c r="G758" t="n">
+        <v>32</v>
+      </c>
+      <c r="H758" t="inlineStr">
+        <is>
+          <t>19/32</t>
+        </is>
+      </c>
+      <c r="I758" s="5" t="n">
+        <v>59.4</v>
+      </c>
+      <c r="J758" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K758" t="n">
+        <v>39647900</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K752"/>
+  <autoFilter ref="A1:K758"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-07-23)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$758</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$763</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K758"/>
+  <dimension ref="A1:K763"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -36101,8 +36101,243 @@
         <v>39647900</v>
       </c>
     </row>
+    <row r="759">
+      <c r="A759" s="2" t="n">
+        <v>46225</v>
+      </c>
+      <c r="B759" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C759" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D759" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E759" t="inlineStr">
+        <is>
+          <t>Alice Dunoyer</t>
+        </is>
+      </c>
+      <c r="F759" t="n">
+        <v>14</v>
+      </c>
+      <c r="G759" t="n">
+        <v>33</v>
+      </c>
+      <c r="H759" t="inlineStr">
+        <is>
+          <t>14/33</t>
+        </is>
+      </c>
+      <c r="I759" s="4" t="n">
+        <v>42.4</v>
+      </c>
+      <c r="J759" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K759" t="n">
+        <v>36321411</v>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" s="2" t="n">
+        <v>46225</v>
+      </c>
+      <c r="B760" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C760" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D760" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E760" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F760" t="n">
+        <v>12</v>
+      </c>
+      <c r="G760" t="n">
+        <v>18</v>
+      </c>
+      <c r="H760" t="inlineStr">
+        <is>
+          <t>12/18</t>
+        </is>
+      </c>
+      <c r="I760" s="5" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J760" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K760" t="n">
+        <v>36929293</v>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" s="2" t="n">
+        <v>46225</v>
+      </c>
+      <c r="B761" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C761" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D761" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E761" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F761" t="n">
+        <v>10</v>
+      </c>
+      <c r="G761" t="n">
+        <v>18</v>
+      </c>
+      <c r="H761" t="inlineStr">
+        <is>
+          <t>10/18</t>
+        </is>
+      </c>
+      <c r="I761" s="5" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="J761" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K761" t="n">
+        <v>36298342</v>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" s="2" t="n">
+        <v>46225</v>
+      </c>
+      <c r="B762" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C762" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D762" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E762" t="inlineStr">
+        <is>
+          <t>Pauline Ramon</t>
+        </is>
+      </c>
+      <c r="F762" t="n">
+        <v>26</v>
+      </c>
+      <c r="G762" t="n">
+        <v>33</v>
+      </c>
+      <c r="H762" t="inlineStr">
+        <is>
+          <t>26/33</t>
+        </is>
+      </c>
+      <c r="I762" s="5" t="n">
+        <v>78.8</v>
+      </c>
+      <c r="J762" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K762" t="n">
+        <v>36298383</v>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" s="2" t="n">
+        <v>46225</v>
+      </c>
+      <c r="B763" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C763" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D763" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E763" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F763" t="n">
+        <v>13</v>
+      </c>
+      <c r="G763" t="n">
+        <v>33</v>
+      </c>
+      <c r="H763" t="inlineStr">
+        <is>
+          <t>13/33</t>
+        </is>
+      </c>
+      <c r="I763" s="4" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="J763" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K763" t="n">
+        <v>36298580</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K758"/>
+  <autoFilter ref="A1:K763"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-07-24)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$763</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$768</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K763"/>
+  <dimension ref="A1:K768"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -36126,18 +36126,18 @@
         </is>
       </c>
       <c r="F759" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G759" t="n">
         <v>33</v>
       </c>
       <c r="H759" t="inlineStr">
         <is>
-          <t>14/33</t>
+          <t>13/33</t>
         </is>
       </c>
       <c r="I759" s="4" t="n">
-        <v>42.4</v>
+        <v>39.4</v>
       </c>
       <c r="J759" t="inlineStr">
         <is>
@@ -36336,8 +36336,243 @@
         <v>36298580</v>
       </c>
     </row>
+    <row r="764">
+      <c r="A764" s="2" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B764" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C764" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D764" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E764" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F764" t="n">
+        <v>13</v>
+      </c>
+      <c r="G764" t="n">
+        <v>33</v>
+      </c>
+      <c r="H764" t="inlineStr">
+        <is>
+          <t>13/33</t>
+        </is>
+      </c>
+      <c r="I764" s="4" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="J764" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K764" t="n">
+        <v>36321562</v>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" s="2" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B765" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C765" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D765" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E765" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F765" t="n">
+        <v>12</v>
+      </c>
+      <c r="G765" t="n">
+        <v>18</v>
+      </c>
+      <c r="H765" t="inlineStr">
+        <is>
+          <t>12/18</t>
+        </is>
+      </c>
+      <c r="I765" s="5" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J765" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K765" t="n">
+        <v>36929384</v>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" s="2" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B766" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C766" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D766" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E766" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F766" t="n">
+        <v>11</v>
+      </c>
+      <c r="G766" t="n">
+        <v>18</v>
+      </c>
+      <c r="H766" t="inlineStr">
+        <is>
+          <t>11/18</t>
+        </is>
+      </c>
+      <c r="I766" s="5" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="J766" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K766" t="n">
+        <v>36298757</v>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" s="2" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B767" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C767" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D767" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E767" t="inlineStr">
+        <is>
+          <t>Faustine CHOPIN</t>
+        </is>
+      </c>
+      <c r="F767" t="n">
+        <v>20</v>
+      </c>
+      <c r="G767" t="n">
+        <v>33</v>
+      </c>
+      <c r="H767" t="inlineStr">
+        <is>
+          <t>20/33</t>
+        </is>
+      </c>
+      <c r="I767" s="5" t="n">
+        <v>60.6</v>
+      </c>
+      <c r="J767" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K767" t="n">
+        <v>36298811</v>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" s="2" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B768" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C768" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D768" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E768" t="inlineStr">
+        <is>
+          <t>Nina Petitjean</t>
+        </is>
+      </c>
+      <c r="F768" t="n">
+        <v>16</v>
+      </c>
+      <c r="G768" t="n">
+        <v>28</v>
+      </c>
+      <c r="H768" t="inlineStr">
+        <is>
+          <t>16/28</t>
+        </is>
+      </c>
+      <c r="I768" s="5" t="n">
+        <v>57.1</v>
+      </c>
+      <c r="J768" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K768" t="n">
+        <v>36298864</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K763"/>
+  <autoFilter ref="A1:K768"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-07-25)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$768</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$775</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K768"/>
+  <dimension ref="A1:K775"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -36571,8 +36571,337 @@
         <v>36298864</v>
       </c>
     </row>
+    <row r="769">
+      <c r="A769" s="2" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B769" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C769" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D769" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E769" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F769" t="n">
+        <v>19</v>
+      </c>
+      <c r="G769" t="n">
+        <v>32</v>
+      </c>
+      <c r="H769" t="inlineStr">
+        <is>
+          <t>19/32</t>
+        </is>
+      </c>
+      <c r="I769" s="5" t="n">
+        <v>59.4</v>
+      </c>
+      <c r="J769" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K769" t="n">
+        <v>36319500</v>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" s="2" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B770" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C770" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D770" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E770" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F770" t="n">
+        <v>4</v>
+      </c>
+      <c r="G770" t="n">
+        <v>16</v>
+      </c>
+      <c r="H770" t="inlineStr">
+        <is>
+          <t>4/16</t>
+        </is>
+      </c>
+      <c r="I770" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="J770" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K770" t="n">
+        <v>36320658</v>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" s="2" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B771" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C771" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D771" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E771" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F771" t="n">
+        <v>3</v>
+      </c>
+      <c r="G771" t="n">
+        <v>16</v>
+      </c>
+      <c r="H771" t="inlineStr">
+        <is>
+          <t>3/16</t>
+        </is>
+      </c>
+      <c r="I771" s="4" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="J771" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K771" t="n">
+        <v>36320057</v>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" s="2" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B772" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C772" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D772" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E772" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F772" t="n">
+        <v>13</v>
+      </c>
+      <c r="G772" t="n">
+        <v>33</v>
+      </c>
+      <c r="H772" t="inlineStr">
+        <is>
+          <t>13/33</t>
+        </is>
+      </c>
+      <c r="I772" s="4" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="J772" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K772" t="n">
+        <v>36320781</v>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" s="2" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B773" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C773" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D773" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E773" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F773" t="n">
+        <v>26</v>
+      </c>
+      <c r="G773" t="n">
+        <v>33</v>
+      </c>
+      <c r="H773" t="inlineStr">
+        <is>
+          <t>26/33</t>
+        </is>
+      </c>
+      <c r="I773" s="5" t="n">
+        <v>78.8</v>
+      </c>
+      <c r="J773" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K773" t="n">
+        <v>36320891</v>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" s="2" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B774" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C774" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D774" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E774" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F774" t="n">
+        <v>12</v>
+      </c>
+      <c r="G774" t="n">
+        <v>20</v>
+      </c>
+      <c r="H774" t="inlineStr">
+        <is>
+          <t>12/20</t>
+        </is>
+      </c>
+      <c r="I774" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="J774" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K774" t="n">
+        <v>36893828</v>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" s="2" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B775" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C775" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D775" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E775" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F775" t="n">
+        <v>5</v>
+      </c>
+      <c r="G775" t="n">
+        <v>20</v>
+      </c>
+      <c r="H775" t="inlineStr">
+        <is>
+          <t>5/20</t>
+        </is>
+      </c>
+      <c r="I775" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="J775" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K775" t="n">
+        <v>36893884</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K768"/>
+  <autoFilter ref="A1:K775"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-07-26)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$775</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$781</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K775"/>
+  <dimension ref="A1:K781"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -36900,8 +36900,290 @@
         <v>36893884</v>
       </c>
     </row>
+    <row r="776">
+      <c r="A776" s="2" t="n">
+        <v>46228</v>
+      </c>
+      <c r="B776" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C776" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D776" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E776" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F776" t="n">
+        <v>5</v>
+      </c>
+      <c r="G776" t="n">
+        <v>32</v>
+      </c>
+      <c r="H776" t="inlineStr">
+        <is>
+          <t>5/32</t>
+        </is>
+      </c>
+      <c r="I776" s="4" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="J776" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K776" t="n">
+        <v>36323275</v>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" s="2" t="n">
+        <v>46228</v>
+      </c>
+      <c r="B777" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C777" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D777" t="inlineStr">
+        <is>
+          <t>RE-BOOST  (English version)</t>
+        </is>
+      </c>
+      <c r="E777" t="inlineStr">
+        <is>
+          <t>Alice Dunoyer</t>
+        </is>
+      </c>
+      <c r="F777" t="n">
+        <v>19</v>
+      </c>
+      <c r="G777" t="n">
+        <v>33</v>
+      </c>
+      <c r="H777" t="inlineStr">
+        <is>
+          <t>19/33</t>
+        </is>
+      </c>
+      <c r="I777" s="5" t="n">
+        <v>57.6</v>
+      </c>
+      <c r="J777" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K777" t="n">
+        <v>36323121</v>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" s="2" t="n">
+        <v>46228</v>
+      </c>
+      <c r="B778" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C778" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D778" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E778" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F778" t="n">
+        <v>6</v>
+      </c>
+      <c r="G778" t="n">
+        <v>32</v>
+      </c>
+      <c r="H778" t="inlineStr">
+        <is>
+          <t>6/32</t>
+        </is>
+      </c>
+      <c r="I778" s="4" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="J778" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K778" t="n">
+        <v>38771773</v>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" s="2" t="n">
+        <v>46228</v>
+      </c>
+      <c r="B779" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C779" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D779" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E779" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F779" t="n">
+        <v>28</v>
+      </c>
+      <c r="G779" t="n">
+        <v>33</v>
+      </c>
+      <c r="H779" t="inlineStr">
+        <is>
+          <t>28/33</t>
+        </is>
+      </c>
+      <c r="I779" s="5" t="n">
+        <v>84.8</v>
+      </c>
+      <c r="J779" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K779" t="n">
+        <v>36329203</v>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" s="2" t="n">
+        <v>46228</v>
+      </c>
+      <c r="B780" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C780" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="D780" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E780" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F780" t="n">
+        <v>22</v>
+      </c>
+      <c r="G780" t="n">
+        <v>32</v>
+      </c>
+      <c r="H780" t="inlineStr">
+        <is>
+          <t>22/32</t>
+        </is>
+      </c>
+      <c r="I780" s="5" t="n">
+        <v>68.8</v>
+      </c>
+      <c r="J780" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K780" t="n">
+        <v>38771873</v>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" s="2" t="n">
+        <v>46228</v>
+      </c>
+      <c r="B781" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C781" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D781" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E781" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F781" t="n">
+        <v>27</v>
+      </c>
+      <c r="G781" t="n">
+        <v>33</v>
+      </c>
+      <c r="H781" t="inlineStr">
+        <is>
+          <t>27/33</t>
+        </is>
+      </c>
+      <c r="I781" s="5" t="n">
+        <v>81.8</v>
+      </c>
+      <c r="J781" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K781" t="n">
+        <v>36329968</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K775"/>
+  <autoFilter ref="A1:K781"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-07-27)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$781</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$787</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K781"/>
+  <dimension ref="A1:K787"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -37182,8 +37182,290 @@
         <v>36329968</v>
       </c>
     </row>
+    <row r="782">
+      <c r="A782" s="2" t="n">
+        <v>46229</v>
+      </c>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C782" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D782" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E782" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F782" t="n">
+        <v>11</v>
+      </c>
+      <c r="G782" t="n">
+        <v>36</v>
+      </c>
+      <c r="H782" t="inlineStr">
+        <is>
+          <t>11/36</t>
+        </is>
+      </c>
+      <c r="I782" s="4" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="J782" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K782" t="n">
+        <v>37240285</v>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" s="2" t="n">
+        <v>46229</v>
+      </c>
+      <c r="B783" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C783" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D783" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E783" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F783" t="n">
+        <v>23</v>
+      </c>
+      <c r="G783" t="n">
+        <v>33</v>
+      </c>
+      <c r="H783" t="inlineStr">
+        <is>
+          <t>23/33</t>
+        </is>
+      </c>
+      <c r="I783" s="5" t="n">
+        <v>69.7</v>
+      </c>
+      <c r="J783" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K783" t="n">
+        <v>36336031</v>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" s="2" t="n">
+        <v>46229</v>
+      </c>
+      <c r="B784" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C784" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D784" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E784" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F784" t="n">
+        <v>2</v>
+      </c>
+      <c r="G784" t="n">
+        <v>28</v>
+      </c>
+      <c r="H784" t="inlineStr">
+        <is>
+          <t>2/28</t>
+        </is>
+      </c>
+      <c r="I784" s="4" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="J784" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K784" t="n">
+        <v>37240428</v>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" s="2" t="n">
+        <v>46229</v>
+      </c>
+      <c r="B785" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C785" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="D785" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E785" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F785" t="n">
+        <v>35</v>
+      </c>
+      <c r="G785" t="n">
+        <v>28</v>
+      </c>
+      <c r="H785" t="inlineStr">
+        <is>
+          <t>35/28</t>
+        </is>
+      </c>
+      <c r="I785" s="3" t="n">
+        <v>125</v>
+      </c>
+      <c r="J785" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K785" t="n">
+        <v>36892145</v>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" s="2" t="n">
+        <v>46229</v>
+      </c>
+      <c r="B786" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C786" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="D786" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E786" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F786" t="n">
+        <v>33</v>
+      </c>
+      <c r="G786" t="n">
+        <v>33</v>
+      </c>
+      <c r="H786" t="inlineStr">
+        <is>
+          <t>33/33</t>
+        </is>
+      </c>
+      <c r="I786" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J786" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K786" t="n">
+        <v>36336246</v>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" s="2" t="n">
+        <v>46229</v>
+      </c>
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C787" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="D787" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E787" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F787" t="n">
+        <v>31</v>
+      </c>
+      <c r="G787" t="n">
+        <v>33</v>
+      </c>
+      <c r="H787" t="inlineStr">
+        <is>
+          <t>31/33</t>
+        </is>
+      </c>
+      <c r="I787" s="3" t="n">
+        <v>93.90000000000001</v>
+      </c>
+      <c r="J787" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K787" t="n">
+        <v>36692758</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K781"/>
+  <autoFilter ref="A1:K787"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-07-28)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$787</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$793</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K787"/>
+  <dimension ref="A1:K793"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -37464,8 +37464,290 @@
         <v>36692758</v>
       </c>
     </row>
+    <row r="788">
+      <c r="A788" s="2" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C788" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D788" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E788" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F788" t="n">
+        <v>6</v>
+      </c>
+      <c r="G788" t="n">
+        <v>28</v>
+      </c>
+      <c r="H788" t="inlineStr">
+        <is>
+          <t>6/28</t>
+        </is>
+      </c>
+      <c r="I788" s="4" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="J788" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K788" t="n">
+        <v>36390332</v>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" s="2" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C789" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D789" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E789" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F789" t="n">
+        <v>8</v>
+      </c>
+      <c r="G789" t="n">
+        <v>18</v>
+      </c>
+      <c r="H789" t="inlineStr">
+        <is>
+          <t>8/18</t>
+        </is>
+      </c>
+      <c r="I789" s="4" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="J789" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K789" t="n">
+        <v>38531911</v>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" s="2" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C790" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D790" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E790" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F790" t="n">
+        <v>11</v>
+      </c>
+      <c r="G790" t="n">
+        <v>18</v>
+      </c>
+      <c r="H790" t="inlineStr">
+        <is>
+          <t>11/18</t>
+        </is>
+      </c>
+      <c r="I790" s="5" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="J790" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K790" t="n">
+        <v>36928730</v>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" s="2" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C791" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D791" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E791" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F791" t="n">
+        <v>22</v>
+      </c>
+      <c r="G791" t="n">
+        <v>28</v>
+      </c>
+      <c r="H791" t="inlineStr">
+        <is>
+          <t>22/28</t>
+        </is>
+      </c>
+      <c r="I791" s="5" t="n">
+        <v>78.59999999999999</v>
+      </c>
+      <c r="J791" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K791" t="n">
+        <v>36280999</v>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" s="2" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C792" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="D792" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E792" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F792" t="n">
+        <v>18</v>
+      </c>
+      <c r="G792" t="n">
+        <v>28</v>
+      </c>
+      <c r="H792" t="inlineStr">
+        <is>
+          <t>18/28</t>
+        </is>
+      </c>
+      <c r="I792" s="5" t="n">
+        <v>64.3</v>
+      </c>
+      <c r="J792" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K792" t="n">
+        <v>37873141</v>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" s="2" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D793" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E793" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F793" t="n">
+        <v>10</v>
+      </c>
+      <c r="G793" t="n">
+        <v>32</v>
+      </c>
+      <c r="H793" t="inlineStr">
+        <is>
+          <t>10/32</t>
+        </is>
+      </c>
+      <c r="I793" s="4" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="J793" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K793" t="n">
+        <v>36929036</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K787"/>
+  <autoFilter ref="A1:K793"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-07-29)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$793</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$799</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K793"/>
+  <dimension ref="A1:K799"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -37746,8 +37746,290 @@
         <v>36929036</v>
       </c>
     </row>
+    <row r="794">
+      <c r="A794" s="2" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C794" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D794" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E794" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F794" t="n">
+        <v>10</v>
+      </c>
+      <c r="G794" t="n">
+        <v>33</v>
+      </c>
+      <c r="H794" t="inlineStr">
+        <is>
+          <t>10/33</t>
+        </is>
+      </c>
+      <c r="I794" s="4" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="J794" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K794" t="n">
+        <v>36321363</v>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" s="2" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C795" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D795" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E795" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F795" t="n">
+        <v>9</v>
+      </c>
+      <c r="G795" t="n">
+        <v>18</v>
+      </c>
+      <c r="H795" t="inlineStr">
+        <is>
+          <t>9/18</t>
+        </is>
+      </c>
+      <c r="I795" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J795" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K795" t="n">
+        <v>36929162</v>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" s="2" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C796" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D796" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E796" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F796" t="n">
+        <v>5</v>
+      </c>
+      <c r="G796" t="n">
+        <v>18</v>
+      </c>
+      <c r="H796" t="inlineStr">
+        <is>
+          <t>5/18</t>
+        </is>
+      </c>
+      <c r="I796" s="4" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="J796" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K796" t="n">
+        <v>36298242</v>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" s="2" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C797" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D797" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E797" t="inlineStr">
+        <is>
+          <t>Faustine CHOPIN</t>
+        </is>
+      </c>
+      <c r="F797" t="n">
+        <v>16</v>
+      </c>
+      <c r="G797" t="n">
+        <v>28</v>
+      </c>
+      <c r="H797" t="inlineStr">
+        <is>
+          <t>16/28</t>
+        </is>
+      </c>
+      <c r="I797" s="5" t="n">
+        <v>57.1</v>
+      </c>
+      <c r="J797" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K797" t="n">
+        <v>36297687</v>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" s="2" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C798" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="D798" t="inlineStr">
+        <is>
+          <t>RE-LAX  (English version)</t>
+        </is>
+      </c>
+      <c r="E798" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F798" t="n">
+        <v>20</v>
+      </c>
+      <c r="G798" t="n">
+        <v>28</v>
+      </c>
+      <c r="H798" t="inlineStr">
+        <is>
+          <t>20/28</t>
+        </is>
+      </c>
+      <c r="I798" s="5" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="J798" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K798" t="n">
+        <v>36298049</v>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" s="2" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C799" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D799" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E799" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F799" t="n">
+        <v>11</v>
+      </c>
+      <c r="G799" t="n">
+        <v>32</v>
+      </c>
+      <c r="H799" t="inlineStr">
+        <is>
+          <t>11/32</t>
+        </is>
+      </c>
+      <c r="I799" s="4" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="J799" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K799" t="n">
+        <v>40419636</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K793"/>
+  <autoFilter ref="A1:K799"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-07-30)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$799</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$804</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K799"/>
+  <dimension ref="A1:K804"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -38028,8 +38028,243 @@
         <v>40419636</v>
       </c>
     </row>
+    <row r="800">
+      <c r="A800" s="2" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C800" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D800" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E800" t="inlineStr">
+        <is>
+          <t>Alice Dunoyer</t>
+        </is>
+      </c>
+      <c r="F800" t="n">
+        <v>12</v>
+      </c>
+      <c r="G800" t="n">
+        <v>33</v>
+      </c>
+      <c r="H800" t="inlineStr">
+        <is>
+          <t>12/33</t>
+        </is>
+      </c>
+      <c r="I800" s="4" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="J800" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K800" t="n">
+        <v>36321412</v>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" s="2" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C801" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D801" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E801" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F801" t="n">
+        <v>6</v>
+      </c>
+      <c r="G801" t="n">
+        <v>18</v>
+      </c>
+      <c r="H801" t="inlineStr">
+        <is>
+          <t>6/18</t>
+        </is>
+      </c>
+      <c r="I801" s="4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J801" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K801" t="n">
+        <v>36929294</v>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" s="2" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B802" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C802" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D802" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E802" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F802" t="n">
+        <v>4</v>
+      </c>
+      <c r="G802" t="n">
+        <v>18</v>
+      </c>
+      <c r="H802" t="inlineStr">
+        <is>
+          <t>4/18</t>
+        </is>
+      </c>
+      <c r="I802" s="4" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="J802" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K802" t="n">
+        <v>36298343</v>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" s="2" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B803" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C803" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D803" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E803" t="inlineStr">
+        <is>
+          <t>Pauline Ramon</t>
+        </is>
+      </c>
+      <c r="F803" t="n">
+        <v>33</v>
+      </c>
+      <c r="G803" t="n">
+        <v>33</v>
+      </c>
+      <c r="H803" t="inlineStr">
+        <is>
+          <t>33/33</t>
+        </is>
+      </c>
+      <c r="I803" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J803" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K803" t="n">
+        <v>36298384</v>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" s="2" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C804" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D804" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E804" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F804" t="n">
+        <v>25</v>
+      </c>
+      <c r="G804" t="n">
+        <v>33</v>
+      </c>
+      <c r="H804" t="inlineStr">
+        <is>
+          <t>25/33</t>
+        </is>
+      </c>
+      <c r="I804" s="5" t="n">
+        <v>75.8</v>
+      </c>
+      <c r="J804" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K804" t="n">
+        <v>36298581</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K799"/>
+  <autoFilter ref="A1:K804"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-07-31)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$804</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$809</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K804"/>
+  <dimension ref="A1:K809"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -38263,8 +38263,243 @@
         <v>36298581</v>
       </c>
     </row>
+    <row r="805">
+      <c r="A805" s="2" t="n">
+        <v>46233</v>
+      </c>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C805" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D805" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E805" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F805" t="n">
+        <v>15</v>
+      </c>
+      <c r="G805" t="n">
+        <v>33</v>
+      </c>
+      <c r="H805" t="inlineStr">
+        <is>
+          <t>15/33</t>
+        </is>
+      </c>
+      <c r="I805" s="4" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="J805" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K805" t="n">
+        <v>36321563</v>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" s="2" t="n">
+        <v>46233</v>
+      </c>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C806" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D806" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E806" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F806" t="n">
+        <v>7</v>
+      </c>
+      <c r="G806" t="n">
+        <v>18</v>
+      </c>
+      <c r="H806" t="inlineStr">
+        <is>
+          <t>7/18</t>
+        </is>
+      </c>
+      <c r="I806" s="4" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="J806" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K806" t="n">
+        <v>36929385</v>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" s="2" t="n">
+        <v>46233</v>
+      </c>
+      <c r="B807" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C807" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D807" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E807" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F807" t="n">
+        <v>11</v>
+      </c>
+      <c r="G807" t="n">
+        <v>18</v>
+      </c>
+      <c r="H807" t="inlineStr">
+        <is>
+          <t>11/18</t>
+        </is>
+      </c>
+      <c r="I807" s="5" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="J807" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K807" t="n">
+        <v>36298758</v>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" s="2" t="n">
+        <v>46233</v>
+      </c>
+      <c r="B808" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C808" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D808" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E808" t="inlineStr">
+        <is>
+          <t>Faustine CHOPIN</t>
+        </is>
+      </c>
+      <c r="F808" t="n">
+        <v>26</v>
+      </c>
+      <c r="G808" t="n">
+        <v>33</v>
+      </c>
+      <c r="H808" t="inlineStr">
+        <is>
+          <t>26/33</t>
+        </is>
+      </c>
+      <c r="I808" s="5" t="n">
+        <v>78.8</v>
+      </c>
+      <c r="J808" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K808" t="n">
+        <v>36298812</v>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" s="2" t="n">
+        <v>46233</v>
+      </c>
+      <c r="B809" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D809" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E809" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F809" t="n">
+        <v>20</v>
+      </c>
+      <c r="G809" t="n">
+        <v>33</v>
+      </c>
+      <c r="H809" t="inlineStr">
+        <is>
+          <t>20/33</t>
+        </is>
+      </c>
+      <c r="I809" s="5" t="n">
+        <v>60.6</v>
+      </c>
+      <c r="J809" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K809" t="n">
+        <v>36298865</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K804"/>
+  <autoFilter ref="A1:K809"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-08-01)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$809</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$816</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K809"/>
+  <dimension ref="A1:K816"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -38498,8 +38498,337 @@
         <v>36298865</v>
       </c>
     </row>
+    <row r="810">
+      <c r="A810" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D810" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E810" t="inlineStr">
+        <is>
+          <t>David Bertin</t>
+        </is>
+      </c>
+      <c r="F810" t="n">
+        <v>8</v>
+      </c>
+      <c r="G810" t="n">
+        <v>33</v>
+      </c>
+      <c r="H810" t="inlineStr">
+        <is>
+          <t>8/33</t>
+        </is>
+      </c>
+      <c r="I810" s="4" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="J810" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K810" t="n">
+        <v>36319501</v>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D811" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E811" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F811" t="n">
+        <v>3</v>
+      </c>
+      <c r="G811" t="n">
+        <v>16</v>
+      </c>
+      <c r="H811" t="inlineStr">
+        <is>
+          <t>3/16</t>
+        </is>
+      </c>
+      <c r="I811" s="4" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="J811" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K811" t="n">
+        <v>36320659</v>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B812" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D812" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E812" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F812" t="n">
+        <v>4</v>
+      </c>
+      <c r="G812" t="n">
+        <v>16</v>
+      </c>
+      <c r="H812" t="inlineStr">
+        <is>
+          <t>4/16</t>
+        </is>
+      </c>
+      <c r="I812" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="J812" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K812" t="n">
+        <v>36320058</v>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B813" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C813" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D813" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E813" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F813" t="n">
+        <v>6</v>
+      </c>
+      <c r="G813" t="n">
+        <v>33</v>
+      </c>
+      <c r="H813" t="inlineStr">
+        <is>
+          <t>6/33</t>
+        </is>
+      </c>
+      <c r="I813" s="4" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="J813" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K813" t="n">
+        <v>36320782</v>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B814" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C814" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D814" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E814" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F814" t="n">
+        <v>25</v>
+      </c>
+      <c r="G814" t="n">
+        <v>33</v>
+      </c>
+      <c r="H814" t="inlineStr">
+        <is>
+          <t>25/33</t>
+        </is>
+      </c>
+      <c r="I814" s="5" t="n">
+        <v>75.8</v>
+      </c>
+      <c r="J814" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K814" t="n">
+        <v>36320892</v>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B815" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C815" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D815" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E815" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F815" t="n">
+        <v>8</v>
+      </c>
+      <c r="G815" t="n">
+        <v>20</v>
+      </c>
+      <c r="H815" t="inlineStr">
+        <is>
+          <t>8/20</t>
+        </is>
+      </c>
+      <c r="I815" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="J815" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K815" t="n">
+        <v>36893829</v>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B816" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C816" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D816" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E816" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F816" t="n">
+        <v>6</v>
+      </c>
+      <c r="G816" t="n">
+        <v>20</v>
+      </c>
+      <c r="H816" t="inlineStr">
+        <is>
+          <t>6/20</t>
+        </is>
+      </c>
+      <c r="I816" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="J816" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K816" t="n">
+        <v>36893887</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K809"/>
+  <autoFilter ref="A1:K816"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-08-02)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$816</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$822</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K816"/>
+  <dimension ref="A1:K822"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -38827,8 +38827,290 @@
         <v>36893887</v>
       </c>
     </row>
+    <row r="817">
+      <c r="A817" s="2" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B817" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C817" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D817" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E817" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F817" t="n">
+        <v>4</v>
+      </c>
+      <c r="G817" t="n">
+        <v>32</v>
+      </c>
+      <c r="H817" t="inlineStr">
+        <is>
+          <t>4/32</t>
+        </is>
+      </c>
+      <c r="I817" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="J817" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K817" t="n">
+        <v>36323276</v>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" s="2" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B818" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C818" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D818" t="inlineStr">
+        <is>
+          <t>RE-BOOST  (English version)</t>
+        </is>
+      </c>
+      <c r="E818" t="inlineStr">
+        <is>
+          <t>Alice Dunoyer</t>
+        </is>
+      </c>
+      <c r="F818" t="n">
+        <v>10</v>
+      </c>
+      <c r="G818" t="n">
+        <v>33</v>
+      </c>
+      <c r="H818" t="inlineStr">
+        <is>
+          <t>10/33</t>
+        </is>
+      </c>
+      <c r="I818" s="4" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="J818" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K818" t="n">
+        <v>36323122</v>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" s="2" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B819" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C819" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D819" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E819" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F819" t="n">
+        <v>11</v>
+      </c>
+      <c r="G819" t="n">
+        <v>32</v>
+      </c>
+      <c r="H819" t="inlineStr">
+        <is>
+          <t>11/32</t>
+        </is>
+      </c>
+      <c r="I819" s="4" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="J819" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K819" t="n">
+        <v>38771774</v>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" s="2" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B820" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C820" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D820" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E820" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F820" t="n">
+        <v>13</v>
+      </c>
+      <c r="G820" t="n">
+        <v>33</v>
+      </c>
+      <c r="H820" t="inlineStr">
+        <is>
+          <t>13/33</t>
+        </is>
+      </c>
+      <c r="I820" s="4" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="J820" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K820" t="n">
+        <v>36329204</v>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" s="2" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B821" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C821" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="D821" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E821" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F821" t="n">
+        <v>8</v>
+      </c>
+      <c r="G821" t="n">
+        <v>32</v>
+      </c>
+      <c r="H821" t="inlineStr">
+        <is>
+          <t>8/32</t>
+        </is>
+      </c>
+      <c r="I821" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="J821" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K821" t="n">
+        <v>38771874</v>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" s="2" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D822" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E822" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F822" t="n">
+        <v>19</v>
+      </c>
+      <c r="G822" t="n">
+        <v>33</v>
+      </c>
+      <c r="H822" t="inlineStr">
+        <is>
+          <t>19/33</t>
+        </is>
+      </c>
+      <c r="I822" s="5" t="n">
+        <v>57.6</v>
+      </c>
+      <c r="J822" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K822" t="n">
+        <v>36329969</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K816"/>
+  <autoFilter ref="A1:K822"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-08-03)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$822</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$828</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K822"/>
+  <dimension ref="A1:K828"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -39109,8 +39109,290 @@
         <v>36329969</v>
       </c>
     </row>
+    <row r="823">
+      <c r="A823" s="2" t="n">
+        <v>46236</v>
+      </c>
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D823" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E823" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F823" t="n">
+        <v>4</v>
+      </c>
+      <c r="G823" t="n">
+        <v>36</v>
+      </c>
+      <c r="H823" t="inlineStr">
+        <is>
+          <t>4/36</t>
+        </is>
+      </c>
+      <c r="I823" s="4" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="J823" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K823" t="n">
+        <v>37240286</v>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" s="2" t="n">
+        <v>46236</v>
+      </c>
+      <c r="B824" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C824" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D824" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E824" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F824" t="n">
+        <v>11</v>
+      </c>
+      <c r="G824" t="n">
+        <v>33</v>
+      </c>
+      <c r="H824" t="inlineStr">
+        <is>
+          <t>11/33</t>
+        </is>
+      </c>
+      <c r="I824" s="4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J824" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K824" t="n">
+        <v>36336032</v>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" s="2" t="n">
+        <v>46236</v>
+      </c>
+      <c r="B825" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C825" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D825" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E825" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F825" t="n">
+        <v>11</v>
+      </c>
+      <c r="G825" t="n">
+        <v>32</v>
+      </c>
+      <c r="H825" t="inlineStr">
+        <is>
+          <t>11/32</t>
+        </is>
+      </c>
+      <c r="I825" s="4" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="J825" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K825" t="n">
+        <v>37240429</v>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" s="2" t="n">
+        <v>46236</v>
+      </c>
+      <c r="B826" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C826" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="D826" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E826" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F826" t="n">
+        <v>12</v>
+      </c>
+      <c r="G826" t="n">
+        <v>28</v>
+      </c>
+      <c r="H826" t="inlineStr">
+        <is>
+          <t>12/28</t>
+        </is>
+      </c>
+      <c r="I826" s="4" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="J826" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K826" t="n">
+        <v>36892146</v>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" s="2" t="n">
+        <v>46236</v>
+      </c>
+      <c r="B827" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C827" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="D827" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E827" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F827" t="n">
+        <v>27</v>
+      </c>
+      <c r="G827" t="n">
+        <v>33</v>
+      </c>
+      <c r="H827" t="inlineStr">
+        <is>
+          <t>27/33</t>
+        </is>
+      </c>
+      <c r="I827" s="5" t="n">
+        <v>81.8</v>
+      </c>
+      <c r="J827" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K827" t="n">
+        <v>36336247</v>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" s="2" t="n">
+        <v>46236</v>
+      </c>
+      <c r="B828" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C828" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="D828" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E828" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F828" t="n">
+        <v>29</v>
+      </c>
+      <c r="G828" t="n">
+        <v>33</v>
+      </c>
+      <c r="H828" t="inlineStr">
+        <is>
+          <t>29/33</t>
+        </is>
+      </c>
+      <c r="I828" s="3" t="n">
+        <v>87.90000000000001</v>
+      </c>
+      <c r="J828" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K828" t="n">
+        <v>36692759</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K822"/>
+  <autoFilter ref="A1:K828"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-08-04)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$828</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$832</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K828"/>
+  <dimension ref="A1:K832"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -39391,8 +39391,196 @@
         <v>36692759</v>
       </c>
     </row>
+    <row r="829">
+      <c r="A829" s="2" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D829" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E829" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F829" t="n">
+        <v>7</v>
+      </c>
+      <c r="G829" t="n">
+        <v>18</v>
+      </c>
+      <c r="H829" t="inlineStr">
+        <is>
+          <t>7/18</t>
+        </is>
+      </c>
+      <c r="I829" s="4" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="J829" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K829" t="n">
+        <v>36928731</v>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" s="2" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D830" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E830" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F830" t="n">
+        <v>4</v>
+      </c>
+      <c r="G830" t="n">
+        <v>18</v>
+      </c>
+      <c r="H830" t="inlineStr">
+        <is>
+          <t>4/18</t>
+        </is>
+      </c>
+      <c r="I830" s="4" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="J830" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K830" t="n">
+        <v>38531912</v>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" s="2" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D831" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E831" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F831" t="n">
+        <v>28</v>
+      </c>
+      <c r="G831" t="n">
+        <v>28</v>
+      </c>
+      <c r="H831" t="inlineStr">
+        <is>
+          <t>28/28</t>
+        </is>
+      </c>
+      <c r="I831" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J831" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K831" t="n">
+        <v>36281000</v>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" s="2" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B832" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C832" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D832" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E832" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F832" t="n">
+        <v>19</v>
+      </c>
+      <c r="G832" t="n">
+        <v>34</v>
+      </c>
+      <c r="H832" t="inlineStr">
+        <is>
+          <t>19/34</t>
+        </is>
+      </c>
+      <c r="I832" s="5" t="n">
+        <v>55.9</v>
+      </c>
+      <c r="J832" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K832" t="n">
+        <v>36929037</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K828"/>
+  <autoFilter ref="A1:K832"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-08-05)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$832</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$836</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K832"/>
+  <dimension ref="A1:K836"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -39579,8 +39579,196 @@
         <v>36929037</v>
       </c>
     </row>
+    <row r="833">
+      <c r="A833" s="2" t="n">
+        <v>46238</v>
+      </c>
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D833" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E833" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F833" t="n">
+        <v>5</v>
+      </c>
+      <c r="G833" t="n">
+        <v>18</v>
+      </c>
+      <c r="H833" t="inlineStr">
+        <is>
+          <t>5/18</t>
+        </is>
+      </c>
+      <c r="I833" s="4" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="J833" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K833" t="n">
+        <v>36929163</v>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" s="2" t="n">
+        <v>46238</v>
+      </c>
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D834" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E834" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F834" t="n">
+        <v>3</v>
+      </c>
+      <c r="G834" t="n">
+        <v>18</v>
+      </c>
+      <c r="H834" t="inlineStr">
+        <is>
+          <t>3/18</t>
+        </is>
+      </c>
+      <c r="I834" s="4" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="J834" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K834" t="n">
+        <v>36298243</v>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" s="2" t="n">
+        <v>46238</v>
+      </c>
+      <c r="B835" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C835" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D835" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E835" t="inlineStr">
+        <is>
+          <t>Faustine CHOPIN</t>
+        </is>
+      </c>
+      <c r="F835" t="n">
+        <v>24</v>
+      </c>
+      <c r="G835" t="n">
+        <v>28</v>
+      </c>
+      <c r="H835" t="inlineStr">
+        <is>
+          <t>24/28</t>
+        </is>
+      </c>
+      <c r="I835" s="3" t="n">
+        <v>85.7</v>
+      </c>
+      <c r="J835" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K835" t="n">
+        <v>36297688</v>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" s="2" t="n">
+        <v>46238</v>
+      </c>
+      <c r="B836" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D836" t="inlineStr">
+        <is>
+          <t>RE-LAX  (English version)</t>
+        </is>
+      </c>
+      <c r="E836" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F836" t="n">
+        <v>21</v>
+      </c>
+      <c r="G836" t="n">
+        <v>28</v>
+      </c>
+      <c r="H836" t="inlineStr">
+        <is>
+          <t>21/28</t>
+        </is>
+      </c>
+      <c r="I836" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="J836" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K836" t="n">
+        <v>36298050</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K832"/>
+  <autoFilter ref="A1:K836"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-08-06)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$836</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$840</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K836"/>
+  <dimension ref="A1:K840"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -39767,8 +39767,196 @@
         <v>36298050</v>
       </c>
     </row>
+    <row r="837">
+      <c r="A837" s="2" t="n">
+        <v>46239</v>
+      </c>
+      <c r="B837" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C837" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D837" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E837" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F837" t="n">
+        <v>11</v>
+      </c>
+      <c r="G837" t="n">
+        <v>18</v>
+      </c>
+      <c r="H837" t="inlineStr">
+        <is>
+          <t>11/18</t>
+        </is>
+      </c>
+      <c r="I837" s="5" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="J837" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K837" t="n">
+        <v>36929295</v>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" s="2" t="n">
+        <v>46239</v>
+      </c>
+      <c r="B838" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C838" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D838" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E838" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F838" t="n">
+        <v>2</v>
+      </c>
+      <c r="G838" t="n">
+        <v>18</v>
+      </c>
+      <c r="H838" t="inlineStr">
+        <is>
+          <t>2/18</t>
+        </is>
+      </c>
+      <c r="I838" s="4" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="J838" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K838" t="n">
+        <v>36298344</v>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" s="2" t="n">
+        <v>46239</v>
+      </c>
+      <c r="B839" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C839" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D839" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E839" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F839" t="n">
+        <v>10</v>
+      </c>
+      <c r="G839" t="n">
+        <v>33</v>
+      </c>
+      <c r="H839" t="inlineStr">
+        <is>
+          <t>10/33</t>
+        </is>
+      </c>
+      <c r="I839" s="4" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="J839" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K839" t="n">
+        <v>36298385</v>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" s="2" t="n">
+        <v>46239</v>
+      </c>
+      <c r="B840" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C840" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D840" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E840" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F840" t="n">
+        <v>18</v>
+      </c>
+      <c r="G840" t="n">
+        <v>33</v>
+      </c>
+      <c r="H840" t="inlineStr">
+        <is>
+          <t>18/33</t>
+        </is>
+      </c>
+      <c r="I840" s="5" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="J840" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K840" t="n">
+        <v>36298582</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K836"/>
+  <autoFilter ref="A1:K840"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-08-07)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$840</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$844</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K840"/>
+  <dimension ref="A1:K844"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -39792,18 +39792,18 @@
         </is>
       </c>
       <c r="F837" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G837" t="n">
         <v>18</v>
       </c>
       <c r="H837" t="inlineStr">
         <is>
-          <t>11/18</t>
+          <t>10/18</t>
         </is>
       </c>
       <c r="I837" s="5" t="n">
-        <v>61.1</v>
+        <v>55.6</v>
       </c>
       <c r="J837" t="inlineStr">
         <is>
@@ -39955,8 +39955,196 @@
         <v>36298582</v>
       </c>
     </row>
+    <row r="841">
+      <c r="A841" s="2" t="n">
+        <v>46240</v>
+      </c>
+      <c r="B841" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C841" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D841" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E841" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F841" t="n">
+        <v>13</v>
+      </c>
+      <c r="G841" t="n">
+        <v>18</v>
+      </c>
+      <c r="H841" t="inlineStr">
+        <is>
+          <t>13/18</t>
+        </is>
+      </c>
+      <c r="I841" s="5" t="n">
+        <v>72.2</v>
+      </c>
+      <c r="J841" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K841" t="n">
+        <v>36929386</v>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" s="2" t="n">
+        <v>46240</v>
+      </c>
+      <c r="B842" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C842" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D842" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E842" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F842" t="n">
+        <v>9</v>
+      </c>
+      <c r="G842" t="n">
+        <v>18</v>
+      </c>
+      <c r="H842" t="inlineStr">
+        <is>
+          <t>9/18</t>
+        </is>
+      </c>
+      <c r="I842" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J842" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K842" t="n">
+        <v>36298759</v>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" s="2" t="n">
+        <v>46240</v>
+      </c>
+      <c r="B843" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C843" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D843" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E843" t="inlineStr">
+        <is>
+          <t>Faustine CHOPIN</t>
+        </is>
+      </c>
+      <c r="F843" t="n">
+        <v>33</v>
+      </c>
+      <c r="G843" t="n">
+        <v>33</v>
+      </c>
+      <c r="H843" t="inlineStr">
+        <is>
+          <t>33/33</t>
+        </is>
+      </c>
+      <c r="I843" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J843" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K843" t="n">
+        <v>36298813</v>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" s="2" t="n">
+        <v>46240</v>
+      </c>
+      <c r="B844" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C844" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D844" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E844" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F844" t="n">
+        <v>19</v>
+      </c>
+      <c r="G844" t="n">
+        <v>28</v>
+      </c>
+      <c r="H844" t="inlineStr">
+        <is>
+          <t>19/28</t>
+        </is>
+      </c>
+      <c r="I844" s="5" t="n">
+        <v>67.90000000000001</v>
+      </c>
+      <c r="J844" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K844" t="n">
+        <v>36298866</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K840"/>
+  <autoFilter ref="A1:K844"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-08-08)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$844</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$848</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K844"/>
+  <dimension ref="A1:K848"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -40143,8 +40143,196 @@
         <v>36298866</v>
       </c>
     </row>
+    <row r="845">
+      <c r="A845" s="2" t="n">
+        <v>46241</v>
+      </c>
+      <c r="B845" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C845" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D845" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E845" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F845" t="n">
+        <v>9</v>
+      </c>
+      <c r="G845" t="n">
+        <v>33</v>
+      </c>
+      <c r="H845" t="inlineStr">
+        <is>
+          <t>9/33</t>
+        </is>
+      </c>
+      <c r="I845" s="4" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="J845" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K845" t="n">
+        <v>36320783</v>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" s="2" t="n">
+        <v>46241</v>
+      </c>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C846" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D846" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E846" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F846" t="n">
+        <v>15</v>
+      </c>
+      <c r="G846" t="n">
+        <v>33</v>
+      </c>
+      <c r="H846" t="inlineStr">
+        <is>
+          <t>15/33</t>
+        </is>
+      </c>
+      <c r="I846" s="4" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="J846" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K846" t="n">
+        <v>36320893</v>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" s="2" t="n">
+        <v>46241</v>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C847" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D847" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E847" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F847" t="n">
+        <v>9</v>
+      </c>
+      <c r="G847" t="n">
+        <v>20</v>
+      </c>
+      <c r="H847" t="inlineStr">
+        <is>
+          <t>9/20</t>
+        </is>
+      </c>
+      <c r="I847" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="J847" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K847" t="n">
+        <v>36893830</v>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" s="2" t="n">
+        <v>46241</v>
+      </c>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C848" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D848" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E848" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F848" t="n">
+        <v>5</v>
+      </c>
+      <c r="G848" t="n">
+        <v>20</v>
+      </c>
+      <c r="H848" t="inlineStr">
+        <is>
+          <t>5/20</t>
+        </is>
+      </c>
+      <c r="I848" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="J848" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K848" t="n">
+        <v>36893889</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K844"/>
+  <autoFilter ref="A1:K848"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-08-09)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$848</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$852</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K848"/>
+  <dimension ref="A1:K852"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -40331,8 +40331,196 @@
         <v>36893889</v>
       </c>
     </row>
+    <row r="849">
+      <c r="A849" s="2" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="D849" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E849" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F849" t="n">
+        <v>8</v>
+      </c>
+      <c r="G849" t="n">
+        <v>32</v>
+      </c>
+      <c r="H849" t="inlineStr">
+        <is>
+          <t>8/32</t>
+        </is>
+      </c>
+      <c r="I849" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="J849" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K849" t="n">
+        <v>36323277</v>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" s="2" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="D850" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E850" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F850" t="n">
+        <v>9</v>
+      </c>
+      <c r="G850" t="n">
+        <v>32</v>
+      </c>
+      <c r="H850" t="inlineStr">
+        <is>
+          <t>9/32</t>
+        </is>
+      </c>
+      <c r="I850" s="4" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="J850" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K850" t="n">
+        <v>38771775</v>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" s="2" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C851" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D851" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E851" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F851" t="n">
+        <v>13</v>
+      </c>
+      <c r="G851" t="n">
+        <v>33</v>
+      </c>
+      <c r="H851" t="inlineStr">
+        <is>
+          <t>13/33</t>
+        </is>
+      </c>
+      <c r="I851" s="4" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="J851" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K851" t="n">
+        <v>36329205</v>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" s="2" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B852" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C852" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="D852" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E852" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F852" t="n">
+        <v>18</v>
+      </c>
+      <c r="G852" t="n">
+        <v>33</v>
+      </c>
+      <c r="H852" t="inlineStr">
+        <is>
+          <t>18/33</t>
+        </is>
+      </c>
+      <c r="I852" s="5" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="J852" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K852" t="n">
+        <v>36329970</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K848"/>
+  <autoFilter ref="A1:K852"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-08-10)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$852</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$857</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K852"/>
+  <dimension ref="A1:K857"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -40168,18 +40168,18 @@
         </is>
       </c>
       <c r="F845" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G845" t="n">
         <v>33</v>
       </c>
       <c r="H845" t="inlineStr">
         <is>
-          <t>9/33</t>
+          <t>8/33</t>
         </is>
       </c>
       <c r="I845" s="4" t="n">
-        <v>27.3</v>
+        <v>24.2</v>
       </c>
       <c r="J845" t="inlineStr">
         <is>
@@ -40519,8 +40519,243 @@
         <v>36329970</v>
       </c>
     </row>
+    <row r="853">
+      <c r="A853" s="2" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C853" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="D853" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E853" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F853" t="n">
+        <v>2</v>
+      </c>
+      <c r="G853" t="n">
+        <v>33</v>
+      </c>
+      <c r="H853" t="inlineStr">
+        <is>
+          <t>2/33</t>
+        </is>
+      </c>
+      <c r="I853" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="J853" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K853" t="n">
+        <v>36336033</v>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" s="2" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C854" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D854" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E854" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F854" t="n">
+        <v>9</v>
+      </c>
+      <c r="G854" t="n">
+        <v>28</v>
+      </c>
+      <c r="H854" t="inlineStr">
+        <is>
+          <t>9/28</t>
+        </is>
+      </c>
+      <c r="I854" s="4" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="J854" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K854" t="n">
+        <v>37240430</v>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" s="2" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C855" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D855" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E855" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F855" t="n">
+        <v>14</v>
+      </c>
+      <c r="G855" t="n">
+        <v>28</v>
+      </c>
+      <c r="H855" t="inlineStr">
+        <is>
+          <t>14/28</t>
+        </is>
+      </c>
+      <c r="I855" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J855" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K855" t="n">
+        <v>36892147</v>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" s="2" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C856" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D856" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E856" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F856" t="n">
+        <v>14</v>
+      </c>
+      <c r="G856" t="n">
+        <v>33</v>
+      </c>
+      <c r="H856" t="inlineStr">
+        <is>
+          <t>14/33</t>
+        </is>
+      </c>
+      <c r="I856" s="4" t="n">
+        <v>42.4</v>
+      </c>
+      <c r="J856" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K856" t="n">
+        <v>36336248</v>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" s="2" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C857" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="D857" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E857" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F857" t="n">
+        <v>25</v>
+      </c>
+      <c r="G857" t="n">
+        <v>33</v>
+      </c>
+      <c r="H857" t="inlineStr">
+        <is>
+          <t>25/33</t>
+        </is>
+      </c>
+      <c r="I857" s="5" t="n">
+        <v>75.8</v>
+      </c>
+      <c r="J857" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K857" t="n">
+        <v>36692760</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K852"/>
+  <autoFilter ref="A1:K857"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-08-11)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$857</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$864</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K857"/>
+  <dimension ref="A1:K864"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -40754,8 +40754,337 @@
         <v>36692760</v>
       </c>
     </row>
+    <row r="858">
+      <c r="A858" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C858" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D858" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E858" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F858" t="n">
+        <v>0</v>
+      </c>
+      <c r="G858" t="n">
+        <v>28</v>
+      </c>
+      <c r="H858" t="inlineStr">
+        <is>
+          <t>0/28</t>
+        </is>
+      </c>
+      <c r="I858" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J858" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K858" t="n">
+        <v>36390334</v>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B859" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C859" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D859" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E859" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F859" t="n">
+        <v>0</v>
+      </c>
+      <c r="G859" t="n">
+        <v>28</v>
+      </c>
+      <c r="H859" t="inlineStr">
+        <is>
+          <t>0/28</t>
+        </is>
+      </c>
+      <c r="I859" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J859" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K859" t="n">
+        <v>36281137</v>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C860" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D860" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E860" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F860" t="n">
+        <v>0</v>
+      </c>
+      <c r="G860" t="n">
+        <v>18</v>
+      </c>
+      <c r="H860" t="inlineStr">
+        <is>
+          <t>0/18</t>
+        </is>
+      </c>
+      <c r="I860" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J860" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K860" t="n">
+        <v>38531913</v>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C861" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D861" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E861" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F861" t="n">
+        <v>0</v>
+      </c>
+      <c r="G861" t="n">
+        <v>18</v>
+      </c>
+      <c r="H861" t="inlineStr">
+        <is>
+          <t>0/18</t>
+        </is>
+      </c>
+      <c r="I861" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J861" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K861" t="n">
+        <v>36928732</v>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C862" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D862" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E862" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F862" t="n">
+        <v>0</v>
+      </c>
+      <c r="G862" t="n">
+        <v>28</v>
+      </c>
+      <c r="H862" t="inlineStr">
+        <is>
+          <t>0/28</t>
+        </is>
+      </c>
+      <c r="I862" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J862" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K862" t="n">
+        <v>36281001</v>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C863" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="D863" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E863" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F863" t="n">
+        <v>0</v>
+      </c>
+      <c r="G863" t="n">
+        <v>28</v>
+      </c>
+      <c r="H863" t="inlineStr">
+        <is>
+          <t>0/28</t>
+        </is>
+      </c>
+      <c r="I863" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J863" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K863" t="n">
+        <v>37873143</v>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C864" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D864" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E864" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F864" t="n">
+        <v>0</v>
+      </c>
+      <c r="G864" t="n">
+        <v>32</v>
+      </c>
+      <c r="H864" t="inlineStr">
+        <is>
+          <t>0/32</t>
+        </is>
+      </c>
+      <c r="I864" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J864" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K864" t="n">
+        <v>36929038</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K857"/>
+  <autoFilter ref="A1:K864"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-08-12)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$864</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$869</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K864"/>
+  <dimension ref="A1:K869"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -41083,8 +41083,243 @@
         <v>36929038</v>
       </c>
     </row>
+    <row r="865">
+      <c r="A865" s="2" t="n">
+        <v>46245</v>
+      </c>
+      <c r="B865" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C865" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D865" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E865" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F865" t="n">
+        <v>0</v>
+      </c>
+      <c r="G865" t="n">
+        <v>33</v>
+      </c>
+      <c r="H865" t="inlineStr">
+        <is>
+          <t>0/33</t>
+        </is>
+      </c>
+      <c r="I865" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J865" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K865" t="n">
+        <v>36321365</v>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" s="2" t="n">
+        <v>46245</v>
+      </c>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C866" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D866" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E866" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F866" t="n">
+        <v>0</v>
+      </c>
+      <c r="G866" t="n">
+        <v>18</v>
+      </c>
+      <c r="H866" t="inlineStr">
+        <is>
+          <t>0/18</t>
+        </is>
+      </c>
+      <c r="I866" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J866" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K866" t="n">
+        <v>36929164</v>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" s="2" t="n">
+        <v>46245</v>
+      </c>
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C867" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D867" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E867" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F867" t="n">
+        <v>0</v>
+      </c>
+      <c r="G867" t="n">
+        <v>18</v>
+      </c>
+      <c r="H867" t="inlineStr">
+        <is>
+          <t>0/18</t>
+        </is>
+      </c>
+      <c r="I867" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J867" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K867" t="n">
+        <v>36298244</v>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" s="2" t="n">
+        <v>46245</v>
+      </c>
+      <c r="B868" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C868" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D868" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E868" t="inlineStr">
+        <is>
+          <t>Faustine CHOPIN</t>
+        </is>
+      </c>
+      <c r="F868" t="n">
+        <v>0</v>
+      </c>
+      <c r="G868" t="n">
+        <v>28</v>
+      </c>
+      <c r="H868" t="inlineStr">
+        <is>
+          <t>0/28</t>
+        </is>
+      </c>
+      <c r="I868" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J868" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K868" t="n">
+        <v>36297689</v>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" s="2" t="n">
+        <v>46245</v>
+      </c>
+      <c r="B869" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C869" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="D869" t="inlineStr">
+        <is>
+          <t>RE-LAX  (English version)</t>
+        </is>
+      </c>
+      <c r="E869" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F869" t="n">
+        <v>0</v>
+      </c>
+      <c r="G869" t="n">
+        <v>28</v>
+      </c>
+      <c r="H869" t="inlineStr">
+        <is>
+          <t>0/28</t>
+        </is>
+      </c>
+      <c r="I869" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J869" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K869" t="n">
+        <v>36298051</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K864"/>
+  <autoFilter ref="A1:K869"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-08-13)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$869</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$874</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K869"/>
+  <dimension ref="A1:K874"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -41318,8 +41318,243 @@
         <v>36298051</v>
       </c>
     </row>
+    <row r="870">
+      <c r="A870" s="2" t="n">
+        <v>46246</v>
+      </c>
+      <c r="B870" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C870" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D870" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E870" t="inlineStr">
+        <is>
+          <t>Alice Dunoyer</t>
+        </is>
+      </c>
+      <c r="F870" t="n">
+        <v>0</v>
+      </c>
+      <c r="G870" t="n">
+        <v>33</v>
+      </c>
+      <c r="H870" t="inlineStr">
+        <is>
+          <t>0/33</t>
+        </is>
+      </c>
+      <c r="I870" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J870" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K870" t="n">
+        <v>36321414</v>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" s="2" t="n">
+        <v>46246</v>
+      </c>
+      <c r="B871" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C871" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D871" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E871" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F871" t="n">
+        <v>0</v>
+      </c>
+      <c r="G871" t="n">
+        <v>18</v>
+      </c>
+      <c r="H871" t="inlineStr">
+        <is>
+          <t>0/18</t>
+        </is>
+      </c>
+      <c r="I871" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J871" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K871" t="n">
+        <v>36929296</v>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" s="2" t="n">
+        <v>46246</v>
+      </c>
+      <c r="B872" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C872" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D872" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E872" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F872" t="n">
+        <v>0</v>
+      </c>
+      <c r="G872" t="n">
+        <v>18</v>
+      </c>
+      <c r="H872" t="inlineStr">
+        <is>
+          <t>0/18</t>
+        </is>
+      </c>
+      <c r="I872" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J872" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K872" t="n">
+        <v>36298345</v>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" s="2" t="n">
+        <v>46246</v>
+      </c>
+      <c r="B873" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C873" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D873" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E873" t="inlineStr">
+        <is>
+          <t>Pauline Ramon</t>
+        </is>
+      </c>
+      <c r="F873" t="n">
+        <v>0</v>
+      </c>
+      <c r="G873" t="n">
+        <v>33</v>
+      </c>
+      <c r="H873" t="inlineStr">
+        <is>
+          <t>0/33</t>
+        </is>
+      </c>
+      <c r="I873" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J873" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K873" t="n">
+        <v>36298386</v>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" s="2" t="n">
+        <v>46246</v>
+      </c>
+      <c r="B874" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C874" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D874" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E874" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F874" t="n">
+        <v>0</v>
+      </c>
+      <c r="G874" t="n">
+        <v>33</v>
+      </c>
+      <c r="H874" t="inlineStr">
+        <is>
+          <t>0/33</t>
+        </is>
+      </c>
+      <c r="I874" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J874" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K874" t="n">
+        <v>36298583</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K869"/>
+  <autoFilter ref="A1:K874"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-08-14)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$874</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$883</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K874"/>
+  <dimension ref="A1:K883"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -41553,8 +41553,431 @@
         <v>36298583</v>
       </c>
     </row>
+    <row r="875">
+      <c r="A875" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="B875" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C875" t="inlineStr">
+        <is>
+          <t>07:45</t>
+        </is>
+      </c>
+      <c r="D875" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E875" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F875" t="n">
+        <v>0</v>
+      </c>
+      <c r="G875" t="n">
+        <v>28</v>
+      </c>
+      <c r="H875" t="inlineStr">
+        <is>
+          <t>0/28</t>
+        </is>
+      </c>
+      <c r="I875" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J875" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K875" t="n">
+        <v>37090010</v>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="B876" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C876" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D876" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E876" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F876" t="n">
+        <v>0</v>
+      </c>
+      <c r="G876" t="n">
+        <v>13</v>
+      </c>
+      <c r="H876" t="inlineStr">
+        <is>
+          <t>0/13</t>
+        </is>
+      </c>
+      <c r="I876" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J876" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K876" t="n">
+        <v>37230118</v>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="B877" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C877" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="D877" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E877" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F877" t="n">
+        <v>0</v>
+      </c>
+      <c r="G877" t="n">
+        <v>13</v>
+      </c>
+      <c r="H877" t="inlineStr">
+        <is>
+          <t>0/13</t>
+        </is>
+      </c>
+      <c r="I877" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J877" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K877" t="n">
+        <v>37230154</v>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="B878" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C878" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D878" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E878" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F878" t="n">
+        <v>0</v>
+      </c>
+      <c r="G878" t="n">
+        <v>13</v>
+      </c>
+      <c r="H878" t="inlineStr">
+        <is>
+          <t>0/13</t>
+        </is>
+      </c>
+      <c r="I878" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J878" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K878" t="n">
+        <v>37090968</v>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="B879" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C879" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D879" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E879" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F879" t="n">
+        <v>0</v>
+      </c>
+      <c r="G879" t="n">
+        <v>33</v>
+      </c>
+      <c r="H879" t="inlineStr">
+        <is>
+          <t>0/33</t>
+        </is>
+      </c>
+      <c r="I879" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J879" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K879" t="n">
+        <v>36321565</v>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="B880" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C880" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D880" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E880" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F880" t="n">
+        <v>0</v>
+      </c>
+      <c r="G880" t="n">
+        <v>18</v>
+      </c>
+      <c r="H880" t="inlineStr">
+        <is>
+          <t>0/18</t>
+        </is>
+      </c>
+      <c r="I880" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J880" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K880" t="n">
+        <v>36929387</v>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="B881" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C881" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D881" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E881" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F881" t="n">
+        <v>0</v>
+      </c>
+      <c r="G881" t="n">
+        <v>18</v>
+      </c>
+      <c r="H881" t="inlineStr">
+        <is>
+          <t>0/18</t>
+        </is>
+      </c>
+      <c r="I881" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J881" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K881" t="n">
+        <v>36298760</v>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="B882" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C882" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D882" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E882" t="inlineStr">
+        <is>
+          <t>Faustine CHOPIN</t>
+        </is>
+      </c>
+      <c r="F882" t="n">
+        <v>0</v>
+      </c>
+      <c r="G882" t="n">
+        <v>33</v>
+      </c>
+      <c r="H882" t="inlineStr">
+        <is>
+          <t>0/33</t>
+        </is>
+      </c>
+      <c r="I882" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J882" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K882" t="n">
+        <v>36298814</v>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="B883" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C883" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D883" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E883" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F883" t="n">
+        <v>0</v>
+      </c>
+      <c r="G883" t="n">
+        <v>33</v>
+      </c>
+      <c r="H883" t="inlineStr">
+        <is>
+          <t>0/33</t>
+        </is>
+      </c>
+      <c r="I883" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J883" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K883" t="n">
+        <v>36298867</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K874"/>
+  <autoFilter ref="A1:K883"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-08-15)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$883</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$890</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K883"/>
+  <dimension ref="A1:K890"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -41976,8 +41976,337 @@
         <v>36298867</v>
       </c>
     </row>
+    <row r="884">
+      <c r="A884" s="2" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B884" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C884" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D884" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E884" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F884" t="n">
+        <v>0</v>
+      </c>
+      <c r="G884" t="n">
+        <v>33</v>
+      </c>
+      <c r="H884" t="inlineStr">
+        <is>
+          <t>0/33</t>
+        </is>
+      </c>
+      <c r="I884" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J884" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K884" t="n">
+        <v>36319503</v>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" s="2" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B885" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C885" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D885" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E885" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F885" t="n">
+        <v>0</v>
+      </c>
+      <c r="G885" t="n">
+        <v>16</v>
+      </c>
+      <c r="H885" t="inlineStr">
+        <is>
+          <t>0/16</t>
+        </is>
+      </c>
+      <c r="I885" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J885" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K885" t="n">
+        <v>36320661</v>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" s="2" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B886" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C886" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D886" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E886" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F886" t="n">
+        <v>0</v>
+      </c>
+      <c r="G886" t="n">
+        <v>16</v>
+      </c>
+      <c r="H886" t="inlineStr">
+        <is>
+          <t>0/16</t>
+        </is>
+      </c>
+      <c r="I886" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J886" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K886" t="n">
+        <v>36320060</v>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" s="2" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B887" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C887" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D887" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E887" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F887" t="n">
+        <v>0</v>
+      </c>
+      <c r="G887" t="n">
+        <v>33</v>
+      </c>
+      <c r="H887" t="inlineStr">
+        <is>
+          <t>0/33</t>
+        </is>
+      </c>
+      <c r="I887" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J887" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K887" t="n">
+        <v>36320784</v>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" s="2" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B888" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C888" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D888" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E888" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F888" t="n">
+        <v>0</v>
+      </c>
+      <c r="G888" t="n">
+        <v>33</v>
+      </c>
+      <c r="H888" t="inlineStr">
+        <is>
+          <t>0/33</t>
+        </is>
+      </c>
+      <c r="I888" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J888" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K888" t="n">
+        <v>36320894</v>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" s="2" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B889" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C889" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D889" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E889" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F889" t="n">
+        <v>0</v>
+      </c>
+      <c r="G889" t="n">
+        <v>20</v>
+      </c>
+      <c r="H889" t="inlineStr">
+        <is>
+          <t>0/20</t>
+        </is>
+      </c>
+      <c r="I889" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J889" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K889" t="n">
+        <v>36893831</v>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" s="2" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B890" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C890" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D890" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E890" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F890" t="n">
+        <v>0</v>
+      </c>
+      <c r="G890" t="n">
+        <v>20</v>
+      </c>
+      <c r="H890" t="inlineStr">
+        <is>
+          <t>0/20</t>
+        </is>
+      </c>
+      <c r="I890" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J890" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K890" t="n">
+        <v>36893891</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K883"/>
+  <autoFilter ref="A1:K890"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-08-16)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$890</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$898</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K890"/>
+  <dimension ref="A1:K898"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -42305,8 +42305,384 @@
         <v>36893891</v>
       </c>
     </row>
+    <row r="891">
+      <c r="A891" s="2" t="n">
+        <v>46249</v>
+      </c>
+      <c r="B891" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C891" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D891" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E891" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F891" t="n">
+        <v>0</v>
+      </c>
+      <c r="G891" t="n">
+        <v>32</v>
+      </c>
+      <c r="H891" t="inlineStr">
+        <is>
+          <t>0/32</t>
+        </is>
+      </c>
+      <c r="I891" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J891" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K891" t="n">
+        <v>36323278</v>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" s="2" t="n">
+        <v>46249</v>
+      </c>
+      <c r="B892" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C892" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D892" t="inlineStr">
+        <is>
+          <t>RE-BOOST  (English version)</t>
+        </is>
+      </c>
+      <c r="E892" t="inlineStr">
+        <is>
+          <t>Alice Dunoyer</t>
+        </is>
+      </c>
+      <c r="F892" t="n">
+        <v>0</v>
+      </c>
+      <c r="G892" t="n">
+        <v>33</v>
+      </c>
+      <c r="H892" t="inlineStr">
+        <is>
+          <t>0/33</t>
+        </is>
+      </c>
+      <c r="I892" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J892" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K892" t="n">
+        <v>36323124</v>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" s="2" t="n">
+        <v>46249</v>
+      </c>
+      <c r="B893" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C893" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D893" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E893" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F893" t="n">
+        <v>0</v>
+      </c>
+      <c r="G893" t="n">
+        <v>32</v>
+      </c>
+      <c r="H893" t="inlineStr">
+        <is>
+          <t>0/32</t>
+        </is>
+      </c>
+      <c r="I893" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J893" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K893" t="n">
+        <v>38771776</v>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" s="2" t="n">
+        <v>46249</v>
+      </c>
+      <c r="B894" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C894" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D894" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E894" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F894" t="n">
+        <v>0</v>
+      </c>
+      <c r="G894" t="n">
+        <v>33</v>
+      </c>
+      <c r="H894" t="inlineStr">
+        <is>
+          <t>0/33</t>
+        </is>
+      </c>
+      <c r="I894" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J894" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K894" t="n">
+        <v>36329206</v>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" s="2" t="n">
+        <v>46249</v>
+      </c>
+      <c r="B895" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C895" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="D895" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E895" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F895" t="n">
+        <v>0</v>
+      </c>
+      <c r="G895" t="n">
+        <v>32</v>
+      </c>
+      <c r="H895" t="inlineStr">
+        <is>
+          <t>0/32</t>
+        </is>
+      </c>
+      <c r="I895" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J895" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K895" t="n">
+        <v>38771876</v>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" s="2" t="n">
+        <v>46249</v>
+      </c>
+      <c r="B896" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C896" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D896" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E896" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F896" t="n">
+        <v>0</v>
+      </c>
+      <c r="G896" t="n">
+        <v>33</v>
+      </c>
+      <c r="H896" t="inlineStr">
+        <is>
+          <t>0/33</t>
+        </is>
+      </c>
+      <c r="I896" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J896" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K896" t="n">
+        <v>36329971</v>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" s="2" t="n">
+        <v>46249</v>
+      </c>
+      <c r="B897" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C897" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D897" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E897" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F897" t="n">
+        <v>0</v>
+      </c>
+      <c r="G897" t="n">
+        <v>20</v>
+      </c>
+      <c r="H897" t="inlineStr">
+        <is>
+          <t>0/20</t>
+        </is>
+      </c>
+      <c r="I897" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J897" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K897" t="n">
+        <v>36935878</v>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" s="2" t="n">
+        <v>46249</v>
+      </c>
+      <c r="B898" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C898" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="D898" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E898" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F898" t="n">
+        <v>0</v>
+      </c>
+      <c r="G898" t="n">
+        <v>20</v>
+      </c>
+      <c r="H898" t="inlineStr">
+        <is>
+          <t>0/20</t>
+        </is>
+      </c>
+      <c r="I898" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J898" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K898" t="n">
+        <v>36323863</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K890"/>
+  <autoFilter ref="A1:K898"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-08-17)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$898</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$905</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K898"/>
+  <dimension ref="A1:K905"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -42681,8 +42681,337 @@
         <v>36323863</v>
       </c>
     </row>
+    <row r="899">
+      <c r="A899" s="2" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B899" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C899" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D899" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E899" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F899" t="n">
+        <v>0</v>
+      </c>
+      <c r="G899" t="n">
+        <v>36</v>
+      </c>
+      <c r="H899" t="inlineStr">
+        <is>
+          <t>0/36</t>
+        </is>
+      </c>
+      <c r="I899" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J899" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K899" t="n">
+        <v>37240288</v>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" s="2" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B900" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C900" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D900" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E900" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F900" t="n">
+        <v>0</v>
+      </c>
+      <c r="G900" t="n">
+        <v>33</v>
+      </c>
+      <c r="H900" t="inlineStr">
+        <is>
+          <t>0/33</t>
+        </is>
+      </c>
+      <c r="I900" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J900" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K900" t="n">
+        <v>36336034</v>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" s="2" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B901" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C901" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D901" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E901" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F901" t="n">
+        <v>0</v>
+      </c>
+      <c r="G901" t="n">
+        <v>28</v>
+      </c>
+      <c r="H901" t="inlineStr">
+        <is>
+          <t>0/28</t>
+        </is>
+      </c>
+      <c r="I901" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J901" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K901" t="n">
+        <v>37240431</v>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" s="2" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B902" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C902" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D902" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E902" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F902" t="n">
+        <v>0</v>
+      </c>
+      <c r="G902" t="n">
+        <v>28</v>
+      </c>
+      <c r="H902" t="inlineStr">
+        <is>
+          <t>0/28</t>
+        </is>
+      </c>
+      <c r="I902" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J902" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K902" t="n">
+        <v>36892148</v>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" s="2" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B903" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C903" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="D903" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E903" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F903" t="n">
+        <v>0</v>
+      </c>
+      <c r="G903" t="n">
+        <v>33</v>
+      </c>
+      <c r="H903" t="inlineStr">
+        <is>
+          <t>0/33</t>
+        </is>
+      </c>
+      <c r="I903" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J903" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K903" t="n">
+        <v>36336249</v>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" s="2" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B904" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C904" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="D904" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E904" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F904" t="n">
+        <v>0</v>
+      </c>
+      <c r="G904" t="n">
+        <v>33</v>
+      </c>
+      <c r="H904" t="inlineStr">
+        <is>
+          <t>0/33</t>
+        </is>
+      </c>
+      <c r="I904" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J904" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K904" t="n">
+        <v>36692761</v>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" s="2" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B905" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C905" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="D905" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E905" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F905" t="n">
+        <v>0</v>
+      </c>
+      <c r="G905" t="n">
+        <v>36</v>
+      </c>
+      <c r="H905" t="inlineStr">
+        <is>
+          <t>0/36</t>
+        </is>
+      </c>
+      <c r="I905" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J905" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K905" t="n">
+        <v>36892103</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K898"/>
+  <autoFilter ref="A1:K905"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-08-18)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$905</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$909</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K905"/>
+  <dimension ref="A1:K909"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -43010,8 +43010,196 @@
         <v>36892103</v>
       </c>
     </row>
+    <row r="906">
+      <c r="A906" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="B906" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C906" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D906" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E906" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F906" t="n">
+        <v>9</v>
+      </c>
+      <c r="G906" t="n">
+        <v>18</v>
+      </c>
+      <c r="H906" t="inlineStr">
+        <is>
+          <t>9/18</t>
+        </is>
+      </c>
+      <c r="I906" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J906" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K906" t="n">
+        <v>36928733</v>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="B907" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C907" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D907" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E907" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F907" t="n">
+        <v>8</v>
+      </c>
+      <c r="G907" t="n">
+        <v>18</v>
+      </c>
+      <c r="H907" t="inlineStr">
+        <is>
+          <t>8/18</t>
+        </is>
+      </c>
+      <c r="I907" s="4" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="J907" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K907" t="n">
+        <v>38531914</v>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="B908" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C908" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D908" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E908" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F908" t="n">
+        <v>20</v>
+      </c>
+      <c r="G908" t="n">
+        <v>33</v>
+      </c>
+      <c r="H908" t="inlineStr">
+        <is>
+          <t>20/33</t>
+        </is>
+      </c>
+      <c r="I908" s="5" t="n">
+        <v>60.6</v>
+      </c>
+      <c r="J908" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K908" t="n">
+        <v>36281002</v>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="B909" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C909" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D909" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E909" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F909" t="n">
+        <v>26</v>
+      </c>
+      <c r="G909" t="n">
+        <v>32</v>
+      </c>
+      <c r="H909" t="inlineStr">
+        <is>
+          <t>26/32</t>
+        </is>
+      </c>
+      <c r="I909" s="5" t="n">
+        <v>81.2</v>
+      </c>
+      <c r="J909" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K909" t="n">
+        <v>36929039</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K905"/>
+  <autoFilter ref="A1:K909"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-08-19)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$909</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$913</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K909"/>
+  <dimension ref="A1:K913"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -43198,8 +43198,196 @@
         <v>36929039</v>
       </c>
     </row>
+    <row r="910">
+      <c r="A910" s="2" t="n">
+        <v>46252</v>
+      </c>
+      <c r="B910" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C910" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D910" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E910" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F910" t="n">
+        <v>4</v>
+      </c>
+      <c r="G910" t="n">
+        <v>18</v>
+      </c>
+      <c r="H910" t="inlineStr">
+        <is>
+          <t>4/18</t>
+        </is>
+      </c>
+      <c r="I910" s="4" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="J910" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K910" t="n">
+        <v>36298245</v>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" s="2" t="n">
+        <v>46252</v>
+      </c>
+      <c r="B911" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C911" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D911" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E911" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F911" t="n">
+        <v>8</v>
+      </c>
+      <c r="G911" t="n">
+        <v>18</v>
+      </c>
+      <c r="H911" t="inlineStr">
+        <is>
+          <t>8/18</t>
+        </is>
+      </c>
+      <c r="I911" s="4" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="J911" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K911" t="n">
+        <v>36929165</v>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" s="2" t="n">
+        <v>46252</v>
+      </c>
+      <c r="B912" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C912" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D912" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E912" t="inlineStr">
+        <is>
+          <t>Faustine CHOPIN</t>
+        </is>
+      </c>
+      <c r="F912" t="n">
+        <v>26</v>
+      </c>
+      <c r="G912" t="n">
+        <v>33</v>
+      </c>
+      <c r="H912" t="inlineStr">
+        <is>
+          <t>26/33</t>
+        </is>
+      </c>
+      <c r="I912" s="5" t="n">
+        <v>78.8</v>
+      </c>
+      <c r="J912" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K912" t="n">
+        <v>36297690</v>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" s="2" t="n">
+        <v>46252</v>
+      </c>
+      <c r="B913" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C913" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D913" t="inlineStr">
+        <is>
+          <t>RE-LAX  (English version)</t>
+        </is>
+      </c>
+      <c r="E913" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F913" t="n">
+        <v>12</v>
+      </c>
+      <c r="G913" t="n">
+        <v>33</v>
+      </c>
+      <c r="H913" t="inlineStr">
+        <is>
+          <t>12/33</t>
+        </is>
+      </c>
+      <c r="I913" s="4" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="J913" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K913" t="n">
+        <v>36298052</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K909"/>
+  <autoFilter ref="A1:K913"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-08-20)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$913</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$917</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K913"/>
+  <dimension ref="A1:K917"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -43386,8 +43386,196 @@
         <v>36298052</v>
       </c>
     </row>
+    <row r="914">
+      <c r="A914" s="2" t="n">
+        <v>46253</v>
+      </c>
+      <c r="B914" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C914" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D914" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E914" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F914" t="n">
+        <v>12</v>
+      </c>
+      <c r="G914" t="n">
+        <v>18</v>
+      </c>
+      <c r="H914" t="inlineStr">
+        <is>
+          <t>12/18</t>
+        </is>
+      </c>
+      <c r="I914" s="5" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J914" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K914" t="n">
+        <v>36929297</v>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" s="2" t="n">
+        <v>46253</v>
+      </c>
+      <c r="B915" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C915" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D915" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E915" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F915" t="n">
+        <v>7</v>
+      </c>
+      <c r="G915" t="n">
+        <v>18</v>
+      </c>
+      <c r="H915" t="inlineStr">
+        <is>
+          <t>7/18</t>
+        </is>
+      </c>
+      <c r="I915" s="4" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="J915" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K915" t="n">
+        <v>36298346</v>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" s="2" t="n">
+        <v>46253</v>
+      </c>
+      <c r="B916" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C916" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D916" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E916" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F916" t="n">
+        <v>21</v>
+      </c>
+      <c r="G916" t="n">
+        <v>32</v>
+      </c>
+      <c r="H916" t="inlineStr">
+        <is>
+          <t>21/32</t>
+        </is>
+      </c>
+      <c r="I916" s="5" t="n">
+        <v>65.59999999999999</v>
+      </c>
+      <c r="J916" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K916" t="n">
+        <v>36298387</v>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" s="2" t="n">
+        <v>46253</v>
+      </c>
+      <c r="B917" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C917" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D917" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E917" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F917" t="n">
+        <v>21</v>
+      </c>
+      <c r="G917" t="n">
+        <v>33</v>
+      </c>
+      <c r="H917" t="inlineStr">
+        <is>
+          <t>21/33</t>
+        </is>
+      </c>
+      <c r="I917" s="5" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="J917" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K917" t="n">
+        <v>36298584</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K913"/>
+  <autoFilter ref="A1:K917"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-08-21)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$917</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$921</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K917"/>
+  <dimension ref="A1:K921"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -43458,18 +43458,18 @@
         </is>
       </c>
       <c r="F915" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G915" t="n">
         <v>18</v>
       </c>
       <c r="H915" t="inlineStr">
         <is>
-          <t>7/18</t>
+          <t>6/18</t>
         </is>
       </c>
       <c r="I915" s="4" t="n">
-        <v>38.9</v>
+        <v>33.3</v>
       </c>
       <c r="J915" t="inlineStr">
         <is>
@@ -43574,8 +43574,196 @@
         <v>36298584</v>
       </c>
     </row>
+    <row r="918">
+      <c r="A918" s="2" t="n">
+        <v>46254</v>
+      </c>
+      <c r="B918" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C918" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D918" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E918" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F918" t="n">
+        <v>9</v>
+      </c>
+      <c r="G918" t="n">
+        <v>18</v>
+      </c>
+      <c r="H918" t="inlineStr">
+        <is>
+          <t>9/18</t>
+        </is>
+      </c>
+      <c r="I918" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J918" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K918" t="n">
+        <v>36929388</v>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" s="2" t="n">
+        <v>46254</v>
+      </c>
+      <c r="B919" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C919" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D919" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E919" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F919" t="n">
+        <v>7</v>
+      </c>
+      <c r="G919" t="n">
+        <v>18</v>
+      </c>
+      <c r="H919" t="inlineStr">
+        <is>
+          <t>7/18</t>
+        </is>
+      </c>
+      <c r="I919" s="4" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="J919" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K919" t="n">
+        <v>36298761</v>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" s="2" t="n">
+        <v>46254</v>
+      </c>
+      <c r="B920" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C920" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D920" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E920" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F920" t="n">
+        <v>24</v>
+      </c>
+      <c r="G920" t="n">
+        <v>32</v>
+      </c>
+      <c r="H920" t="inlineStr">
+        <is>
+          <t>24/32</t>
+        </is>
+      </c>
+      <c r="I920" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="J920" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K920" t="n">
+        <v>36298815</v>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" s="2" t="n">
+        <v>46254</v>
+      </c>
+      <c r="B921" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C921" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D921" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E921" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F921" t="n">
+        <v>19</v>
+      </c>
+      <c r="G921" t="n">
+        <v>33</v>
+      </c>
+      <c r="H921" t="inlineStr">
+        <is>
+          <t>19/33</t>
+        </is>
+      </c>
+      <c r="I921" s="5" t="n">
+        <v>57.6</v>
+      </c>
+      <c r="J921" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K921" t="n">
+        <v>36298868</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K917"/>
+  <autoFilter ref="A1:K921"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-08-22)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$921</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$925</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K921"/>
+  <dimension ref="A1:K925"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -43505,18 +43505,18 @@
         </is>
       </c>
       <c r="F916" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G916" t="n">
         <v>32</v>
       </c>
       <c r="H916" t="inlineStr">
         <is>
-          <t>21/32</t>
+          <t>20/32</t>
         </is>
       </c>
       <c r="I916" s="5" t="n">
-        <v>65.59999999999999</v>
+        <v>62.5</v>
       </c>
       <c r="J916" t="inlineStr">
         <is>
@@ -43762,8 +43762,196 @@
         <v>36298868</v>
       </c>
     </row>
+    <row r="922">
+      <c r="A922" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B922" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C922" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D922" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E922" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F922" t="n">
+        <v>15</v>
+      </c>
+      <c r="G922" t="n">
+        <v>33</v>
+      </c>
+      <c r="H922" t="inlineStr">
+        <is>
+          <t>15/33</t>
+        </is>
+      </c>
+      <c r="I922" s="4" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="J922" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K922" t="n">
+        <v>36320785</v>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B923" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C923" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D923" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E923" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F923" t="n">
+        <v>31</v>
+      </c>
+      <c r="G923" t="n">
+        <v>33</v>
+      </c>
+      <c r="H923" t="inlineStr">
+        <is>
+          <t>31/33</t>
+        </is>
+      </c>
+      <c r="I923" s="3" t="n">
+        <v>93.90000000000001</v>
+      </c>
+      <c r="J923" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K923" t="n">
+        <v>36320895</v>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B924" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C924" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D924" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E924" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F924" t="n">
+        <v>13</v>
+      </c>
+      <c r="G924" t="n">
+        <v>20</v>
+      </c>
+      <c r="H924" t="inlineStr">
+        <is>
+          <t>13/20</t>
+        </is>
+      </c>
+      <c r="I924" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="J924" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K924" t="n">
+        <v>36893832</v>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B925" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C925" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D925" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E925" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F925" t="n">
+        <v>14</v>
+      </c>
+      <c r="G925" t="n">
+        <v>20</v>
+      </c>
+      <c r="H925" t="inlineStr">
+        <is>
+          <t>14/20</t>
+        </is>
+      </c>
+      <c r="I925" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="J925" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K925" t="n">
+        <v>36893894</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K921"/>
+  <autoFilter ref="A1:K925"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-08-23)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$925</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$931</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K925"/>
+  <dimension ref="A1:K931"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -43950,8 +43950,290 @@
         <v>36893894</v>
       </c>
     </row>
+    <row r="926">
+      <c r="A926" s="2" t="n">
+        <v>46256</v>
+      </c>
+      <c r="B926" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C926" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D926" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E926" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F926" t="n">
+        <v>4</v>
+      </c>
+      <c r="G926" t="n">
+        <v>32</v>
+      </c>
+      <c r="H926" t="inlineStr">
+        <is>
+          <t>4/32</t>
+        </is>
+      </c>
+      <c r="I926" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="J926" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K926" t="n">
+        <v>36323279</v>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" s="2" t="n">
+        <v>46256</v>
+      </c>
+      <c r="B927" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C927" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D927" t="inlineStr">
+        <is>
+          <t>RE-BOOST  (English version)</t>
+        </is>
+      </c>
+      <c r="E927" t="inlineStr">
+        <is>
+          <t>Alice Dunoyer</t>
+        </is>
+      </c>
+      <c r="F927" t="n">
+        <v>10</v>
+      </c>
+      <c r="G927" t="n">
+        <v>33</v>
+      </c>
+      <c r="H927" t="inlineStr">
+        <is>
+          <t>10/33</t>
+        </is>
+      </c>
+      <c r="I927" s="4" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="J927" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K927" t="n">
+        <v>36323125</v>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" s="2" t="n">
+        <v>46256</v>
+      </c>
+      <c r="B928" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C928" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D928" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E928" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F928" t="n">
+        <v>5</v>
+      </c>
+      <c r="G928" t="n">
+        <v>32</v>
+      </c>
+      <c r="H928" t="inlineStr">
+        <is>
+          <t>5/32</t>
+        </is>
+      </c>
+      <c r="I928" s="4" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="J928" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K928" t="n">
+        <v>38771777</v>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" s="2" t="n">
+        <v>46256</v>
+      </c>
+      <c r="B929" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C929" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D929" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E929" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F929" t="n">
+        <v>7</v>
+      </c>
+      <c r="G929" t="n">
+        <v>33</v>
+      </c>
+      <c r="H929" t="inlineStr">
+        <is>
+          <t>7/33</t>
+        </is>
+      </c>
+      <c r="I929" s="4" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="J929" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K929" t="n">
+        <v>36329207</v>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" s="2" t="n">
+        <v>46256</v>
+      </c>
+      <c r="B930" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C930" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="D930" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E930" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F930" t="n">
+        <v>22</v>
+      </c>
+      <c r="G930" t="n">
+        <v>32</v>
+      </c>
+      <c r="H930" t="inlineStr">
+        <is>
+          <t>22/32</t>
+        </is>
+      </c>
+      <c r="I930" s="5" t="n">
+        <v>68.8</v>
+      </c>
+      <c r="J930" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K930" t="n">
+        <v>38771877</v>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" s="2" t="n">
+        <v>46256</v>
+      </c>
+      <c r="B931" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C931" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D931" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E931" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F931" t="n">
+        <v>31</v>
+      </c>
+      <c r="G931" t="n">
+        <v>33</v>
+      </c>
+      <c r="H931" t="inlineStr">
+        <is>
+          <t>31/33</t>
+        </is>
+      </c>
+      <c r="I931" s="3" t="n">
+        <v>93.90000000000001</v>
+      </c>
+      <c r="J931" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K931" t="n">
+        <v>36329972</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K925"/>
+  <autoFilter ref="A1:K931"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-08-24)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$931</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$938</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K931"/>
+  <dimension ref="A1:K938"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -44232,8 +44232,337 @@
         <v>36329972</v>
       </c>
     </row>
+    <row r="932">
+      <c r="A932" s="2" t="n">
+        <v>46257</v>
+      </c>
+      <c r="B932" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C932" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D932" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E932" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F932" t="n">
+        <v>6</v>
+      </c>
+      <c r="G932" t="n">
+        <v>36</v>
+      </c>
+      <c r="H932" t="inlineStr">
+        <is>
+          <t>6/36</t>
+        </is>
+      </c>
+      <c r="I932" s="4" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="J932" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K932" t="n">
+        <v>37240289</v>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" s="2" t="n">
+        <v>46257</v>
+      </c>
+      <c r="B933" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C933" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D933" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E933" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F933" t="n">
+        <v>15</v>
+      </c>
+      <c r="G933" t="n">
+        <v>33</v>
+      </c>
+      <c r="H933" t="inlineStr">
+        <is>
+          <t>15/33</t>
+        </is>
+      </c>
+      <c r="I933" s="4" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="J933" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K933" t="n">
+        <v>36336035</v>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" s="2" t="n">
+        <v>46257</v>
+      </c>
+      <c r="B934" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C934" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D934" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E934" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F934" t="n">
+        <v>8</v>
+      </c>
+      <c r="G934" t="n">
+        <v>32</v>
+      </c>
+      <c r="H934" t="inlineStr">
+        <is>
+          <t>8/32</t>
+        </is>
+      </c>
+      <c r="I934" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="J934" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K934" t="n">
+        <v>37240432</v>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" s="2" t="n">
+        <v>46257</v>
+      </c>
+      <c r="B935" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C935" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="D935" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E935" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F935" t="n">
+        <v>19</v>
+      </c>
+      <c r="G935" t="n">
+        <v>28</v>
+      </c>
+      <c r="H935" t="inlineStr">
+        <is>
+          <t>19/28</t>
+        </is>
+      </c>
+      <c r="I935" s="5" t="n">
+        <v>67.90000000000001</v>
+      </c>
+      <c r="J935" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K935" t="n">
+        <v>36892149</v>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" s="2" t="n">
+        <v>46257</v>
+      </c>
+      <c r="B936" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C936" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="D936" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E936" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F936" t="n">
+        <v>34</v>
+      </c>
+      <c r="G936" t="n">
+        <v>33</v>
+      </c>
+      <c r="H936" t="inlineStr">
+        <is>
+          <t>34/33</t>
+        </is>
+      </c>
+      <c r="I936" s="3" t="n">
+        <v>103</v>
+      </c>
+      <c r="J936" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K936" t="n">
+        <v>36336250</v>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" s="2" t="n">
+        <v>46257</v>
+      </c>
+      <c r="B937" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C937" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="D937" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E937" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F937" t="n">
+        <v>32</v>
+      </c>
+      <c r="G937" t="n">
+        <v>33</v>
+      </c>
+      <c r="H937" t="inlineStr">
+        <is>
+          <t>32/33</t>
+        </is>
+      </c>
+      <c r="I937" s="3" t="n">
+        <v>97</v>
+      </c>
+      <c r="J937" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K937" t="n">
+        <v>36692762</v>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" s="2" t="n">
+        <v>46257</v>
+      </c>
+      <c r="B938" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C938" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="D938" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E938" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F938" t="n">
+        <v>19</v>
+      </c>
+      <c r="G938" t="n">
+        <v>36</v>
+      </c>
+      <c r="H938" t="inlineStr">
+        <is>
+          <t>19/36</t>
+        </is>
+      </c>
+      <c r="I938" s="5" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="J938" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K938" t="n">
+        <v>36892104</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K931"/>
+  <autoFilter ref="A1:K938"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-08-25)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$938</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$943</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K938"/>
+  <dimension ref="A1:K943"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -44561,8 +44561,243 @@
         <v>36892104</v>
       </c>
     </row>
+    <row r="939">
+      <c r="A939" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B939" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C939" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D939" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E939" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F939" t="n">
+        <v>8</v>
+      </c>
+      <c r="G939" t="n">
+        <v>28</v>
+      </c>
+      <c r="H939" t="inlineStr">
+        <is>
+          <t>8/28</t>
+        </is>
+      </c>
+      <c r="I939" s="4" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="J939" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K939" t="n">
+        <v>36390336</v>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B940" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C940" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D940" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E940" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F940" t="n">
+        <v>6</v>
+      </c>
+      <c r="G940" t="n">
+        <v>18</v>
+      </c>
+      <c r="H940" t="inlineStr">
+        <is>
+          <t>6/18</t>
+        </is>
+      </c>
+      <c r="I940" s="4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J940" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K940" t="n">
+        <v>36928734</v>
+      </c>
+    </row>
+    <row r="941">
+      <c r="A941" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B941" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C941" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D941" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E941" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F941" t="n">
+        <v>8</v>
+      </c>
+      <c r="G941" t="n">
+        <v>18</v>
+      </c>
+      <c r="H941" t="inlineStr">
+        <is>
+          <t>8/18</t>
+        </is>
+      </c>
+      <c r="I941" s="4" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="J941" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K941" t="n">
+        <v>38531915</v>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B942" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C942" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D942" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E942" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F942" t="n">
+        <v>15</v>
+      </c>
+      <c r="G942" t="n">
+        <v>33</v>
+      </c>
+      <c r="H942" t="inlineStr">
+        <is>
+          <t>15/33</t>
+        </is>
+      </c>
+      <c r="I942" s="4" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="J942" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K942" t="n">
+        <v>36281003</v>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B943" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C943" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D943" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E943" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F943" t="n">
+        <v>20</v>
+      </c>
+      <c r="G943" t="n">
+        <v>33</v>
+      </c>
+      <c r="H943" t="inlineStr">
+        <is>
+          <t>20/33</t>
+        </is>
+      </c>
+      <c r="I943" s="5" t="n">
+        <v>60.6</v>
+      </c>
+      <c r="J943" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K943" t="n">
+        <v>37873145</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K938"/>
+  <autoFilter ref="A1:K943"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-08-26)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$943</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$948</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K943"/>
+  <dimension ref="A1:K948"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -44796,8 +44796,243 @@
         <v>37873145</v>
       </c>
     </row>
+    <row r="944">
+      <c r="A944" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B944" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C944" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D944" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E944" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F944" t="n">
+        <v>15</v>
+      </c>
+      <c r="G944" t="n">
+        <v>33</v>
+      </c>
+      <c r="H944" t="inlineStr">
+        <is>
+          <t>15/33</t>
+        </is>
+      </c>
+      <c r="I944" s="4" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="J944" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K944" t="n">
+        <v>36321367</v>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B945" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C945" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D945" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E945" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F945" t="n">
+        <v>18</v>
+      </c>
+      <c r="G945" t="n">
+        <v>18</v>
+      </c>
+      <c r="H945" t="inlineStr">
+        <is>
+          <t>18/18</t>
+        </is>
+      </c>
+      <c r="I945" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J945" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K945" t="n">
+        <v>36298246</v>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B946" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C946" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D946" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E946" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F946" t="n">
+        <v>10</v>
+      </c>
+      <c r="G946" t="n">
+        <v>18</v>
+      </c>
+      <c r="H946" t="inlineStr">
+        <is>
+          <t>10/18</t>
+        </is>
+      </c>
+      <c r="I946" s="5" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="J946" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K946" t="n">
+        <v>36929166</v>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B947" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C947" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D947" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E947" t="inlineStr">
+        <is>
+          <t>Faustine CHOPIN</t>
+        </is>
+      </c>
+      <c r="F947" t="n">
+        <v>23</v>
+      </c>
+      <c r="G947" t="n">
+        <v>33</v>
+      </c>
+      <c r="H947" t="inlineStr">
+        <is>
+          <t>23/33</t>
+        </is>
+      </c>
+      <c r="I947" s="5" t="n">
+        <v>69.7</v>
+      </c>
+      <c r="J947" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K947" t="n">
+        <v>36297691</v>
+      </c>
+    </row>
+    <row r="948">
+      <c r="A948" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B948" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C948" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D948" t="inlineStr">
+        <is>
+          <t>RE-LAX  (English version)</t>
+        </is>
+      </c>
+      <c r="E948" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F948" t="n">
+        <v>28</v>
+      </c>
+      <c r="G948" t="n">
+        <v>33</v>
+      </c>
+      <c r="H948" t="inlineStr">
+        <is>
+          <t>28/33</t>
+        </is>
+      </c>
+      <c r="I948" s="5" t="n">
+        <v>84.8</v>
+      </c>
+      <c r="J948" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K948" t="n">
+        <v>36298053</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K943"/>
+  <autoFilter ref="A1:K948"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-08-27)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$948</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$953</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K948"/>
+  <dimension ref="A1:K953"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -44398,18 +44398,18 @@
         </is>
       </c>
       <c r="F935" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G935" t="n">
         <v>28</v>
       </c>
       <c r="H935" t="inlineStr">
         <is>
-          <t>19/28</t>
+          <t>18/28</t>
         </is>
       </c>
       <c r="I935" s="5" t="n">
-        <v>67.90000000000001</v>
+        <v>64.3</v>
       </c>
       <c r="J935" t="inlineStr">
         <is>
@@ -45031,8 +45031,243 @@
         <v>36298053</v>
       </c>
     </row>
+    <row r="949">
+      <c r="A949" s="2" t="n">
+        <v>46260</v>
+      </c>
+      <c r="B949" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C949" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D949" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E949" t="inlineStr">
+        <is>
+          <t>Alice Dunoyer</t>
+        </is>
+      </c>
+      <c r="F949" t="n">
+        <v>15</v>
+      </c>
+      <c r="G949" t="n">
+        <v>33</v>
+      </c>
+      <c r="H949" t="inlineStr">
+        <is>
+          <t>15/33</t>
+        </is>
+      </c>
+      <c r="I949" s="4" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="J949" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K949" t="n">
+        <v>36321416</v>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" s="2" t="n">
+        <v>46260</v>
+      </c>
+      <c r="B950" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C950" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D950" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E950" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F950" t="n">
+        <v>7</v>
+      </c>
+      <c r="G950" t="n">
+        <v>18</v>
+      </c>
+      <c r="H950" t="inlineStr">
+        <is>
+          <t>7/18</t>
+        </is>
+      </c>
+      <c r="I950" s="4" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="J950" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K950" t="n">
+        <v>36929298</v>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" s="2" t="n">
+        <v>46260</v>
+      </c>
+      <c r="B951" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C951" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D951" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E951" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F951" t="n">
+        <v>5</v>
+      </c>
+      <c r="G951" t="n">
+        <v>18</v>
+      </c>
+      <c r="H951" t="inlineStr">
+        <is>
+          <t>5/18</t>
+        </is>
+      </c>
+      <c r="I951" s="4" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="J951" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K951" t="n">
+        <v>36298347</v>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" s="2" t="n">
+        <v>46260</v>
+      </c>
+      <c r="B952" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C952" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D952" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E952" t="inlineStr">
+        <is>
+          <t>Pauline Ramon</t>
+        </is>
+      </c>
+      <c r="F952" t="n">
+        <v>29</v>
+      </c>
+      <c r="G952" t="n">
+        <v>33</v>
+      </c>
+      <c r="H952" t="inlineStr">
+        <is>
+          <t>29/33</t>
+        </is>
+      </c>
+      <c r="I952" s="3" t="n">
+        <v>87.90000000000001</v>
+      </c>
+      <c r="J952" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K952" t="n">
+        <v>36298388</v>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" s="2" t="n">
+        <v>46260</v>
+      </c>
+      <c r="B953" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C953" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D953" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E953" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F953" t="n">
+        <v>24</v>
+      </c>
+      <c r="G953" t="n">
+        <v>33</v>
+      </c>
+      <c r="H953" t="inlineStr">
+        <is>
+          <t>24/33</t>
+        </is>
+      </c>
+      <c r="I953" s="5" t="n">
+        <v>72.7</v>
+      </c>
+      <c r="J953" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K953" t="n">
+        <v>36298585</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K948"/>
+  <autoFilter ref="A1:K953"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-08-28)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$953</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$958</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K953"/>
+  <dimension ref="A1:K958"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -45266,8 +45266,243 @@
         <v>36298585</v>
       </c>
     </row>
+    <row r="954">
+      <c r="A954" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B954" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C954" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D954" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E954" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F954" t="n">
+        <v>10</v>
+      </c>
+      <c r="G954" t="n">
+        <v>33</v>
+      </c>
+      <c r="H954" t="inlineStr">
+        <is>
+          <t>10/33</t>
+        </is>
+      </c>
+      <c r="I954" s="4" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="J954" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K954" t="n">
+        <v>36321567</v>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B955" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C955" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D955" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E955" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F955" t="n">
+        <v>11</v>
+      </c>
+      <c r="G955" t="n">
+        <v>18</v>
+      </c>
+      <c r="H955" t="inlineStr">
+        <is>
+          <t>11/18</t>
+        </is>
+      </c>
+      <c r="I955" s="5" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="J955" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K955" t="n">
+        <v>36929389</v>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B956" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C956" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D956" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E956" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F956" t="n">
+        <v>10</v>
+      </c>
+      <c r="G956" t="n">
+        <v>18</v>
+      </c>
+      <c r="H956" t="inlineStr">
+        <is>
+          <t>10/18</t>
+        </is>
+      </c>
+      <c r="I956" s="5" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="J956" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K956" t="n">
+        <v>36298762</v>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B957" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C957" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D957" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E957" t="inlineStr">
+        <is>
+          <t>Faustine CHOPIN</t>
+        </is>
+      </c>
+      <c r="F957" t="n">
+        <v>24</v>
+      </c>
+      <c r="G957" t="n">
+        <v>33</v>
+      </c>
+      <c r="H957" t="inlineStr">
+        <is>
+          <t>24/33</t>
+        </is>
+      </c>
+      <c r="I957" s="5" t="n">
+        <v>72.7</v>
+      </c>
+      <c r="J957" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K957" t="n">
+        <v>36298816</v>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" s="2" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B958" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C958" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D958" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E958" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F958" t="n">
+        <v>26</v>
+      </c>
+      <c r="G958" t="n">
+        <v>33</v>
+      </c>
+      <c r="H958" t="inlineStr">
+        <is>
+          <t>26/33</t>
+        </is>
+      </c>
+      <c r="I958" s="5" t="n">
+        <v>78.8</v>
+      </c>
+      <c r="J958" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K958" t="n">
+        <v>36298869</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K953"/>
+  <autoFilter ref="A1:K958"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-08-29)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$958</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$965</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K958"/>
+  <dimension ref="A1:K965"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -43787,18 +43787,18 @@
         </is>
       </c>
       <c r="F922" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G922" t="n">
         <v>33</v>
       </c>
       <c r="H922" t="inlineStr">
         <is>
-          <t>15/33</t>
+          <t>14/33</t>
         </is>
       </c>
       <c r="I922" s="4" t="n">
-        <v>45.5</v>
+        <v>42.4</v>
       </c>
       <c r="J922" t="inlineStr">
         <is>
@@ -45479,18 +45479,18 @@
         </is>
       </c>
       <c r="F958" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G958" t="n">
         <v>33</v>
       </c>
       <c r="H958" t="inlineStr">
         <is>
-          <t>26/33</t>
+          <t>25/33</t>
         </is>
       </c>
       <c r="I958" s="5" t="n">
-        <v>78.8</v>
+        <v>75.8</v>
       </c>
       <c r="J958" t="inlineStr">
         <is>
@@ -45501,8 +45501,337 @@
         <v>36298869</v>
       </c>
     </row>
+    <row r="959">
+      <c r="A959" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B959" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C959" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D959" t="inlineStr">
+        <is>
+          <t>RE-BOOST</t>
+        </is>
+      </c>
+      <c r="E959" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F959" t="n">
+        <v>6</v>
+      </c>
+      <c r="G959" t="n">
+        <v>33</v>
+      </c>
+      <c r="H959" t="inlineStr">
+        <is>
+          <t>6/33</t>
+        </is>
+      </c>
+      <c r="I959" s="4" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="J959" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K959" t="n">
+        <v>36319505</v>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B960" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C960" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D960" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E960" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F960" t="n">
+        <v>1</v>
+      </c>
+      <c r="G960" t="n">
+        <v>16</v>
+      </c>
+      <c r="H960" t="inlineStr">
+        <is>
+          <t>1/16</t>
+        </is>
+      </c>
+      <c r="I960" s="4" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="J960" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K960" t="n">
+        <v>36320663</v>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B961" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C961" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D961" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E961" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F961" t="n">
+        <v>8</v>
+      </c>
+      <c r="G961" t="n">
+        <v>16</v>
+      </c>
+      <c r="H961" t="inlineStr">
+        <is>
+          <t>8/16</t>
+        </is>
+      </c>
+      <c r="I961" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J961" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K961" t="n">
+        <v>36320062</v>
+      </c>
+    </row>
+    <row r="962">
+      <c r="A962" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B962" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C962" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D962" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E962" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F962" t="n">
+        <v>10</v>
+      </c>
+      <c r="G962" t="n">
+        <v>33</v>
+      </c>
+      <c r="H962" t="inlineStr">
+        <is>
+          <t>10/33</t>
+        </is>
+      </c>
+      <c r="I962" s="4" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="J962" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K962" t="n">
+        <v>36320786</v>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B963" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C963" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D963" t="inlineStr">
+        <is>
+          <t>RE-LAX</t>
+        </is>
+      </c>
+      <c r="E963" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F963" t="n">
+        <v>27</v>
+      </c>
+      <c r="G963" t="n">
+        <v>33</v>
+      </c>
+      <c r="H963" t="inlineStr">
+        <is>
+          <t>27/33</t>
+        </is>
+      </c>
+      <c r="I963" s="5" t="n">
+        <v>81.8</v>
+      </c>
+      <c r="J963" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K963" t="n">
+        <v>36320896</v>
+      </c>
+    </row>
+    <row r="964">
+      <c r="A964" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B964" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C964" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D964" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E964" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F964" t="n">
+        <v>20</v>
+      </c>
+      <c r="G964" t="n">
+        <v>20</v>
+      </c>
+      <c r="H964" t="inlineStr">
+        <is>
+          <t>20/20</t>
+        </is>
+      </c>
+      <c r="I964" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J964" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K964" t="n">
+        <v>36893833</v>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B965" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C965" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D965" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E965" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F965" t="n">
+        <v>7</v>
+      </c>
+      <c r="G965" t="n">
+        <v>20</v>
+      </c>
+      <c r="H965" t="inlineStr">
+        <is>
+          <t>7/20</t>
+        </is>
+      </c>
+      <c r="I965" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="J965" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K965" t="n">
+        <v>36893896</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K958"/>
+  <autoFilter ref="A1:K965"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-08-30)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$965</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$973</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K965"/>
+  <dimension ref="A1:K973"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1619,7 +1619,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1807,7 +1807,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1901,7 +1901,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1995,7 +1995,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2042,7 +2042,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2089,7 +2089,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2230,7 +2230,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2277,7 +2277,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2418,7 +2418,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2559,7 +2559,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2606,7 +2606,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2747,7 +2747,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>RE-BOOST  (English version)</t>
+          <t>Guided Session (English version)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2794,7 +2794,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2841,7 +2841,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -3076,7 +3076,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -3123,7 +3123,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -3170,7 +3170,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -3217,7 +3217,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -3264,7 +3264,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -3640,7 +3640,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3687,7 +3687,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3734,7 +3734,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3828,7 +3828,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -3875,7 +3875,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3922,7 +3922,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -4016,7 +4016,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -4063,7 +4063,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -4110,7 +4110,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -4251,7 +4251,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -4392,7 +4392,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -4439,7 +4439,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4580,7 +4580,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>RE-BOOST  (English version)</t>
+          <t>Guided Session (English version)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -4627,7 +4627,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -4674,7 +4674,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -4956,7 +4956,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -5097,7 +5097,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -5144,7 +5144,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -5379,7 +5379,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -5520,7 +5520,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -5614,7 +5614,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -5661,7 +5661,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -5802,7 +5802,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -5849,7 +5849,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -5896,7 +5896,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -5990,7 +5990,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -6131,7 +6131,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -6272,7 +6272,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -6413,7 +6413,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -6460,7 +6460,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -6648,7 +6648,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>RE-BOOST  (English version)</t>
+          <t>Guided Session (English version)</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -6695,7 +6695,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -6742,7 +6742,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
@@ -6789,7 +6789,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -7024,7 +7024,7 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
@@ -7212,7 +7212,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
@@ -7259,7 +7259,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
@@ -7353,7 +7353,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
@@ -7494,7 +7494,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
@@ -7635,7 +7635,7 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
@@ -7776,7 +7776,7 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
@@ -7823,7 +7823,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
@@ -7870,7 +7870,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
@@ -8011,7 +8011,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
@@ -8058,7 +8058,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
@@ -8105,7 +8105,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
@@ -8246,7 +8246,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
@@ -8293,7 +8293,7 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
@@ -8340,7 +8340,7 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
@@ -8481,7 +8481,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
@@ -8622,7 +8622,7 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
@@ -8669,7 +8669,7 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
@@ -8904,7 +8904,7 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
@@ -8951,7 +8951,7 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
@@ -9233,7 +9233,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
@@ -9421,7 +9421,7 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
@@ -9468,7 +9468,7 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
@@ -9562,7 +9562,7 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
@@ -9703,7 +9703,7 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
@@ -9844,7 +9844,7 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
@@ -9985,7 +9985,7 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
@@ -10032,7 +10032,7 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E204" t="inlineStr">
@@ -10079,7 +10079,7 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E205" t="inlineStr">
@@ -10126,7 +10126,7 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E206" t="inlineStr">
@@ -10173,7 +10173,7 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E207" t="inlineStr">
@@ -10220,7 +10220,7 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E208" t="inlineStr">
@@ -10408,7 +10408,7 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E212" t="inlineStr">
@@ -10549,7 +10549,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E215" t="inlineStr">
@@ -10596,7 +10596,7 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E216" t="inlineStr">
@@ -10643,7 +10643,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E217" t="inlineStr">
@@ -10690,7 +10690,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E218" t="inlineStr">
@@ -10784,7 +10784,7 @@
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E220" t="inlineStr">
@@ -10831,7 +10831,7 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E221" t="inlineStr">
@@ -11019,7 +11019,7 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>RE-BOOST  (English version)</t>
+          <t>Guided Session (English version)</t>
         </is>
       </c>
       <c r="E225" t="inlineStr">
@@ -11066,7 +11066,7 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E226" t="inlineStr">
@@ -11160,7 +11160,7 @@
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E228" t="inlineStr">
@@ -11724,7 +11724,7 @@
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E240" t="inlineStr">
@@ -11771,7 +11771,7 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E241" t="inlineStr">
@@ -11818,7 +11818,7 @@
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E242" t="inlineStr">
@@ -11959,7 +11959,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E245" t="inlineStr">
@@ -12241,7 +12241,7 @@
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E251" t="inlineStr">
@@ -12288,7 +12288,7 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E252" t="inlineStr">
@@ -12335,7 +12335,7 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E253" t="inlineStr">
@@ -12476,7 +12476,7 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E256" t="inlineStr">
@@ -12523,7 +12523,7 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E257" t="inlineStr">
@@ -12711,7 +12711,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E261" t="inlineStr">
@@ -12852,7 +12852,7 @@
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E264" t="inlineStr">
@@ -12899,7 +12899,7 @@
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E265" t="inlineStr">
@@ -13040,7 +13040,7 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E268" t="inlineStr">
@@ -13087,7 +13087,7 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E269" t="inlineStr">
@@ -13134,7 +13134,7 @@
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E270" t="inlineStr">
@@ -13181,7 +13181,7 @@
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E271" t="inlineStr">
@@ -13369,7 +13369,7 @@
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>RE-BOOST  (English version)</t>
+          <t>Guided Session (English version)</t>
         </is>
       </c>
       <c r="E275" t="inlineStr">
@@ -13557,7 +13557,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
@@ -13604,7 +13604,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
@@ -13886,7 +13886,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -14074,7 +14074,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -14121,7 +14121,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -14215,7 +14215,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
@@ -14356,7 +14356,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
@@ -14497,7 +14497,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -14638,7 +14638,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
@@ -14685,7 +14685,7 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
@@ -14732,7 +14732,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
@@ -14873,7 +14873,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
@@ -14920,7 +14920,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
@@ -15061,7 +15061,7 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
@@ -15296,7 +15296,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -15343,7 +15343,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -15390,7 +15390,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -15531,7 +15531,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -15578,7 +15578,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -15766,7 +15766,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>RE-BOOST  (English version)</t>
+          <t>Guided Session (English version)</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -15813,7 +15813,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -15860,7 +15860,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -15907,7 +15907,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -16189,7 +16189,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
@@ -16377,7 +16377,7 @@
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E339" t="inlineStr">
@@ -16424,7 +16424,7 @@
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E340" t="inlineStr">
@@ -16518,7 +16518,7 @@
       </c>
       <c r="D342" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E342" t="inlineStr">
@@ -16659,7 +16659,7 @@
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E345" t="inlineStr">
@@ -16800,7 +16800,7 @@
       </c>
       <c r="D348" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E348" t="inlineStr">
@@ -16941,7 +16941,7 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E351" t="inlineStr">
@@ -16988,7 +16988,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>RE-LAX  (English version)</t>
+          <t>Guided Session  (English version)</t>
         </is>
       </c>
       <c r="E352" t="inlineStr">
@@ -17035,7 +17035,7 @@
       </c>
       <c r="D353" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E353" t="inlineStr">
@@ -17176,7 +17176,7 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E356" t="inlineStr">
@@ -17223,7 +17223,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E357" t="inlineStr">
@@ -17270,7 +17270,7 @@
       </c>
       <c r="D358" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E358" t="inlineStr">
@@ -17458,7 +17458,7 @@
       </c>
       <c r="D362" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E362" t="inlineStr">
@@ -17599,7 +17599,7 @@
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E365" t="inlineStr">
@@ -17646,7 +17646,7 @@
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E366" t="inlineStr">
@@ -17740,7 +17740,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E368" t="inlineStr">
@@ -17881,7 +17881,7 @@
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E371" t="inlineStr">
@@ -17928,7 +17928,7 @@
       </c>
       <c r="D372" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E372" t="inlineStr">
@@ -18210,7 +18210,7 @@
       </c>
       <c r="D378" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E378" t="inlineStr">
@@ -18257,7 +18257,7 @@
       </c>
       <c r="D379" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E379" t="inlineStr">
@@ -18304,7 +18304,7 @@
       </c>
       <c r="D380" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E380" t="inlineStr">
@@ -18351,7 +18351,7 @@
       </c>
       <c r="D381" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E381" t="inlineStr">
@@ -18539,7 +18539,7 @@
       </c>
       <c r="D385" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E385" t="inlineStr">
@@ -18680,7 +18680,7 @@
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E388" t="inlineStr">
@@ -18727,7 +18727,7 @@
       </c>
       <c r="D389" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E389" t="inlineStr">
@@ -18821,7 +18821,7 @@
       </c>
       <c r="D391" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E391" t="inlineStr">
@@ -18962,7 +18962,7 @@
       </c>
       <c r="D394" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E394" t="inlineStr">
@@ -19009,7 +19009,7 @@
       </c>
       <c r="D395" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E395" t="inlineStr">
@@ -19103,7 +19103,7 @@
       </c>
       <c r="D397" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E397" t="inlineStr">
@@ -19244,7 +19244,7 @@
       </c>
       <c r="D400" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E400" t="inlineStr">
@@ -19291,7 +19291,7 @@
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>RE-LAX  (English version)</t>
+          <t>Guided Session  (English version)</t>
         </is>
       </c>
       <c r="E401" t="inlineStr">
@@ -19338,7 +19338,7 @@
       </c>
       <c r="D402" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E402" t="inlineStr">
@@ -19479,7 +19479,7 @@
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E405" t="inlineStr">
@@ -19526,7 +19526,7 @@
       </c>
       <c r="D406" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E406" t="inlineStr">
@@ -19573,7 +19573,7 @@
       </c>
       <c r="D407" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E407" t="inlineStr">
@@ -19667,7 +19667,7 @@
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E409" t="inlineStr">
@@ -19808,7 +19808,7 @@
       </c>
       <c r="D412" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E412" t="inlineStr">
@@ -19855,7 +19855,7 @@
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E413" t="inlineStr">
@@ -19902,7 +19902,7 @@
       </c>
       <c r="D414" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E414" t="inlineStr">
@@ -20043,7 +20043,7 @@
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E417" t="inlineStr">
@@ -20090,7 +20090,7 @@
       </c>
       <c r="D418" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E418" t="inlineStr">
@@ -20278,7 +20278,7 @@
       </c>
       <c r="D422" t="inlineStr">
         <is>
-          <t>RE-BOOST  (English version)</t>
+          <t>Guided Session (English version)</t>
         </is>
       </c>
       <c r="E422" t="inlineStr">
@@ -20325,7 +20325,7 @@
       </c>
       <c r="D423" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E423" t="inlineStr">
@@ -20513,7 +20513,7 @@
       </c>
       <c r="D427" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E427" t="inlineStr">
@@ -20654,7 +20654,7 @@
       </c>
       <c r="D430" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E430" t="inlineStr">
@@ -20701,7 +20701,7 @@
       </c>
       <c r="D431" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E431" t="inlineStr">
@@ -20795,7 +20795,7 @@
       </c>
       <c r="D433" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E433" t="inlineStr">
@@ -20936,7 +20936,7 @@
       </c>
       <c r="D436" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E436" t="inlineStr">
@@ -20983,7 +20983,7 @@
       </c>
       <c r="D437" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E437" t="inlineStr">
@@ -21077,7 +21077,7 @@
       </c>
       <c r="D439" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E439" t="inlineStr">
@@ -21218,7 +21218,7 @@
       </c>
       <c r="D442" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E442" t="inlineStr">
@@ -21265,7 +21265,7 @@
       </c>
       <c r="D443" t="inlineStr">
         <is>
-          <t>RE-LAX  (English version)</t>
+          <t>Guided Session  (English version)</t>
         </is>
       </c>
       <c r="E443" t="inlineStr">
@@ -21312,7 +21312,7 @@
       </c>
       <c r="D444" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E444" t="inlineStr">
@@ -21453,7 +21453,7 @@
       </c>
       <c r="D447" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E447" t="inlineStr">
@@ -21500,7 +21500,7 @@
       </c>
       <c r="D448" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E448" t="inlineStr">
@@ -21547,7 +21547,7 @@
       </c>
       <c r="D449" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E449" t="inlineStr">
@@ -21735,7 +21735,7 @@
       </c>
       <c r="D453" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E453" t="inlineStr">
@@ -21876,7 +21876,7 @@
       </c>
       <c r="D456" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E456" t="inlineStr">
@@ -21923,7 +21923,7 @@
       </c>
       <c r="D457" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E457" t="inlineStr">
@@ -22111,7 +22111,7 @@
       </c>
       <c r="D461" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E461" t="inlineStr">
@@ -22158,7 +22158,7 @@
       </c>
       <c r="D462" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E462" t="inlineStr">
@@ -22440,7 +22440,7 @@
       </c>
       <c r="D468" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E468" t="inlineStr">
@@ -22534,7 +22534,7 @@
       </c>
       <c r="D470" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E470" t="inlineStr">
@@ -22722,7 +22722,7 @@
       </c>
       <c r="D474" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E474" t="inlineStr">
@@ -22863,7 +22863,7 @@
       </c>
       <c r="D477" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E477" t="inlineStr">
@@ -22910,7 +22910,7 @@
       </c>
       <c r="D478" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E478" t="inlineStr">
@@ -23004,7 +23004,7 @@
       </c>
       <c r="D480" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E480" t="inlineStr">
@@ -23192,7 +23192,7 @@
       </c>
       <c r="D484" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E484" t="inlineStr">
@@ -23239,7 +23239,7 @@
       </c>
       <c r="D485" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E485" t="inlineStr">
@@ -23286,7 +23286,7 @@
       </c>
       <c r="D486" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E486" t="inlineStr">
@@ -23427,7 +23427,7 @@
       </c>
       <c r="D489" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E489" t="inlineStr">
@@ -23474,7 +23474,7 @@
       </c>
       <c r="D490" t="inlineStr">
         <is>
-          <t>RE-LAX  (English version)</t>
+          <t>Guided Session  (English version)</t>
         </is>
       </c>
       <c r="E490" t="inlineStr">
@@ -23568,7 +23568,7 @@
       </c>
       <c r="D492" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E492" t="inlineStr">
@@ -23709,7 +23709,7 @@
       </c>
       <c r="D495" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E495" t="inlineStr">
@@ -23756,7 +23756,7 @@
       </c>
       <c r="D496" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E496" t="inlineStr">
@@ -23803,7 +23803,7 @@
       </c>
       <c r="D497" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E497" t="inlineStr">
@@ -23991,7 +23991,7 @@
       </c>
       <c r="D501" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E501" t="inlineStr">
@@ -24132,7 +24132,7 @@
       </c>
       <c r="D504" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E504" t="inlineStr">
@@ -24179,7 +24179,7 @@
       </c>
       <c r="D505" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E505" t="inlineStr">
@@ -24226,7 +24226,7 @@
       </c>
       <c r="D506" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E506" t="inlineStr">
@@ -24367,7 +24367,7 @@
       </c>
       <c r="D509" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E509" t="inlineStr">
@@ -24414,7 +24414,7 @@
       </c>
       <c r="D510" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E510" t="inlineStr">
@@ -24602,7 +24602,7 @@
       </c>
       <c r="D514" t="inlineStr">
         <is>
-          <t>RE-BOOST  (English version)</t>
+          <t>Guided Session (English version)</t>
         </is>
       </c>
       <c r="E514" t="inlineStr">
@@ -24790,7 +24790,7 @@
       </c>
       <c r="D518" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E518" t="inlineStr">
@@ -24837,7 +24837,7 @@
       </c>
       <c r="D519" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E519" t="inlineStr">
@@ -24931,7 +24931,7 @@
       </c>
       <c r="D521" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E521" t="inlineStr">
@@ -25072,7 +25072,7 @@
       </c>
       <c r="D524" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E524" t="inlineStr">
@@ -25119,7 +25119,7 @@
       </c>
       <c r="D525" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E525" t="inlineStr">
@@ -25213,7 +25213,7 @@
       </c>
       <c r="D527" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E527" t="inlineStr">
@@ -25354,7 +25354,7 @@
       </c>
       <c r="D530" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E530" t="inlineStr">
@@ -25448,7 +25448,7 @@
       </c>
       <c r="D532" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E532" t="inlineStr">
@@ -25589,7 +25589,7 @@
       </c>
       <c r="D535" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E535" t="inlineStr">
@@ -25636,7 +25636,7 @@
       </c>
       <c r="D536" t="inlineStr">
         <is>
-          <t>RE-LAX  (English version)</t>
+          <t>Guided Session  (English version)</t>
         </is>
       </c>
       <c r="E536" t="inlineStr">
@@ -25683,7 +25683,7 @@
       </c>
       <c r="D537" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E537" t="inlineStr">
@@ -25824,7 +25824,7 @@
       </c>
       <c r="D540" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E540" t="inlineStr">
@@ -25871,7 +25871,7 @@
       </c>
       <c r="D541" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E541" t="inlineStr">
@@ -25918,7 +25918,7 @@
       </c>
       <c r="D542" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E542" t="inlineStr">
@@ -26106,7 +26106,7 @@
       </c>
       <c r="D546" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E546" t="inlineStr">
@@ -26247,7 +26247,7 @@
       </c>
       <c r="D549" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E549" t="inlineStr">
@@ -26294,7 +26294,7 @@
       </c>
       <c r="D550" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E550" t="inlineStr">
@@ -26341,7 +26341,7 @@
       </c>
       <c r="D551" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E551" t="inlineStr">
@@ -26482,7 +26482,7 @@
       </c>
       <c r="D554" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E554" t="inlineStr">
@@ -26529,7 +26529,7 @@
       </c>
       <c r="D555" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E555" t="inlineStr">
@@ -26717,7 +26717,7 @@
       </c>
       <c r="D559" t="inlineStr">
         <is>
-          <t>RE-BOOST  (English version)</t>
+          <t>Guided Session (English version)</t>
         </is>
       </c>
       <c r="E559" t="inlineStr">
@@ -26811,7 +26811,7 @@
       </c>
       <c r="D561" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E561" t="inlineStr">
@@ -27093,7 +27093,7 @@
       </c>
       <c r="D567" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E567" t="inlineStr">
@@ -27281,7 +27281,7 @@
       </c>
       <c r="D571" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E571" t="inlineStr">
@@ -27375,7 +27375,7 @@
       </c>
       <c r="D573" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E573" t="inlineStr">
@@ -27563,7 +27563,7 @@
       </c>
       <c r="D577" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E577" t="inlineStr">
@@ -27610,7 +27610,7 @@
       </c>
       <c r="D578" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E578" t="inlineStr">
@@ -27704,7 +27704,7 @@
       </c>
       <c r="D580" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E580" t="inlineStr">
@@ -27845,7 +27845,7 @@
       </c>
       <c r="D583" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E583" t="inlineStr">
@@ -27892,7 +27892,7 @@
       </c>
       <c r="D584" t="inlineStr">
         <is>
-          <t>RE-LAX  (English version)</t>
+          <t>Guided Session  (English version)</t>
         </is>
       </c>
       <c r="E584" t="inlineStr">
@@ -27939,7 +27939,7 @@
       </c>
       <c r="D585" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E585" t="inlineStr">
@@ -28080,7 +28080,7 @@
       </c>
       <c r="D588" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E588" t="inlineStr">
@@ -28127,7 +28127,7 @@
       </c>
       <c r="D589" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E589" t="inlineStr">
@@ -28315,7 +28315,7 @@
       </c>
       <c r="D593" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E593" t="inlineStr">
@@ -28362,7 +28362,7 @@
       </c>
       <c r="D594" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E594" t="inlineStr">
@@ -28409,7 +28409,7 @@
       </c>
       <c r="D595" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E595" t="inlineStr">
@@ -28597,7 +28597,7 @@
       </c>
       <c r="D599" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E599" t="inlineStr">
@@ -29302,7 +29302,7 @@
       </c>
       <c r="D614" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E614" t="inlineStr">
@@ -29490,7 +29490,7 @@
       </c>
       <c r="D618" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E618" t="inlineStr">
@@ -29537,7 +29537,7 @@
       </c>
       <c r="D619" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E619" t="inlineStr">
@@ -29631,7 +29631,7 @@
       </c>
       <c r="D621" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E621" t="inlineStr">
@@ -29772,7 +29772,7 @@
       </c>
       <c r="D624" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E624" t="inlineStr">
@@ -29819,7 +29819,7 @@
       </c>
       <c r="D625" t="inlineStr">
         <is>
-          <t>RE-LAX  (English version)</t>
+          <t>Guided Session  (English version)</t>
         </is>
       </c>
       <c r="E625" t="inlineStr">
@@ -29913,7 +29913,7 @@
       </c>
       <c r="D627" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E627" t="inlineStr">
@@ -30054,7 +30054,7 @@
       </c>
       <c r="D630" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E630" t="inlineStr">
@@ -30101,7 +30101,7 @@
       </c>
       <c r="D631" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E631" t="inlineStr">
@@ -30336,7 +30336,7 @@
       </c>
       <c r="D636" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E636" t="inlineStr">
@@ -30477,7 +30477,7 @@
       </c>
       <c r="D639" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E639" t="inlineStr">
@@ -30524,7 +30524,7 @@
       </c>
       <c r="D640" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E640" t="inlineStr">
@@ -30618,7 +30618,7 @@
       </c>
       <c r="D642" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E642" t="inlineStr">
@@ -30759,7 +30759,7 @@
       </c>
       <c r="D645" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E645" t="inlineStr">
@@ -30806,7 +30806,7 @@
       </c>
       <c r="D646" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E646" t="inlineStr">
@@ -30994,7 +30994,7 @@
       </c>
       <c r="D650" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E650" t="inlineStr">
@@ -31088,7 +31088,7 @@
       </c>
       <c r="D652" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E652" t="inlineStr">
@@ -31370,7 +31370,7 @@
       </c>
       <c r="D658" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E658" t="inlineStr">
@@ -31511,7 +31511,7 @@
       </c>
       <c r="D661" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E661" t="inlineStr">
@@ -31558,7 +31558,7 @@
       </c>
       <c r="D662" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E662" t="inlineStr">
@@ -31652,7 +31652,7 @@
       </c>
       <c r="D664" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E664" t="inlineStr">
@@ -31793,7 +31793,7 @@
       </c>
       <c r="D667" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E667" t="inlineStr">
@@ -31840,7 +31840,7 @@
       </c>
       <c r="D668" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E668" t="inlineStr">
@@ -31934,7 +31934,7 @@
       </c>
       <c r="D670" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E670" t="inlineStr">
@@ -32075,7 +32075,7 @@
       </c>
       <c r="D673" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E673" t="inlineStr">
@@ -32122,7 +32122,7 @@
       </c>
       <c r="D674" t="inlineStr">
         <is>
-          <t>RE-LAX  (English version)</t>
+          <t>Guided Session  (English version)</t>
         </is>
       </c>
       <c r="E674" t="inlineStr">
@@ -32216,7 +32216,7 @@
       </c>
       <c r="D676" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E676" t="inlineStr">
@@ -32357,7 +32357,7 @@
       </c>
       <c r="D679" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E679" t="inlineStr">
@@ -32404,7 +32404,7 @@
       </c>
       <c r="D680" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E680" t="inlineStr">
@@ -32451,7 +32451,7 @@
       </c>
       <c r="D681" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E681" t="inlineStr">
@@ -32592,7 +32592,7 @@
       </c>
       <c r="D684" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E684" t="inlineStr">
@@ -32639,7 +32639,7 @@
       </c>
       <c r="D685" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E685" t="inlineStr">
@@ -32686,7 +32686,7 @@
       </c>
       <c r="D686" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E686" t="inlineStr">
@@ -32827,7 +32827,7 @@
       </c>
       <c r="D689" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E689" t="inlineStr">
@@ -32968,7 +32968,7 @@
       </c>
       <c r="D692" t="inlineStr">
         <is>
-          <t>RE-BOOST  (English version)</t>
+          <t>Guided Session (English version)</t>
         </is>
       </c>
       <c r="E692" t="inlineStr">
@@ -33062,7 +33062,7 @@
       </c>
       <c r="D694" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E694" t="inlineStr">
@@ -33156,7 +33156,7 @@
       </c>
       <c r="D696" t="inlineStr">
         <is>
-          <t>RE-LAX  (English version)</t>
+          <t>Guided Session  (English version)</t>
         </is>
       </c>
       <c r="E696" t="inlineStr">
@@ -33203,7 +33203,7 @@
       </c>
       <c r="D697" t="inlineStr">
         <is>
-          <t>RE-LAX  (English version)</t>
+          <t>Guided Session  (English version)</t>
         </is>
       </c>
       <c r="E697" t="inlineStr">
@@ -33344,7 +33344,7 @@
       </c>
       <c r="D700" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E700" t="inlineStr">
@@ -33485,7 +33485,7 @@
       </c>
       <c r="D703" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E703" t="inlineStr">
@@ -33767,7 +33767,7 @@
       </c>
       <c r="D709" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E709" t="inlineStr">
@@ -33861,7 +33861,7 @@
       </c>
       <c r="D711" t="inlineStr">
         <is>
-          <t>RE-LAX  (English version)</t>
+          <t>Guided Session  (English version)</t>
         </is>
       </c>
       <c r="E711" t="inlineStr">
@@ -33955,7 +33955,7 @@
       </c>
       <c r="D713" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E713" t="inlineStr">
@@ -34002,7 +34002,7 @@
       </c>
       <c r="D714" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E714" t="inlineStr">
@@ -34143,7 +34143,7 @@
       </c>
       <c r="D717" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E717" t="inlineStr">
@@ -34190,7 +34190,7 @@
       </c>
       <c r="D718" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E718" t="inlineStr">
@@ -34237,7 +34237,7 @@
       </c>
       <c r="D719" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E719" t="inlineStr">
@@ -34425,7 +34425,7 @@
       </c>
       <c r="D723" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E723" t="inlineStr">
@@ -34566,7 +34566,7 @@
       </c>
       <c r="D726" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E726" t="inlineStr">
@@ -34613,7 +34613,7 @@
       </c>
       <c r="D727" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E727" t="inlineStr">
@@ -34801,7 +34801,7 @@
       </c>
       <c r="D731" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E731" t="inlineStr">
@@ -34848,7 +34848,7 @@
       </c>
       <c r="D732" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E732" t="inlineStr">
@@ -35036,7 +35036,7 @@
       </c>
       <c r="D736" t="inlineStr">
         <is>
-          <t>RE-BOOST  (English version)</t>
+          <t>Guided Session (English version)</t>
         </is>
       </c>
       <c r="E736" t="inlineStr">
@@ -35130,7 +35130,7 @@
       </c>
       <c r="D738" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E738" t="inlineStr">
@@ -35224,7 +35224,7 @@
       </c>
       <c r="D740" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E740" t="inlineStr">
@@ -35318,7 +35318,7 @@
       </c>
       <c r="D742" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E742" t="inlineStr">
@@ -35459,7 +35459,7 @@
       </c>
       <c r="D745" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E745" t="inlineStr">
@@ -35506,7 +35506,7 @@
       </c>
       <c r="D746" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E746" t="inlineStr">
@@ -35553,7 +35553,7 @@
       </c>
       <c r="D747" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E747" t="inlineStr">
@@ -35694,7 +35694,7 @@
       </c>
       <c r="D750" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E750" t="inlineStr">
@@ -35741,7 +35741,7 @@
       </c>
       <c r="D751" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E751" t="inlineStr">
@@ -35835,7 +35835,7 @@
       </c>
       <c r="D753" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E753" t="inlineStr">
@@ -35976,7 +35976,7 @@
       </c>
       <c r="D756" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E756" t="inlineStr">
@@ -36023,7 +36023,7 @@
       </c>
       <c r="D757" t="inlineStr">
         <is>
-          <t>RE-LAX  (English version)</t>
+          <t>Guided Session  (English version)</t>
         </is>
       </c>
       <c r="E757" t="inlineStr">
@@ -36117,7 +36117,7 @@
       </c>
       <c r="D759" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E759" t="inlineStr">
@@ -36258,7 +36258,7 @@
       </c>
       <c r="D762" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E762" t="inlineStr">
@@ -36305,7 +36305,7 @@
       </c>
       <c r="D763" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E763" t="inlineStr">
@@ -36352,7 +36352,7 @@
       </c>
       <c r="D764" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E764" t="inlineStr">
@@ -36493,7 +36493,7 @@
       </c>
       <c r="D767" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E767" t="inlineStr">
@@ -36540,7 +36540,7 @@
       </c>
       <c r="D768" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E768" t="inlineStr">
@@ -36728,7 +36728,7 @@
       </c>
       <c r="D772" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E772" t="inlineStr">
@@ -36775,7 +36775,7 @@
       </c>
       <c r="D773" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E773" t="inlineStr">
@@ -36963,7 +36963,7 @@
       </c>
       <c r="D777" t="inlineStr">
         <is>
-          <t>RE-BOOST  (English version)</t>
+          <t>Guided Session (English version)</t>
         </is>
       </c>
       <c r="E777" t="inlineStr">
@@ -37057,7 +37057,7 @@
       </c>
       <c r="D779" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E779" t="inlineStr">
@@ -37151,7 +37151,7 @@
       </c>
       <c r="D781" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E781" t="inlineStr">
@@ -37245,7 +37245,7 @@
       </c>
       <c r="D783" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E783" t="inlineStr">
@@ -37386,7 +37386,7 @@
       </c>
       <c r="D786" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E786" t="inlineStr">
@@ -37433,7 +37433,7 @@
       </c>
       <c r="D787" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E787" t="inlineStr">
@@ -37480,7 +37480,7 @@
       </c>
       <c r="D788" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E788" t="inlineStr">
@@ -37621,7 +37621,7 @@
       </c>
       <c r="D791" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E791" t="inlineStr">
@@ -37668,7 +37668,7 @@
       </c>
       <c r="D792" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E792" t="inlineStr">
@@ -37762,7 +37762,7 @@
       </c>
       <c r="D794" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E794" t="inlineStr">
@@ -37903,7 +37903,7 @@
       </c>
       <c r="D797" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E797" t="inlineStr">
@@ -37950,7 +37950,7 @@
       </c>
       <c r="D798" t="inlineStr">
         <is>
-          <t>RE-LAX  (English version)</t>
+          <t>Guided Session  (English version)</t>
         </is>
       </c>
       <c r="E798" t="inlineStr">
@@ -38044,7 +38044,7 @@
       </c>
       <c r="D800" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E800" t="inlineStr">
@@ -38185,7 +38185,7 @@
       </c>
       <c r="D803" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E803" t="inlineStr">
@@ -38232,7 +38232,7 @@
       </c>
       <c r="D804" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E804" t="inlineStr">
@@ -38420,7 +38420,7 @@
       </c>
       <c r="D808" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E808" t="inlineStr">
@@ -38467,7 +38467,7 @@
       </c>
       <c r="D809" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E809" t="inlineStr">
@@ -38514,7 +38514,7 @@
       </c>
       <c r="D810" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E810" t="inlineStr">
@@ -38702,7 +38702,7 @@
       </c>
       <c r="D814" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E814" t="inlineStr">
@@ -38890,7 +38890,7 @@
       </c>
       <c r="D818" t="inlineStr">
         <is>
-          <t>RE-BOOST  (English version)</t>
+          <t>Guided Session (English version)</t>
         </is>
       </c>
       <c r="E818" t="inlineStr">
@@ -38984,7 +38984,7 @@
       </c>
       <c r="D820" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E820" t="inlineStr">
@@ -39078,7 +39078,7 @@
       </c>
       <c r="D822" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E822" t="inlineStr">
@@ -39172,7 +39172,7 @@
       </c>
       <c r="D824" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E824" t="inlineStr">
@@ -39313,7 +39313,7 @@
       </c>
       <c r="D827" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E827" t="inlineStr">
@@ -39360,7 +39360,7 @@
       </c>
       <c r="D828" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E828" t="inlineStr">
@@ -39501,7 +39501,7 @@
       </c>
       <c r="D831" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E831" t="inlineStr">
@@ -39689,7 +39689,7 @@
       </c>
       <c r="D835" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E835" t="inlineStr">
@@ -39736,7 +39736,7 @@
       </c>
       <c r="D836" t="inlineStr">
         <is>
-          <t>RE-LAX  (English version)</t>
+          <t>Guided Session  (English version)</t>
         </is>
       </c>
       <c r="E836" t="inlineStr">
@@ -39924,7 +39924,7 @@
       </c>
       <c r="D840" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E840" t="inlineStr">
@@ -40065,7 +40065,7 @@
       </c>
       <c r="D843" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E843" t="inlineStr">
@@ -40112,7 +40112,7 @@
       </c>
       <c r="D844" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E844" t="inlineStr">
@@ -40159,7 +40159,7 @@
       </c>
       <c r="D845" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E845" t="inlineStr">
@@ -40206,7 +40206,7 @@
       </c>
       <c r="D846" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E846" t="inlineStr">
@@ -40441,7 +40441,7 @@
       </c>
       <c r="D851" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E851" t="inlineStr">
@@ -40488,7 +40488,7 @@
       </c>
       <c r="D852" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E852" t="inlineStr">
@@ -40535,7 +40535,7 @@
       </c>
       <c r="D853" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E853" t="inlineStr">
@@ -40676,7 +40676,7 @@
       </c>
       <c r="D856" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E856" t="inlineStr">
@@ -40723,7 +40723,7 @@
       </c>
       <c r="D857" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E857" t="inlineStr">
@@ -40770,7 +40770,7 @@
       </c>
       <c r="D858" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E858" t="inlineStr">
@@ -40958,7 +40958,7 @@
       </c>
       <c r="D862" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E862" t="inlineStr">
@@ -41005,7 +41005,7 @@
       </c>
       <c r="D863" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E863" t="inlineStr">
@@ -41099,7 +41099,7 @@
       </c>
       <c r="D865" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E865" t="inlineStr">
@@ -41240,7 +41240,7 @@
       </c>
       <c r="D868" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E868" t="inlineStr">
@@ -41287,7 +41287,7 @@
       </c>
       <c r="D869" t="inlineStr">
         <is>
-          <t>RE-LAX  (English version)</t>
+          <t>Guided Session  (English version)</t>
         </is>
       </c>
       <c r="E869" t="inlineStr">
@@ -41334,7 +41334,7 @@
       </c>
       <c r="D870" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E870" t="inlineStr">
@@ -41475,7 +41475,7 @@
       </c>
       <c r="D873" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E873" t="inlineStr">
@@ -41522,7 +41522,7 @@
       </c>
       <c r="D874" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E874" t="inlineStr">
@@ -41569,7 +41569,7 @@
       </c>
       <c r="D875" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E875" t="inlineStr">
@@ -41757,7 +41757,7 @@
       </c>
       <c r="D879" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E879" t="inlineStr">
@@ -41898,7 +41898,7 @@
       </c>
       <c r="D882" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E882" t="inlineStr">
@@ -41945,7 +41945,7 @@
       </c>
       <c r="D883" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E883" t="inlineStr">
@@ -41992,7 +41992,7 @@
       </c>
       <c r="D884" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E884" t="inlineStr">
@@ -42133,7 +42133,7 @@
       </c>
       <c r="D887" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E887" t="inlineStr">
@@ -42180,7 +42180,7 @@
       </c>
       <c r="D888" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E888" t="inlineStr">
@@ -42368,7 +42368,7 @@
       </c>
       <c r="D892" t="inlineStr">
         <is>
-          <t>RE-BOOST  (English version)</t>
+          <t>Guided Session (English version)</t>
         </is>
       </c>
       <c r="E892" t="inlineStr">
@@ -42462,7 +42462,7 @@
       </c>
       <c r="D894" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E894" t="inlineStr">
@@ -42556,7 +42556,7 @@
       </c>
       <c r="D896" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E896" t="inlineStr">
@@ -42744,7 +42744,7 @@
       </c>
       <c r="D900" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E900" t="inlineStr">
@@ -42885,7 +42885,7 @@
       </c>
       <c r="D903" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E903" t="inlineStr">
@@ -42932,7 +42932,7 @@
       </c>
       <c r="D904" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E904" t="inlineStr">
@@ -43120,7 +43120,7 @@
       </c>
       <c r="D908" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E908" t="inlineStr">
@@ -43308,7 +43308,7 @@
       </c>
       <c r="D912" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E912" t="inlineStr">
@@ -43355,7 +43355,7 @@
       </c>
       <c r="D913" t="inlineStr">
         <is>
-          <t>RE-LAX  (English version)</t>
+          <t>Guided Session  (English version)</t>
         </is>
       </c>
       <c r="E913" t="inlineStr">
@@ -43543,7 +43543,7 @@
       </c>
       <c r="D917" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E917" t="inlineStr">
@@ -43731,7 +43731,7 @@
       </c>
       <c r="D921" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E921" t="inlineStr">
@@ -43778,7 +43778,7 @@
       </c>
       <c r="D922" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E922" t="inlineStr">
@@ -43825,7 +43825,7 @@
       </c>
       <c r="D923" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E923" t="inlineStr">
@@ -44013,7 +44013,7 @@
       </c>
       <c r="D927" t="inlineStr">
         <is>
-          <t>RE-BOOST  (English version)</t>
+          <t>Guided Session (English version)</t>
         </is>
       </c>
       <c r="E927" t="inlineStr">
@@ -44107,7 +44107,7 @@
       </c>
       <c r="D929" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E929" t="inlineStr">
@@ -44201,7 +44201,7 @@
       </c>
       <c r="D931" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E931" t="inlineStr">
@@ -44295,7 +44295,7 @@
       </c>
       <c r="D933" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E933" t="inlineStr">
@@ -44436,7 +44436,7 @@
       </c>
       <c r="D936" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E936" t="inlineStr">
@@ -44483,7 +44483,7 @@
       </c>
       <c r="D937" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E937" t="inlineStr">
@@ -44577,7 +44577,7 @@
       </c>
       <c r="D939" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E939" t="inlineStr">
@@ -44718,7 +44718,7 @@
       </c>
       <c r="D942" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E942" t="inlineStr">
@@ -44765,7 +44765,7 @@
       </c>
       <c r="D943" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E943" t="inlineStr">
@@ -44812,7 +44812,7 @@
       </c>
       <c r="D944" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E944" t="inlineStr">
@@ -44953,7 +44953,7 @@
       </c>
       <c r="D947" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E947" t="inlineStr">
@@ -45000,7 +45000,7 @@
       </c>
       <c r="D948" t="inlineStr">
         <is>
-          <t>RE-LAX  (English version)</t>
+          <t>Guided Session  (English version)</t>
         </is>
       </c>
       <c r="E948" t="inlineStr">
@@ -45047,7 +45047,7 @@
       </c>
       <c r="D949" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E949" t="inlineStr">
@@ -45188,7 +45188,7 @@
       </c>
       <c r="D952" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E952" t="inlineStr">
@@ -45235,7 +45235,7 @@
       </c>
       <c r="D953" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E953" t="inlineStr">
@@ -45282,7 +45282,7 @@
       </c>
       <c r="D954" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E954" t="inlineStr">
@@ -45423,7 +45423,7 @@
       </c>
       <c r="D957" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E957" t="inlineStr">
@@ -45470,7 +45470,7 @@
       </c>
       <c r="D958" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E958" t="inlineStr">
@@ -45517,7 +45517,7 @@
       </c>
       <c r="D959" t="inlineStr">
         <is>
-          <t>RE-BOOST</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E959" t="inlineStr">
@@ -45658,7 +45658,7 @@
       </c>
       <c r="D962" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E962" t="inlineStr">
@@ -45705,7 +45705,7 @@
       </c>
       <c r="D963" t="inlineStr">
         <is>
-          <t>RE-LAX</t>
+          <t>Guided Session</t>
         </is>
       </c>
       <c r="E963" t="inlineStr">
@@ -45830,8 +45830,384 @@
         <v>36893896</v>
       </c>
     </row>
+    <row r="966">
+      <c r="A966" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B966" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C966" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D966" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E966" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F966" t="n">
+        <v>11</v>
+      </c>
+      <c r="G966" t="n">
+        <v>32</v>
+      </c>
+      <c r="H966" t="inlineStr">
+        <is>
+          <t>11/32</t>
+        </is>
+      </c>
+      <c r="I966" s="4" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="J966" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K966" t="n">
+        <v>36323280</v>
+      </c>
+    </row>
+    <row r="967">
+      <c r="A967" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B967" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C967" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D967" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E967" t="inlineStr">
+        <is>
+          <t>Alice Dunoyer</t>
+        </is>
+      </c>
+      <c r="F967" t="n">
+        <v>10</v>
+      </c>
+      <c r="G967" t="n">
+        <v>33</v>
+      </c>
+      <c r="H967" t="inlineStr">
+        <is>
+          <t>10/33</t>
+        </is>
+      </c>
+      <c r="I967" s="4" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="J967" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K967" t="n">
+        <v>36323126</v>
+      </c>
+    </row>
+    <row r="968">
+      <c r="A968" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B968" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C968" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D968" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E968" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F968" t="n">
+        <v>8</v>
+      </c>
+      <c r="G968" t="n">
+        <v>32</v>
+      </c>
+      <c r="H968" t="inlineStr">
+        <is>
+          <t>8/32</t>
+        </is>
+      </c>
+      <c r="I968" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="J968" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K968" t="n">
+        <v>38771778</v>
+      </c>
+    </row>
+    <row r="969">
+      <c r="A969" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B969" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C969" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D969" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E969" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F969" t="n">
+        <v>12</v>
+      </c>
+      <c r="G969" t="n">
+        <v>33</v>
+      </c>
+      <c r="H969" t="inlineStr">
+        <is>
+          <t>12/33</t>
+        </is>
+      </c>
+      <c r="I969" s="4" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="J969" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K969" t="n">
+        <v>36329208</v>
+      </c>
+    </row>
+    <row r="970">
+      <c r="A970" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B970" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C970" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="D970" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E970" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F970" t="n">
+        <v>24</v>
+      </c>
+      <c r="G970" t="n">
+        <v>32</v>
+      </c>
+      <c r="H970" t="inlineStr">
+        <is>
+          <t>24/32</t>
+        </is>
+      </c>
+      <c r="I970" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="J970" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K970" t="n">
+        <v>38771878</v>
+      </c>
+    </row>
+    <row r="971">
+      <c r="A971" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B971" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C971" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D971" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E971" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F971" t="n">
+        <v>25</v>
+      </c>
+      <c r="G971" t="n">
+        <v>33</v>
+      </c>
+      <c r="H971" t="inlineStr">
+        <is>
+          <t>25/33</t>
+        </is>
+      </c>
+      <c r="I971" s="5" t="n">
+        <v>75.8</v>
+      </c>
+      <c r="J971" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K971" t="n">
+        <v>36329973</v>
+      </c>
+    </row>
+    <row r="972">
+      <c r="A972" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B972" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C972" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D972" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E972" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F972" t="n">
+        <v>17</v>
+      </c>
+      <c r="G972" t="n">
+        <v>20</v>
+      </c>
+      <c r="H972" t="inlineStr">
+        <is>
+          <t>17/20</t>
+        </is>
+      </c>
+      <c r="I972" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="J972" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K972" t="n">
+        <v>36935880</v>
+      </c>
+    </row>
+    <row r="973">
+      <c r="A973" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="B973" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C973" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="D973" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E973" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F973" t="n">
+        <v>0</v>
+      </c>
+      <c r="G973" t="n">
+        <v>20</v>
+      </c>
+      <c r="H973" t="inlineStr">
+        <is>
+          <t>0/20</t>
+        </is>
+      </c>
+      <c r="I973" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J973" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K973" t="n">
+        <v>36323865</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K965"/>
+  <autoFilter ref="A1:K973"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-08-31)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$973</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$980</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K973"/>
+  <dimension ref="A1:K980"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -46206,8 +46206,337 @@
         <v>36323865</v>
       </c>
     </row>
+    <row r="974">
+      <c r="A974" s="2" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B974" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C974" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D974" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E974" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F974" t="n">
+        <v>10</v>
+      </c>
+      <c r="G974" t="n">
+        <v>36</v>
+      </c>
+      <c r="H974" t="inlineStr">
+        <is>
+          <t>10/36</t>
+        </is>
+      </c>
+      <c r="I974" s="4" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="J974" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K974" t="n">
+        <v>37240290</v>
+      </c>
+    </row>
+    <row r="975">
+      <c r="A975" s="2" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B975" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C975" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D975" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E975" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F975" t="n">
+        <v>18</v>
+      </c>
+      <c r="G975" t="n">
+        <v>33</v>
+      </c>
+      <c r="H975" t="inlineStr">
+        <is>
+          <t>18/33</t>
+        </is>
+      </c>
+      <c r="I975" s="5" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="J975" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K975" t="n">
+        <v>36336036</v>
+      </c>
+    </row>
+    <row r="976">
+      <c r="A976" s="2" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B976" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C976" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D976" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E976" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F976" t="n">
+        <v>21</v>
+      </c>
+      <c r="G976" t="n">
+        <v>32</v>
+      </c>
+      <c r="H976" t="inlineStr">
+        <is>
+          <t>21/32</t>
+        </is>
+      </c>
+      <c r="I976" s="5" t="n">
+        <v>65.59999999999999</v>
+      </c>
+      <c r="J976" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K976" t="n">
+        <v>37240433</v>
+      </c>
+    </row>
+    <row r="977">
+      <c r="A977" s="2" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B977" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C977" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="D977" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E977" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F977" t="n">
+        <v>29</v>
+      </c>
+      <c r="G977" t="n">
+        <v>28</v>
+      </c>
+      <c r="H977" t="inlineStr">
+        <is>
+          <t>29/28</t>
+        </is>
+      </c>
+      <c r="I977" s="3" t="n">
+        <v>103.6</v>
+      </c>
+      <c r="J977" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K977" t="n">
+        <v>36892150</v>
+      </c>
+    </row>
+    <row r="978">
+      <c r="A978" s="2" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B978" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C978" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="D978" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E978" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F978" t="n">
+        <v>34</v>
+      </c>
+      <c r="G978" t="n">
+        <v>33</v>
+      </c>
+      <c r="H978" t="inlineStr">
+        <is>
+          <t>34/33</t>
+        </is>
+      </c>
+      <c r="I978" s="3" t="n">
+        <v>103</v>
+      </c>
+      <c r="J978" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K978" t="n">
+        <v>36336251</v>
+      </c>
+    </row>
+    <row r="979">
+      <c r="A979" s="2" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B979" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C979" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="D979" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E979" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F979" t="n">
+        <v>29</v>
+      </c>
+      <c r="G979" t="n">
+        <v>33</v>
+      </c>
+      <c r="H979" t="inlineStr">
+        <is>
+          <t>29/33</t>
+        </is>
+      </c>
+      <c r="I979" s="3" t="n">
+        <v>87.90000000000001</v>
+      </c>
+      <c r="J979" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K979" t="n">
+        <v>36692763</v>
+      </c>
+    </row>
+    <row r="980">
+      <c r="A980" s="2" t="n">
+        <v>46264</v>
+      </c>
+      <c r="B980" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C980" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="D980" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E980" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F980" t="n">
+        <v>18</v>
+      </c>
+      <c r="G980" t="n">
+        <v>36</v>
+      </c>
+      <c r="H980" t="inlineStr">
+        <is>
+          <t>18/36</t>
+        </is>
+      </c>
+      <c r="I980" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J980" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K980" t="n">
+        <v>36892105</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K973"/>
+  <autoFilter ref="A1:K980"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-09-01)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$980</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$987</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K980"/>
+  <dimension ref="A1:K987"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -46535,8 +46535,337 @@
         <v>36892105</v>
       </c>
     </row>
+    <row r="981">
+      <c r="A981" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B981" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C981" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D981" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E981" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F981" t="n">
+        <v>10</v>
+      </c>
+      <c r="G981" t="n">
+        <v>28</v>
+      </c>
+      <c r="H981" t="inlineStr">
+        <is>
+          <t>10/28</t>
+        </is>
+      </c>
+      <c r="I981" s="4" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="J981" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K981" t="n">
+        <v>36390337</v>
+      </c>
+    </row>
+    <row r="982">
+      <c r="A982" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B982" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C982" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D982" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E982" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F982" t="n">
+        <v>2</v>
+      </c>
+      <c r="G982" t="n">
+        <v>28</v>
+      </c>
+      <c r="H982" t="inlineStr">
+        <is>
+          <t>2/28</t>
+        </is>
+      </c>
+      <c r="I982" s="4" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="J982" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K982" t="n">
+        <v>36281140</v>
+      </c>
+    </row>
+    <row r="983">
+      <c r="A983" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B983" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C983" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D983" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E983" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F983" t="n">
+        <v>15</v>
+      </c>
+      <c r="G983" t="n">
+        <v>18</v>
+      </c>
+      <c r="H983" t="inlineStr">
+        <is>
+          <t>15/18</t>
+        </is>
+      </c>
+      <c r="I983" s="5" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J983" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K983" t="n">
+        <v>38531916</v>
+      </c>
+    </row>
+    <row r="984">
+      <c r="A984" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B984" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C984" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D984" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E984" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F984" t="n">
+        <v>10</v>
+      </c>
+      <c r="G984" t="n">
+        <v>18</v>
+      </c>
+      <c r="H984" t="inlineStr">
+        <is>
+          <t>10/18</t>
+        </is>
+      </c>
+      <c r="I984" s="5" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="J984" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K984" t="n">
+        <v>36928735</v>
+      </c>
+    </row>
+    <row r="985">
+      <c r="A985" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B985" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C985" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D985" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E985" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F985" t="n">
+        <v>22</v>
+      </c>
+      <c r="G985" t="n">
+        <v>28</v>
+      </c>
+      <c r="H985" t="inlineStr">
+        <is>
+          <t>22/28</t>
+        </is>
+      </c>
+      <c r="I985" s="5" t="n">
+        <v>78.59999999999999</v>
+      </c>
+      <c r="J985" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K985" t="n">
+        <v>36281004</v>
+      </c>
+    </row>
+    <row r="986">
+      <c r="A986" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B986" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C986" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="D986" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E986" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F986" t="n">
+        <v>11</v>
+      </c>
+      <c r="G986" t="n">
+        <v>28</v>
+      </c>
+      <c r="H986" t="inlineStr">
+        <is>
+          <t>11/28</t>
+        </is>
+      </c>
+      <c r="I986" s="4" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="J986" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K986" t="n">
+        <v>37873146</v>
+      </c>
+    </row>
+    <row r="987">
+      <c r="A987" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B987" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C987" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D987" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E987" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F987" t="n">
+        <v>18</v>
+      </c>
+      <c r="G987" t="n">
+        <v>36</v>
+      </c>
+      <c r="H987" t="inlineStr">
+        <is>
+          <t>18/36</t>
+        </is>
+      </c>
+      <c r="I987" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J987" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K987" t="n">
+        <v>36929041</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K980"/>
+  <autoFilter ref="A1:K987"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-09-02)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$987</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$994</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K987"/>
+  <dimension ref="A1:K994"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -46864,8 +46864,337 @@
         <v>36929041</v>
       </c>
     </row>
+    <row r="988">
+      <c r="A988" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B988" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C988" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D988" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E988" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F988" t="n">
+        <v>12</v>
+      </c>
+      <c r="G988" t="n">
+        <v>28</v>
+      </c>
+      <c r="H988" t="inlineStr">
+        <is>
+          <t>12/28</t>
+        </is>
+      </c>
+      <c r="I988" s="4" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="J988" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K988" t="n">
+        <v>36321368</v>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B989" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C989" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D989" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E989" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F989" t="n">
+        <v>10</v>
+      </c>
+      <c r="G989" t="n">
+        <v>28</v>
+      </c>
+      <c r="H989" t="inlineStr">
+        <is>
+          <t>10/28</t>
+        </is>
+      </c>
+      <c r="I989" s="4" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="J989" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K989" t="n">
+        <v>40188402</v>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B990" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C990" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D990" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E990" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F990" t="n">
+        <v>7</v>
+      </c>
+      <c r="G990" t="n">
+        <v>18</v>
+      </c>
+      <c r="H990" t="inlineStr">
+        <is>
+          <t>7/18</t>
+        </is>
+      </c>
+      <c r="I990" s="4" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="J990" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K990" t="n">
+        <v>36929167</v>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B991" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C991" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D991" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E991" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F991" t="n">
+        <v>5</v>
+      </c>
+      <c r="G991" t="n">
+        <v>18</v>
+      </c>
+      <c r="H991" t="inlineStr">
+        <is>
+          <t>5/18</t>
+        </is>
+      </c>
+      <c r="I991" s="4" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="J991" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K991" t="n">
+        <v>36298247</v>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B992" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C992" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D992" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E992" t="inlineStr">
+        <is>
+          <t>Faustine CHOPIN</t>
+        </is>
+      </c>
+      <c r="F992" t="n">
+        <v>11</v>
+      </c>
+      <c r="G992" t="n">
+        <v>28</v>
+      </c>
+      <c r="H992" t="inlineStr">
+        <is>
+          <t>11/28</t>
+        </is>
+      </c>
+      <c r="I992" s="4" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="J992" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K992" t="n">
+        <v>36297692</v>
+      </c>
+    </row>
+    <row r="993">
+      <c r="A993" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B993" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C993" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="D993" t="inlineStr">
+        <is>
+          <t>Guided Session  (English version)</t>
+        </is>
+      </c>
+      <c r="E993" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F993" t="n">
+        <v>18</v>
+      </c>
+      <c r="G993" t="n">
+        <v>28</v>
+      </c>
+      <c r="H993" t="inlineStr">
+        <is>
+          <t>18/28</t>
+        </is>
+      </c>
+      <c r="I993" s="5" t="n">
+        <v>64.3</v>
+      </c>
+      <c r="J993" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K993" t="n">
+        <v>36298054</v>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B994" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C994" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D994" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E994" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F994" t="n">
+        <v>19</v>
+      </c>
+      <c r="G994" t="n">
+        <v>36</v>
+      </c>
+      <c r="H994" t="inlineStr">
+        <is>
+          <t>19/36</t>
+        </is>
+      </c>
+      <c r="I994" s="5" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="J994" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K994" t="n">
+        <v>40188408</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K987"/>
+  <autoFilter ref="A1:K994"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-09-03)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$994</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$999</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K994"/>
+  <dimension ref="A1:K999"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -47193,8 +47193,243 @@
         <v>40188408</v>
       </c>
     </row>
+    <row r="995">
+      <c r="A995" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B995" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C995" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D995" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E995" t="inlineStr">
+        <is>
+          <t>Alice Dunoyer</t>
+        </is>
+      </c>
+      <c r="F995" t="n">
+        <v>6</v>
+      </c>
+      <c r="G995" t="n">
+        <v>33</v>
+      </c>
+      <c r="H995" t="inlineStr">
+        <is>
+          <t>6/33</t>
+        </is>
+      </c>
+      <c r="I995" s="4" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="J995" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K995" t="n">
+        <v>36321417</v>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B996" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C996" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D996" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E996" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F996" t="n">
+        <v>8</v>
+      </c>
+      <c r="G996" t="n">
+        <v>18</v>
+      </c>
+      <c r="H996" t="inlineStr">
+        <is>
+          <t>8/18</t>
+        </is>
+      </c>
+      <c r="I996" s="4" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="J996" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K996" t="n">
+        <v>36929299</v>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B997" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C997" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D997" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E997" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F997" t="n">
+        <v>13</v>
+      </c>
+      <c r="G997" t="n">
+        <v>18</v>
+      </c>
+      <c r="H997" t="inlineStr">
+        <is>
+          <t>13/18</t>
+        </is>
+      </c>
+      <c r="I997" s="5" t="n">
+        <v>72.2</v>
+      </c>
+      <c r="J997" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K997" t="n">
+        <v>36298348</v>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B998" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C998" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D998" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E998" t="inlineStr">
+        <is>
+          <t>Pauline Ramon</t>
+        </is>
+      </c>
+      <c r="F998" t="n">
+        <v>20</v>
+      </c>
+      <c r="G998" t="n">
+        <v>28</v>
+      </c>
+      <c r="H998" t="inlineStr">
+        <is>
+          <t>20/28</t>
+        </is>
+      </c>
+      <c r="I998" s="5" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="J998" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K998" t="n">
+        <v>36298389</v>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B999" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C999" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D999" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E999" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F999" t="n">
+        <v>22</v>
+      </c>
+      <c r="G999" t="n">
+        <v>33</v>
+      </c>
+      <c r="H999" t="inlineStr">
+        <is>
+          <t>22/33</t>
+        </is>
+      </c>
+      <c r="I999" s="5" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J999" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K999" t="n">
+        <v>36298586</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K994"/>
+  <autoFilter ref="A1:K999"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-09-04)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$999</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1005</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K999"/>
+  <dimension ref="A1:K1005"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -47428,8 +47428,290 @@
         <v>36298586</v>
       </c>
     </row>
+    <row r="1000">
+      <c r="A1000" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B1000" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1000" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="D1000" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1000" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F1000" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1000" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1000" t="inlineStr">
+        <is>
+          <t>7/28</t>
+        </is>
+      </c>
+      <c r="I1000" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="J1000" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1000" t="n">
+        <v>37090013</v>
+      </c>
+    </row>
+    <row r="1001">
+      <c r="A1001" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B1001" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1001" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D1001" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1001" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F1001" t="n">
+        <v>10</v>
+      </c>
+      <c r="G1001" t="n">
+        <v>33</v>
+      </c>
+      <c r="H1001" t="inlineStr">
+        <is>
+          <t>10/33</t>
+        </is>
+      </c>
+      <c r="I1001" s="4" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="J1001" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1001" t="n">
+        <v>36321568</v>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B1002" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1002" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1002" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1002" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1002" t="n">
+        <v>9</v>
+      </c>
+      <c r="G1002" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1002" t="inlineStr">
+        <is>
+          <t>9/18</t>
+        </is>
+      </c>
+      <c r="I1002" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J1002" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1002" t="n">
+        <v>36929390</v>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B1003" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1003" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1003" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1003" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1003" t="n">
+        <v>9</v>
+      </c>
+      <c r="G1003" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1003" t="inlineStr">
+        <is>
+          <t>9/18</t>
+        </is>
+      </c>
+      <c r="I1003" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J1003" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1003" t="n">
+        <v>36298763</v>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B1004" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1004" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D1004" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1004" t="inlineStr">
+        <is>
+          <t>Nina Petitjean</t>
+        </is>
+      </c>
+      <c r="F1004" t="n">
+        <v>26</v>
+      </c>
+      <c r="G1004" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1004" t="inlineStr">
+        <is>
+          <t>26/28</t>
+        </is>
+      </c>
+      <c r="I1004" s="3" t="n">
+        <v>92.90000000000001</v>
+      </c>
+      <c r="J1004" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1004" t="n">
+        <v>36298817</v>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B1005" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1005" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D1005" t="inlineStr">
+        <is>
+          <t>Guided Session  🔥</t>
+        </is>
+      </c>
+      <c r="E1005" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F1005" t="n">
+        <v>25</v>
+      </c>
+      <c r="G1005" t="n">
+        <v>33</v>
+      </c>
+      <c r="H1005" t="inlineStr">
+        <is>
+          <t>25/33</t>
+        </is>
+      </c>
+      <c r="I1005" s="5" t="n">
+        <v>75.8</v>
+      </c>
+      <c r="J1005" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1005" t="n">
+        <v>36298870</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K999"/>
+  <autoFilter ref="A1:K1005"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-09-05)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1005</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1013</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1005"/>
+  <dimension ref="A1:K1013"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -47710,8 +47710,384 @@
         <v>36298870</v>
       </c>
     </row>
+    <row r="1006">
+      <c r="A1006" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B1006" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1006" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D1006" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1006" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F1006" t="n">
+        <v>18</v>
+      </c>
+      <c r="G1006" t="n">
+        <v>33</v>
+      </c>
+      <c r="H1006" t="inlineStr">
+        <is>
+          <t>18/33</t>
+        </is>
+      </c>
+      <c r="I1006" s="5" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="J1006" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1006" t="n">
+        <v>36319506</v>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B1007" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1007" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D1007" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1007" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1007" t="n">
+        <v>12</v>
+      </c>
+      <c r="G1007" t="n">
+        <v>12</v>
+      </c>
+      <c r="H1007" t="inlineStr">
+        <is>
+          <t>12/12</t>
+        </is>
+      </c>
+      <c r="I1007" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1007" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1007" t="n">
+        <v>36320664</v>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B1008" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1008" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="D1008" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1008" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1008" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1008" t="n">
+        <v>12</v>
+      </c>
+      <c r="H1008" t="inlineStr">
+        <is>
+          <t>0/12</t>
+        </is>
+      </c>
+      <c r="I1008" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1008" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1008" t="n">
+        <v>42666070</v>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B1009" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1009" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D1009" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1009" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1009" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1009" t="n">
+        <v>12</v>
+      </c>
+      <c r="H1009" t="inlineStr">
+        <is>
+          <t>7/12</t>
+        </is>
+      </c>
+      <c r="I1009" s="5" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="J1009" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1009" t="n">
+        <v>36320063</v>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B1010" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1010" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1010" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1010" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1010" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1010" t="n">
+        <v>34</v>
+      </c>
+      <c r="H1010" t="inlineStr">
+        <is>
+          <t>5/34</t>
+        </is>
+      </c>
+      <c r="I1010" s="4" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="J1010" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1010" t="n">
+        <v>36320787</v>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B1011" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1011" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D1011" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1011" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F1011" t="n">
+        <v>21</v>
+      </c>
+      <c r="G1011" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1011" t="inlineStr">
+        <is>
+          <t>21/28</t>
+        </is>
+      </c>
+      <c r="I1011" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="J1011" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1011" t="n">
+        <v>36320897</v>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B1012" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1012" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D1012" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1012" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1012" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1012" t="n">
+        <v>20</v>
+      </c>
+      <c r="H1012" t="inlineStr">
+        <is>
+          <t>6/20</t>
+        </is>
+      </c>
+      <c r="I1012" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="J1012" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1012" t="n">
+        <v>36893834</v>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B1013" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1013" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D1013" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1013" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1013" t="n">
+        <v>11</v>
+      </c>
+      <c r="G1013" t="n">
+        <v>20</v>
+      </c>
+      <c r="H1013" t="inlineStr">
+        <is>
+          <t>11/20</t>
+        </is>
+      </c>
+      <c r="I1013" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="J1013" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1013" t="n">
+        <v>36893899</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1005"/>
+  <autoFilter ref="A1:K1013"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-09-06)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1013</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1021</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1013"/>
+  <dimension ref="A1:K1021"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -48086,8 +48086,384 @@
         <v>36893899</v>
       </c>
     </row>
+    <row r="1014">
+      <c r="A1014" s="2" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B1014" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1014" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D1014" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1014" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1014" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1014" t="n">
+        <v>34</v>
+      </c>
+      <c r="H1014" t="inlineStr">
+        <is>
+          <t>8/34</t>
+        </is>
+      </c>
+      <c r="I1014" s="4" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="J1014" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1014" t="n">
+        <v>36323281</v>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" s="2" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B1015" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1015" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="D1015" t="inlineStr">
+        <is>
+          <t>Guided Session (English version)</t>
+        </is>
+      </c>
+      <c r="E1015" t="inlineStr">
+        <is>
+          <t>Alice Dunoyer</t>
+        </is>
+      </c>
+      <c r="F1015" t="n">
+        <v>11</v>
+      </c>
+      <c r="G1015" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1015" t="inlineStr">
+        <is>
+          <t>11/28</t>
+        </is>
+      </c>
+      <c r="I1015" s="4" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="J1015" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1015" t="n">
+        <v>36323127</v>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" s="2" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B1016" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1016" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="D1016" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1016" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1016" t="n">
+        <v>18</v>
+      </c>
+      <c r="G1016" t="n">
+        <v>34</v>
+      </c>
+      <c r="H1016" t="inlineStr">
+        <is>
+          <t>18/34</t>
+        </is>
+      </c>
+      <c r="I1016" s="5" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="J1016" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1016" t="n">
+        <v>38771779</v>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" s="2" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B1017" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1017" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D1017" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1017" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F1017" t="n">
+        <v>24</v>
+      </c>
+      <c r="G1017" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1017" t="inlineStr">
+        <is>
+          <t>24/28</t>
+        </is>
+      </c>
+      <c r="I1017" s="3" t="n">
+        <v>85.7</v>
+      </c>
+      <c r="J1017" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1017" t="n">
+        <v>36329209</v>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" s="2" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B1018" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1018" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D1018" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1018" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1018" t="n">
+        <v>12</v>
+      </c>
+      <c r="G1018" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1018" t="inlineStr">
+        <is>
+          <t>12/36</t>
+        </is>
+      </c>
+      <c r="I1018" s="4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J1018" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1018" t="n">
+        <v>38771879</v>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" s="2" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B1019" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1019" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="D1019" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1019" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1019" t="n">
+        <v>11</v>
+      </c>
+      <c r="G1019" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1019" t="inlineStr">
+        <is>
+          <t>11/28</t>
+        </is>
+      </c>
+      <c r="I1019" s="4" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="J1019" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1019" t="n">
+        <v>36329974</v>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" s="2" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B1020" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1020" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="D1020" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1020" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1020" t="n">
+        <v>11</v>
+      </c>
+      <c r="G1020" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1020" t="inlineStr">
+        <is>
+          <t>11/36</t>
+        </is>
+      </c>
+      <c r="I1020" s="4" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="J1020" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1020" t="n">
+        <v>40517182</v>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" s="2" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B1021" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1021" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="D1021" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1021" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1021" t="n">
+        <v>12</v>
+      </c>
+      <c r="G1021" t="n">
+        <v>34</v>
+      </c>
+      <c r="H1021" t="inlineStr">
+        <is>
+          <t>12/34</t>
+        </is>
+      </c>
+      <c r="I1021" s="4" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="J1021" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1021" t="n">
+        <v>36935881</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1013"/>
+  <autoFilter ref="A1:K1021"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>